<commit_message>
Polish capitalization in GV scripts
</commit_message>
<xml_diff>
--- a/GV_Campaign_NoEmail_20260620.xlsx
+++ b/GV_Campaign_NoEmail_20260620.xlsx
@@ -507,7 +507,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Good day Greg. I'm Charles with Paragon Government Solutions, and I'm a cash investor looking at 125 Deer Hound Trl, Columbia, SC 29223. could the seller look at a cash, as-is offer, quick close and a short inspection? Where can I email the written terms? Appreciate it!</t>
+          <t>Good day Greg. I'm Charles with Paragon Government Solutions, and I'm a cash investor looking at 125 Deer Hound Trl, Columbia, SC 29223. Could the seller look at a cash, as-is offer, quick close and a short inspection? Where can I email the written terms? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -557,7 +557,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Good day Tyjuan. this is Charles Pleasant with Paragon Government Solutions, and I'm a cash buyer interested in 108 Malisa Dr, Columbia, SC 29229. any chance the seller would take a cash, as-is offer, close quickly, short inspection period? Where should I send the offer in writing? Thank you!</t>
+          <t>Good day Tyjuan. This is Charles Pleasant with Paragon Government Solutions, and I'm a cash buyer interested in 108 Malisa Dr, Columbia, SC 29229. Any chance the seller would take a cash, as-is offer, close quickly, short inspection period? Where should I send the offer in writing? Thank you!</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Hi Julie — Charles Pleasant, Paragon Government Solutions. I'm interested in buying 1146 Castle Pinckney Rd, Columbia, SC 29223 for cash. open to a discounted cash, as-is offer with close quickly, short inspection period. What email should I send the written offer to? Much appreciated!</t>
+          <t>Hi Julie — Charles Pleasant, Paragon Government Solutions. I'm interested in buying 1146 Castle Pinckney Rd, Columbia, SC 29223 for cash. Open to a discounted cash, as-is offer with close quickly, short inspection period. What email should I send the written offer to? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Good day Jasmine. Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 13 Gatewood Way, Columbia, SC 29229. open to a discounted cash, as-is offer, quick close and a short inspection? What email should I send the written offer to? Appreciate it!</t>
+          <t>Good day Jasmine. Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 13 Gatewood Way, Columbia, SC 29229. Open to a discounted cash, as-is offer, quick close and a short inspection? What email should I send the written offer to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Hey Lauren — Charles here with Paragon Government Solutions. I'm a cash buyer interested in 1531 Alma Rd, Columbia, SC 29209. could the seller look at a cash, as-is offer with a quick clean close and short due diligence. Best email for the formal offer? Thank you!</t>
+          <t>Hey Lauren — Charles here with Paragon Government Solutions. I'm a cash buyer interested in 1531 Alma Rd, Columbia, SC 29209. Could the seller look at a cash, as-is offer with a quick clean close and short due diligence. Best email for the formal offer? Thank you!</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Hi Tricia. my name's Charles Pleasant, Paragon Government Solutions, and I came across 116 Patio Pl, Columbia, SC 29212 and buy cash. could the seller look at a cash, as-is offer, a quick clean close and short due diligence? Where can I email the written terms? Much appreciated!</t>
+          <t>Hi Tricia. My name's Charles Pleasant, Paragon Government Solutions, and I came across 116 Patio Pl, Columbia, SC 29212 and buy cash. Could the seller look at a cash, as-is offer, a quick clean close and short due diligence? Where can I email the written terms? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Joey, hi. this is Charles Pleasant with Paragon Government Solutions, and I'm a cash buyer interested in 1515 Rushmore Rd, Columbia, SC 29210. any chance the seller would take a cash, as-is offer, fast cash close, short feasibility window? What's the best email to send it to? Appreciate it!</t>
+          <t>Joey, hi. This is Charles Pleasant with Paragon Government Solutions, and I'm a cash buyer interested in 1515 Rushmore Rd, Columbia, SC 29210. Any chance the seller would take a cash, as-is offer, fast cash close, short feasibility window? What's the best email to send it to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -882,7 +882,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Hello Jamila. Charles here with Paragon Government Solutions, and I'm interested in buying 103 Village Way, Columbia, SC 29209 for cash. would the owner entertain a cash as-is offer, a quick clean close and short due diligence? Where can I email the written terms? Thanks much!</t>
+          <t>Hello Jamila. Charles here with Paragon Government Solutions, and I'm interested in buying 103 Village Way, Columbia, SC 29209 for cash. Would the owner entertain a cash as-is offer, a quick clean close and short due diligence? Where can I email the written terms? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -982,7 +982,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Becky, hi. Charles here with Paragon Government Solutions, and I'd like to put in a cash offer on 115 Mulberry Ln, Columbia, SC 29201. would the owner entertain a cash as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Much appreciated!</t>
+          <t>Becky, hi. Charles here with Paragon Government Solutions, and I'd like to put in a cash offer on 115 Mulberry Ln, Columbia, SC 29201. Would the owner entertain a cash as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Hi there Bryant — Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 1111 Cloister Pl, Columbia, SC 29210. open to a discounted cash, as-is offer with fast close with a brief inspection window. Where can I email the written terms? Thanks!</t>
+          <t>Hi there Bryant — Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 1111 Cloister Pl, Columbia, SC 29210. Open to a discounted cash, as-is offer with fast close with a brief inspection window. Where can I email the written terms? Thanks!</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Good day Jamie. this is Charles Pleasant with Paragon Government Solutions, and I'd like to put in a cash offer on 2018 Hallmark Ct, Lakeland, FL 33803. is the seller open to a cash as-is offer, a quick clean close and short due diligence? What email should I send the written offer to? Thank you!</t>
+          <t>Good day Jamie. This is Charles Pleasant with Paragon Government Solutions, and I'd like to put in a cash offer on 2018 Hallmark Ct, Lakeland, FL 33803. Is the seller open to a cash as-is offer, a quick clean close and short due diligence? What email should I send the written offer to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Hey Amber. Charles Pleasant, Paragon Government Solutions, and I came across 314 Leton Dr, Columbia, SC 29210 and buy cash. is the seller open to a cash as-is offer, a quick clean close and short due diligence? What's the best email to send it to? Thank you!</t>
+          <t>Hey Amber. Charles Pleasant, Paragon Government Solutions, and I came across 314 Leton Dr, Columbia, SC 29210 and buy cash. Is the seller open to a cash as-is offer, a quick clean close and short due diligence? What's the best email to send it to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1242,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Hi there Angela — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 1024 Price Ave, Columbia, SC 29201. would the seller consider a cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Thanks!</t>
+          <t>Hi there Angela — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 1024 Price Ave, Columbia, SC 29201. Would the seller consider a cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Thanks!</t>
         </is>
       </c>
     </row>
@@ -1267,7 +1267,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Good day Anthony — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 11439 Ohio St, Detroit, MI 48204. any chance the seller would take a cash, as-is offer with a quick clean close and short due diligence. Where can I email the written terms? Thank you!</t>
+          <t>Good day Anthony — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 11439 Ohio St, Detroit, MI 48204. Any chance the seller would take a cash, as-is offer with a quick clean close and short due diligence. Where can I email the written terms? Thank you!</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Good day Avia. Charles Pleasant, Paragon Government Solutions, and I'm a cash investor looking at 205 Parliament Dr, Columbia, SC 29223. open to a discounted cash, as-is offer, fast cash close, short feasibility window? What email should I send the written offer to? Thank you!</t>
+          <t>Good day Avia. Charles Pleasant, Paragon Government Solutions, and I'm a cash investor looking at 205 Parliament Dr, Columbia, SC 29223. Open to a discounted cash, as-is offer, fast cash close, short feasibility window? What email should I send the written offer to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Good day Billy — Charles here with Paragon Government Solutions. I'm a cash investor looking at 23 Braiden Manor Rd, Columbia, SC 29209. is the seller open to a cash as-is offer with fast cash close, short feasibility window. What email should I send the written offer to? Thanks!</t>
+          <t>Good day Billy — Charles here with Paragon Government Solutions. I'm a cash investor looking at 23 Braiden Manor Rd, Columbia, SC 29209. Is the seller open to a cash as-is offer with fast cash close, short feasibility window. What email should I send the written offer to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Hello CHAD. I'm Charles with Paragon Government Solutions, and I'm a cash investor looking at 1169 WOODRUFF Avenue, Jacksonville, FL 32205. would the owner entertain a cash as-is offer, quick close and a short inspection? Where should I send the offer in writing? Thank you!</t>
+          <t>Hello CHAD. I'm Charles with Paragon Government Solutions, and I'm a cash investor looking at 1169 WOODRUFF Avenue, Jacksonville, FL 32205. Would the owner entertain a cash as-is offer, quick close and a short inspection? Where should I send the offer in writing? Thank you!</t>
         </is>
       </c>
     </row>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Cody, hi. my name's Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 104 Harbor Dr, Columbia, SC 29229 for cash. would the owner entertain a cash as-is offer, fast cash close, short feasibility window? What's the best email to send it to? Appreciate it!</t>
+          <t>Cody, hi. My name's Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 104 Harbor Dr, Columbia, SC 29229 for cash. Would the owner entertain a cash as-is offer, fast cash close, short feasibility window? What's the best email to send it to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>DIETCHI, hi — my name's Charles Pleasant, Paragon Government Solutions. I'm interested in buying 1007 Anarine Rd, Fayetteville, NC 28303 for cash. is the seller open to a cash as-is offer with close quickly, short inspection period. Best email for the formal offer? Thank you!</t>
+          <t>DIETCHI, hi — my name's Charles Pleasant, Paragon Government Solutions. I'm interested in buying 1007 Anarine Rd, Fayetteville, NC 28303 for cash. Is the seller open to a cash as-is offer with close quickly, short inspection period. Best email for the formal offer? Thank you!</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Hey Heather. I'm Charles with Paragon Government Solutions, and I came across 15385 Stansbury St, Detroit, MI 48227 and buy cash. is the seller open to a cash as-is offer, quick close and a short inspection? What email should I send the written offer to? Much appreciated!</t>
+          <t>Hey Heather. I'm Charles with Paragon Government Solutions, and I came across 15385 Stansbury St, Detroit, MI 48227 and buy cash. Is the seller open to a cash as-is offer, quick close and a short inspection? What email should I send the written offer to? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -1617,7 +1617,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Hey Melissa. this is Charles Pleasant with Paragon Government Solutions, and I'd like to put in a cash offer on 15534 Rocco Dr, Baker, LA 70714. could the seller look at a cash, as-is offer, fast cash close, short feasibility window? Where can I email the written terms? Appreciate it!</t>
+          <t>Hey Melissa. This is Charles Pleasant with Paragon Government Solutions, and I'd like to put in a cash offer on 15534 Rocco Dr, Baker, LA 70714. Could the seller look at a cash, as-is offer, fast cash close, short feasibility window? Where can I email the written terms? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Good day Patrick — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 135 Fox Squirrel Cir, Columbia, SC 29209. could the seller look at a cash, as-is offer with quick close and a short inspection. Where can I email the written terms? Thanks so much!</t>
+          <t>Good day Patrick — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 135 Fox Squirrel Cir, Columbia, SC 29209. Could the seller look at a cash, as-is offer with quick close and a short inspection. Where can I email the written terms? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Hello Sam — this is Charles Pleasant with Paragon Government Solutions. I'm reaching out about 10799 Worden St, Detroit, MI 48224. is the seller open to a cash as-is offer with close quickly, short inspection period. Where can I email the written terms? Thanks much!</t>
+          <t>Hello Sam — this is Charles Pleasant with Paragon Government Solutions. I'm reaching out about 10799 Worden St, Detroit, MI 48224. Is the seller open to a cash as-is offer with close quickly, short inspection period. Where can I email the written terms? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Good day there — my name's Charles Pleasant, Paragon Government Solutions. I'm reaching out about 3700 Ulmer Rd, Columbia, SC 29209. could the seller look at a cash, as-is offer with quick close and a short inspection. What's a good email for the written offer? Thanks!</t>
+          <t>Good day there — my name's Charles Pleasant, Paragon Government Solutions. I'm reaching out about 3700 Ulmer Rd, Columbia, SC 29209. Could the seller look at a cash, as-is offer with quick close and a short inspection. What's a good email for the written offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Good day Albert. Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 12717 Riad St, Grosse Pointe, MI 48224. could the seller look at a cash, as-is offer, close quickly, short inspection period? What's a good email for the written offer? Thanks so much!</t>
+          <t>Good day Albert. Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 12717 Riad St, Grosse Pointe, MI 48224. Could the seller look at a cash, as-is offer, close quickly, short inspection period? What's a good email for the written offer? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -1787,7 +1787,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Hi Alex — Charles here with Paragon Government Solutions. I'm reaching out about 201 Sandhurst Rd, Columbia, SC 29210. any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. What's the best email to send it to? Appreciate it!</t>
+          <t>Hi Alex — Charles here with Paragon Government Solutions. I'm reaching out about 201 Sandhurst Rd, Columbia, SC 29210. Any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. What's the best email to send it to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1812,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Hello Alex — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 1152 Vinewood St, Detroit, MI 48216. would the seller consider a cash, as-is offer with close quickly, short inspection period. Where can I email the written terms? Thanks much!</t>
+          <t>Hello Alex — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 1152 Vinewood St, Detroit, MI 48216. Would the seller consider a cash, as-is offer with close quickly, short inspection period. Where can I email the written terms? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -1837,7 +1837,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Hello Alexander. I'm Charles with Paragon Government Solutions, and I came across 16321 Stockbridge Ave, Cleveland, OH 44128 and buy cash. any chance the seller would take a cash, as-is offer, fast close with a brief inspection window? Where can I email the written terms? Appreciate it!</t>
+          <t>Hello Alexander. I'm Charles with Paragon Government Solutions, and I came across 16321 Stockbridge Ave, Cleveland, OH 44128 and buy cash. Any chance the seller would take a cash, as-is offer, fast close with a brief inspection window? Where can I email the written terms? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -1862,7 +1862,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Good day Alexandra. I'm Charles with Paragon Government Solutions, and I came across 219 Dixon Dr, Columbia, SC 29203 and buy cash. could the seller look at a cash, as-is offer, fast close with a brief inspection window? Best email for the formal offer? Thanks much!</t>
+          <t>Good day Alexandra. I'm Charles with Paragon Government Solutions, and I came across 219 Dixon Dr, Columbia, SC 29203 and buy cash. Could the seller look at a cash, as-is offer, fast close with a brief inspection window? Best email for the formal offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Good day Andy. Charles here with Paragon Government Solutions, and I'm reaching out about 6506 Christie Rd, Columbia, SC 29209. could the seller look at a cash, as-is offer, fast cash close, short feasibility window? What's a good email for the written offer? Thanks!</t>
+          <t>Good day Andy. Charles here with Paragon Government Solutions, and I'm reaching out about 6506 Christie Rd, Columbia, SC 29209. Could the seller look at a cash, as-is offer, fast cash close, short feasibility window? What's a good email for the written offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -2037,7 +2037,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Hi Bobby. Charles here with Paragon Government Solutions, and I'm a cash buyer interested in 14941 Littlefield St, Detroit, MI 48227. would the owner entertain a cash as-is offer, fast close with a brief inspection window? What's the best email to send it to? Appreciate it!</t>
+          <t>Hi Bobby. Charles here with Paragon Government Solutions, and I'm a cash buyer interested in 14941 Littlefield St, Detroit, MI 48227. Would the owner entertain a cash as-is offer, fast close with a brief inspection window? What's the best email to send it to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -2062,7 +2062,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Hi there Brad. my name's Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 1253 Mosser Dr, Columbia, SC 29203. would the owner entertain a cash as-is offer, a quick clean close and short due diligence? What email should I send the written offer to? Thank you!</t>
+          <t>Hi there Brad. My name's Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 1253 Mosser Dr, Columbia, SC 29203. Would the owner entertain a cash as-is offer, a quick clean close and short due diligence? What email should I send the written offer to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -2087,7 +2087,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Hey Brittany. Charles Pleasant, Paragon Government Solutions, and I came across 2065 Missouri St, Baton Rouge, LA 70802 and buy cash. is the seller open to a cash as-is offer, a quick clean close and short due diligence? What's a good email for the written offer? Thank you!</t>
+          <t>Hey Brittany. Charles Pleasant, Paragon Government Solutions, and I came across 2065 Missouri St, Baton Rouge, LA 70802 and buy cash. Is the seller open to a cash as-is offer, a quick clean close and short due diligence? What's a good email for the written offer? Thank you!</t>
         </is>
       </c>
     </row>
@@ -2137,7 +2137,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Hey Cameron — Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 9175 Everts St, Detroit, MI 48224. would the seller consider a cash, as-is offer with a quick clean close and short due diligence. What's the best email to send it to? Thanks much!</t>
+          <t>Hey Cameron — Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 9175 Everts St, Detroit, MI 48224. Would the seller consider a cash, as-is offer with a quick clean close and short due diligence. What's the best email to send it to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -2187,7 +2187,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Hi there CHRISTINA — this is Charles Pleasant with Paragon Government Solutions. I'm a cash investor looking at 1602 Gardenia Ave, Fayetteville, NC 28311. is the seller open to a cash as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Appreciate it!</t>
+          <t>Hi there CHRISTINA — this is Charles Pleasant with Paragon Government Solutions. I'm a cash investor looking at 1602 Gardenia Ave, Fayetteville, NC 28311. Is the seller open to a cash as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Hello Crystal — Charles Pleasant, Paragon Government Solutions. I came across 5648 S Sawyer Ave, Chicago, IL 60629 and buy cash. any chance the seller would take a cash, as-is offer with quick close and a short inspection. Best email for the formal offer? Thanks!</t>
+          <t>Hello Crystal — Charles Pleasant, Paragon Government Solutions. I came across 5648 S Sawyer Ave, Chicago, IL 60629 and buy cash. Any chance the seller would take a cash, as-is offer with quick close and a short inspection. Best email for the formal offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Ejaz, hi — Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 14440 Chelsea St, Detroit, MI 48213. is the seller open to a cash as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Appreciate it!</t>
+          <t>Ejaz, hi — Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 14440 Chelsea St, Detroit, MI 48213. Is the seller open to a cash as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -2412,7 +2412,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Hello Evan — my name's Charles Pleasant, Paragon Government Solutions. I'm interested in buying 4203 New Orleans St, Houston, TX 77020 for cash. any chance the seller would take a cash, as-is offer with close quickly, short inspection period. What's the best email to send it to? Much appreciated!</t>
+          <t>Hello Evan — my name's Charles Pleasant, Paragon Government Solutions. I'm interested in buying 4203 New Orleans St, Houston, TX 77020 for cash. Any chance the seller would take a cash, as-is offer with close quickly, short inspection period. What's the best email to send it to? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -2437,7 +2437,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Franco, hi — Charles here with Paragon Government Solutions. I'm a cash investor looking at 13027 Rosemary St, Detroit, MI 48213. could the seller look at a cash, as-is offer with fast close with a brief inspection window. Where should I send the offer in writing? Thanks much!</t>
+          <t>Franco, hi — Charles here with Paragon Government Solutions. I'm a cash investor looking at 13027 Rosemary St, Detroit, MI 48213. Could the seller look at a cash, as-is offer with fast close with a brief inspection window. Where should I send the offer in writing? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Greg, hi — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 20 Shuler Cir, Columbia, SC 29212. any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. Best email for the formal offer? Much appreciated!</t>
+          <t>Greg, hi — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 20 Shuler Cir, Columbia, SC 29212. Any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. Best email for the formal offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -2537,7 +2537,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Gregory, hi. this is Charles Pleasant with Paragon Government Solutions, and I'd like to put in a cash offer on 4440 Sexton Rd, Cleveland, OH 44105. is the seller open to a cash as-is offer, a quick clean close and short due diligence? What's the best email to send it to? Appreciate it!</t>
+          <t>Gregory, hi. This is Charles Pleasant with Paragon Government Solutions, and I'd like to put in a cash offer on 4440 Sexton Rd, Cleveland, OH 44105. Is the seller open to a cash as-is offer, a quick clean close and short due diligence? What's the best email to send it to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -2562,7 +2562,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Hassan, hi — my name's Charles Pleasant, Paragon Government Solutions. I came across 20569 Evergreen Rd, Detroit, MI 48219 and buy cash. would the owner entertain a cash as-is offer with quick close and a short inspection. What's the best email to send it to? Appreciate it!</t>
+          <t>Hassan, hi — my name's Charles Pleasant, Paragon Government Solutions. I came across 20569 Evergreen Rd, Detroit, MI 48219 and buy cash. Would the owner entertain a cash as-is offer with quick close and a short inspection. What's the best email to send it to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -2587,7 +2587,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>JACQUELYN, hi. Charles here with Paragon Government Solutions, and I'm reaching out about 2371 JAYSON Avenue, Jacksonville, FL 32208. could the seller look at a cash, as-is offer, a quick clean close and short due diligence? What's the best email to send it to? Much appreciated!</t>
+          <t>JACQUELYN, hi. Charles here with Paragon Government Solutions, and I'm reaching out about 2371 JAYSON Avenue, Jacksonville, FL 32208. Could the seller look at a cash, as-is offer, a quick clean close and short due diligence? What's the best email to send it to? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Hey Jay. I'm Charles with Paragon Government Solutions, and I'm reaching out about 209 Leago St, Houston, TX 77022. any chance the seller would take a cash, as-is offer, quick close and a short inspection? What email should I send the written offer to? Thanks much!</t>
+          <t>Hey Jay. I'm Charles with Paragon Government Solutions, and I'm reaching out about 209 Leago St, Houston, TX 77022. Any chance the seller would take a cash, as-is offer, quick close and a short inspection? What email should I send the written offer to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -2742,7 +2742,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Good day Kaila. Charles here with Paragon Government Solutions, and I'm a cash buyer interested in 17184 Dresden St, Detroit, MI 48205. open to a discounted cash, as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Much appreciated!</t>
+          <t>Good day Kaila. Charles here with Paragon Government Solutions, and I'm a cash buyer interested in 17184 Dresden St, Detroit, MI 48205. Open to a discounted cash, as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -2767,7 +2767,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Hello Kanaan — I'm Charles with Paragon Government Solutions. I came across 1018 W 104th Pl, Chicago, IL 60643 and buy cash. would the owner entertain a cash as-is offer with a quick clean close and short due diligence. What email should I send the written offer to? Thanks!</t>
+          <t>Hello Kanaan — I'm Charles with Paragon Government Solutions. I came across 1018 W 104th Pl, Chicago, IL 60643 and buy cash. Would the owner entertain a cash as-is offer with a quick clean close and short due diligence. What email should I send the written offer to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -2842,7 +2842,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Hello KRAVIN. Charles here with Paragon Government Solutions, and I'm reaching out about 2051 FRANK E Avenue, Jacksonville, FL 32208. open to a discounted cash, as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Thank you!</t>
+          <t>Hello KRAVIN. Charles here with Paragon Government Solutions, and I'm reaching out about 2051 FRANK E Avenue, Jacksonville, FL 32208. Open to a discounted cash, as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Thank you!</t>
         </is>
       </c>
     </row>
@@ -2892,7 +2892,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Hey LaToya. I'm Charles with Paragon Government Solutions, and I'm a cash investor looking at 1253 Rabon Pond Dr, Columbia, SC 29223. could the seller look at a cash, as-is offer, close quickly, short inspection period? Best email for the formal offer? Thanks so much!</t>
+          <t>Hey LaToya. I'm Charles with Paragon Government Solutions, and I'm a cash investor looking at 1253 Rabon Pond Dr, Columbia, SC 29223. Could the seller look at a cash, as-is offer, close quickly, short inspection period? Best email for the formal offer? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -2917,7 +2917,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Hi there LaTrina — Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 19783 Annott St, Detroit, MI 48205. would the seller consider a cash, as-is offer with close quickly, short inspection period. What email should I send the written offer to? Thanks!</t>
+          <t>Hi there LaTrina — Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 19783 Annott St, Detroit, MI 48205. Would the seller consider a cash, as-is offer with close quickly, short inspection period. What email should I send the written offer to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>Hello MAIDELYS — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 6978 PAUL HOWARD Drive, Jacksonville, FL 32222. would the owner entertain a cash as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Thanks!</t>
+          <t>Hello MAIDELYS — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 6978 PAUL HOWARD Drive, Jacksonville, FL 32222. Would the owner entertain a cash as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -3067,7 +3067,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Good day Mary — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 336 Byron Rd, Columbia, SC 29209. any chance the seller would take a cash, as-is offer with a quick clean close and short due diligence. Where can I email the written terms? Thank you!</t>
+          <t>Good day Mary — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 336 Byron Rd, Columbia, SC 29209. Any chance the seller would take a cash, as-is offer with a quick clean close and short due diligence. Where can I email the written terms? Thank you!</t>
         </is>
       </c>
     </row>
@@ -3217,7 +3217,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Hi Mladenka — Charles Pleasant, Paragon Government Solutions. I'm interested in buying 5308 W LEWIS Avenue W, Phoenix, AZ 85035 for cash. is the seller open to a cash as-is offer with close quickly, short inspection period. What's the best email to send it to? Thank you!</t>
+          <t>Hi Mladenka — Charles Pleasant, Paragon Government Solutions. I'm interested in buying 5308 W LEWIS Avenue W, Phoenix, AZ 85035 for cash. Is the seller open to a cash as-is offer with close quickly, short inspection period. What's the best email to send it to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Good day Mo — Charles here with Paragon Government Solutions. I came across 125 N Lake Pointe Dr, Columbia, SC 29229 and buy cash. is the seller open to a cash as-is offer with fast cash close, short feasibility window. Where can I email the written terms? Much appreciated!</t>
+          <t>Good day Mo — Charles here with Paragon Government Solutions. I came across 125 N Lake Pointe Dr, Columbia, SC 29229 and buy cash. Is the seller open to a cash as-is offer with fast cash close, short feasibility window. Where can I email the written terms? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -3267,7 +3267,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Good day Mohamed — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 16610 Collingham Dr, Detroit, MI 48205. could the seller look at a cash, as-is offer with a quick clean close and short due diligence. Best email for the formal offer? Thanks so much!</t>
+          <t>Good day Mohamed — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 16610 Collingham Dr, Detroit, MI 48205. Could the seller look at a cash, as-is offer with a quick clean close and short due diligence. Best email for the formal offer? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -3317,7 +3317,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>Hello Monika. Charles here with Paragon Government Solutions, and I'm a cash investor looking at 2947 Appaloosa Dr, Dallas, TX 75237. is the seller open to a cash as-is offer, close quickly, short inspection period? Where should I send the offer in writing? Thanks so much!</t>
+          <t>Hello Monika. Charles here with Paragon Government Solutions, and I'm a cash investor looking at 2947 Appaloosa Dr, Dallas, TX 75237. Is the seller open to a cash as-is offer, close quickly, short inspection period? Where should I send the offer in writing? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -3367,7 +3367,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Hi there Nadia — Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 17206 Fenelon St, Detroit, MI 48212. is the seller open to a cash as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Thanks much!</t>
+          <t>Hi there Nadia — Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 17206 Fenelon St, Detroit, MI 48212. Is the seller open to a cash as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -3392,7 +3392,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Good day NAJI. this is Charles Pleasant with Paragon Government Solutions, and I'm a cash buyer interested in 152 W 10TH Street, Jacksonville, FL 32206. is the seller open to a cash as-is offer, quick close and a short inspection? Best email for the formal offer? Thanks much!</t>
+          <t>Good day NAJI. This is Charles Pleasant with Paragon Government Solutions, and I'm a cash buyer interested in 152 W 10TH Street, Jacksonville, FL 32206. Is the seller open to a cash as-is offer, quick close and a short inspection? Best email for the formal offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -3417,7 +3417,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Hello Nazareth — my name's Charles Pleasant, Paragon Government Solutions. I came across 2223 Gray St, Detroit, MI 48215 and buy cash. could the seller look at a cash, as-is offer with quick close and a short inspection. Best email for the formal offer? Thanks!</t>
+          <t>Hello Nazareth — my name's Charles Pleasant, Paragon Government Solutions. I came across 2223 Gray St, Detroit, MI 48215 and buy cash. Could the seller look at a cash, as-is offer with quick close and a short inspection. Best email for the formal offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -3442,7 +3442,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Hello Pamela — Charles here with Paragon Government Solutions. I'm interested in buying 2912 Chestnut St, Columbia, SC 29204 for cash. would the seller consider a cash, as-is offer with a quick clean close and short due diligence. What email should I send the written offer to? Thanks much!</t>
+          <t>Hello Pamela — Charles here with Paragon Government Solutions. I'm interested in buying 2912 Chestnut St, Columbia, SC 29204 for cash. Would the seller consider a cash, as-is offer with a quick clean close and short due diligence. What email should I send the written offer to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -3467,7 +3467,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>Rachel, hi — Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 2539 Cherry St, Columbia, SC 29205. would the seller consider a cash, as-is offer with fast cash close, short feasibility window. Where can I email the written terms? Thanks so much!</t>
+          <t>Rachel, hi — Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 2539 Cherry St, Columbia, SC 29205. Would the seller consider a cash, as-is offer with fast cash close, short feasibility window. Where can I email the written terms? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -3492,7 +3492,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Good day Raquel — I'm Charles with Paragon Government Solutions. I'm interested in buying 1513 Dianne Ct SE, Atlanta, GA for cash. is the seller open to a cash as-is offer with fast close with a brief inspection window. What's the best email to send it to? Thanks so much!</t>
+          <t>Good day Raquel — I'm Charles with Paragon Government Solutions. I'm interested in buying 1513 Dianne Ct SE, Atlanta, GA for cash. Is the seller open to a cash as-is offer with fast close with a brief inspection window. What's the best email to send it to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Hello Sydney — Charles here with Paragon Government Solutions. I came across 425 Columbia St, Shreveport, LA 71104 and buy cash. could the seller look at a cash, as-is offer with fast cash close, short feasibility window. Where can I email the written terms? Appreciate it!</t>
+          <t>Hello Sydney — Charles here with Paragon Government Solutions. I came across 425 Columbia St, Shreveport, LA 71104 and buy cash. Could the seller look at a cash, as-is offer with fast cash close, short feasibility window. Where can I email the written terms? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -3672,7 +3672,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>Hi Timeka — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 2009 Las Cruces Ln, Dallas, TX 75217. open to a discounted cash, as-is offer with a quick clean close and short due diligence. What's the best email to send it to? Thanks!</t>
+          <t>Hi Timeka — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 2009 Las Cruces Ln, Dallas, TX 75217. Open to a discounted cash, as-is offer with a quick clean close and short due diligence. What's the best email to send it to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -3772,7 +3772,7 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>Will, hi. my name's Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 9426 Nyssa St, Houston, TX 77078. is the seller open to a cash as-is offer, close quickly, short inspection period? What's the best email to send it to? Thank you!</t>
+          <t>Will, hi. My name's Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 9426 Nyssa St, Houston, TX 77078. Is the seller open to a cash as-is offer, close quickly, short inspection period? What's the best email to send it to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -3822,7 +3822,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>Hi there WILLIAM — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 2995 Coleman Rd, Eastover, NC 28312. would the owner entertain a cash as-is offer with fast close with a brief inspection window. What's the best email to send it to? Much appreciated!</t>
+          <t>Hi there WILLIAM — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 2995 Coleman Rd, Eastover, NC 28312. Would the owner entertain a cash as-is offer with fast close with a brief inspection window. What's the best email to send it to? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -3882,7 +3882,7 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Good day there. this is Charles Pleasant with Paragon Government Solutions, and I came across 2737 Bristol Pl, New Orleans, LA 70131 and buy cash. could the seller look at a cash, as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Thanks so much!</t>
+          <t>Good day there. This is Charles Pleasant with Paragon Government Solutions, and I came across 2737 Bristol Pl, New Orleans, LA 70131 and buy cash. Could the seller look at a cash, as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -3902,7 +3902,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>there, hi, my name's Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 3109 Downes Grove Rd, Columbia, SC 29209; is the seller open to a cash as-is offer, quick close and a short inspection? I can send written terms today. Where should I send the offer in writing? Thank you!</t>
+          <t>There, hi, my name's Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 3109 Downes Grove Rd, Columbia, SC 29209; is the seller open to a cash as-is offer, quick close and a short inspection? I can send written terms today. Where should I send the offer in writing? Thank you!</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>Good day there — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 950 W ROMA Avenue, Phoenix, AZ 85013. is the seller open to a cash as-is offer with fast cash close, short feasibility window. What email should I send the written offer to? Thanks!</t>
+          <t>Good day there — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 950 W ROMA Avenue, Phoenix, AZ 85013. Is the seller open to a cash as-is offer with fast cash close, short feasibility window. What email should I send the written offer to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -3997,7 +3997,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Acencion, hi — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 16643 Seawolf Dr, Houston, TX 77062. would the seller consider a cash, as-is offer with quick close and a short inspection. Where should I send the offer in writing? Appreciate it!</t>
+          <t>Acencion, hi — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 16643 Seawolf Dr, Houston, TX 77062. Would the seller consider a cash, as-is offer with quick close and a short inspection. Where should I send the offer in writing? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -4022,7 +4022,7 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>Hello Adam — Charles Pleasant, Paragon Government Solutions. I came across 15394 Freeland St, Detroit, MI 48227 and buy cash. is the seller open to a cash as-is offer with close quickly, short inspection period. Where can I email the written terms? Appreciate it!</t>
+          <t>Hello Adam — Charles Pleasant, Paragon Government Solutions. I came across 15394 Freeland St, Detroit, MI 48227 and buy cash. Is the seller open to a cash as-is offer with close quickly, short inspection period. Where can I email the written terms? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -4072,7 +4072,7 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>Good day Adekunle. Charles Pleasant, Paragon Government Solutions, and I'm a cash investor looking at 11722 S Parnell Ave, Chicago, IL 60628. would the seller consider a cash, as-is offer, fast cash close, short feasibility window? Where can I email the written terms? Thanks so much!</t>
+          <t>Good day Adekunle. Charles Pleasant, Paragon Government Solutions, and I'm a cash investor looking at 11722 S Parnell Ave, Chicago, IL 60628. Would the seller consider a cash, as-is offer, fast cash close, short feasibility window? Where can I email the written terms? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -4122,7 +4122,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Hi Adrian. I'm Charles with Paragon Government Solutions, and I'd like to put in a cash offer on 15003 Manor St, Detroit, MI 48238. is the seller open to a cash as-is offer, quick close and a short inspection? Where can I email the written terms? Thanks!</t>
+          <t>Hi Adrian. I'm Charles with Paragon Government Solutions, and I'd like to put in a cash offer on 15003 Manor St, Detroit, MI 48238. Is the seller open to a cash as-is offer, quick close and a short inspection? Where can I email the written terms? Thanks!</t>
         </is>
       </c>
     </row>
@@ -4147,7 +4147,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>Good day Adrienne — I'm Charles with Paragon Government Solutions. I'm interested in buying 18402 Revere St, Detroit, MI 48234 for cash. any chance the seller would take a cash, as-is offer with close quickly, short inspection period. What's a good email for the written offer? Appreciate it!</t>
+          <t>Good day Adrienne — I'm Charles with Paragon Government Solutions. I'm interested in buying 18402 Revere St, Detroit, MI 48234 for cash. Any chance the seller would take a cash, as-is offer with close quickly, short inspection period. What's a good email for the written offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -4197,7 +4197,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>Hey Alannah. Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 1314 Red Ridge Ter, Columbia, SC 29203. any chance the seller would take a cash, as-is offer, close quickly, short inspection period? What's the best email to send it to? Appreciate it!</t>
+          <t>Hey Alannah. Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 1314 Red Ridge Ter, Columbia, SC 29203. Any chance the seller would take a cash, as-is offer, close quickly, short inspection period? What's the best email to send it to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>Hi Alejandro — this is Charles Pleasant with Paragon Government Solutions. I'm a cash investor looking at 919 Christine St, Houston, TX 77017. would the owner entertain a cash as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Appreciate it!</t>
+          <t>Hi Alejandro — this is Charles Pleasant with Paragon Government Solutions. I'm a cash investor looking at 919 Christine St, Houston, TX 77017. Would the owner entertain a cash as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>Hey Alex — I'm Charles with Paragon Government Solutions. I'm a cash buyer interested in 3906 Metropolitan Ave, Dallas, TX 75210. any chance the seller would take a cash, as-is offer with fast close with a brief inspection window. Best email for the formal offer? Thank you!</t>
+          <t>Hey Alex — I'm Charles with Paragon Government Solutions. I'm a cash buyer interested in 3906 Metropolitan Ave, Dallas, TX 75210. Any chance the seller would take a cash, as-is offer with fast close with a brief inspection window. Best email for the formal offer? Thank you!</t>
         </is>
       </c>
     </row>
@@ -4322,7 +4322,7 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>Alex, hi. my name's Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 423 Exchange St, Houston, TX 77020 for cash. would the seller consider a cash, as-is offer, quick close and a short inspection? Where should I send the offer in writing? Thanks much!</t>
+          <t>Alex, hi. My name's Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 423 Exchange St, Houston, TX 77020 for cash. Would the seller consider a cash, as-is offer, quick close and a short inspection? Where should I send the offer in writing? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -4347,7 +4347,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>Hi Alexander — this is Charles Pleasant with Paragon Government Solutions. I'm a cash investor looking at 2317 NW 30th Ter, Cape Coral, FL 33993. open to a discounted cash, as-is offer with quick close and a short inspection. What's a good email for the written offer? Much appreciated!</t>
+          <t>Hi Alexander — this is Charles Pleasant with Paragon Government Solutions. I'm a cash investor looking at 2317 NW 30th Ter, Cape Coral, FL 33993. Open to a discounted cash, as-is offer with quick close and a short inspection. What's a good email for the written offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -4372,7 +4372,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>Alexandria, hi. I'm Charles with Paragon Government Solutions, and I'm interested in buying 5981 Arapaho Rd #1607, Dallas TX 75248 for cash. could the seller look at a cash, as-is offer, fast cash close, short feasibility window? What email should I send the written offer to? Thanks much!</t>
+          <t>Alexandria, hi. I'm Charles with Paragon Government Solutions, and I'm interested in buying 5981 Arapaho Rd #1607, Dallas TX 75248 for cash. Could the seller look at a cash, as-is offer, fast cash close, short feasibility window? What email should I send the written offer to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -4397,7 +4397,7 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>Good day Alexis. Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 17360 Mansfield St, Detroit, MI 48235. would the seller consider a cash, as-is offer, close quickly, short inspection period? Where can I email the written terms? Thanks!</t>
+          <t>Good day Alexis. Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 17360 Mansfield St, Detroit, MI 48235. Would the seller consider a cash, as-is offer, close quickly, short inspection period? Where can I email the written terms? Thanks!</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4422,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>Hi Ali — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 11718 Plainview Ave, Detroit, MI 48228. any chance the seller would take a cash, as-is offer with quick close and a short inspection. Where should I send the offer in writing? Thanks!</t>
+          <t>Hi Ali — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 11718 Plainview Ave, Detroit, MI 48228. Any chance the seller would take a cash, as-is offer with quick close and a short inspection. Where should I send the offer in writing? Thanks!</t>
         </is>
       </c>
     </row>
@@ -4447,7 +4447,7 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>Hi Ali. Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 9030 Plainview Ave, Detroit, MI 48228 for cash. is the seller open to a cash as-is offer, fast close with a brief inspection window? What's a good email for the written offer? Thanks much!</t>
+          <t>Hi Ali. Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 9030 Plainview Ave, Detroit, MI 48228 for cash. Is the seller open to a cash as-is offer, fast close with a brief inspection window? What's a good email for the written offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -4522,7 +4522,7 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>Hey Amanda — I'm Charles with Paragon Government Solutions. I'm a cash buyer interested in 10323 Sweetbrook Dr, Houston, TX 77038. is the seller open to a cash as-is offer with fast close with a brief inspection window. Where can I email the written terms? Much appreciated!</t>
+          <t>Hey Amanda — I'm Charles with Paragon Government Solutions. I'm a cash buyer interested in 10323 Sweetbrook Dr, Houston, TX 77038. Is the seller open to a cash as-is offer with fast close with a brief inspection window. Where can I email the written terms? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -4547,7 +4547,7 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>Hello AMANDA. I'm Charles with Paragon Government Solutions, and I'm a cash investor looking at 1009 Bugle Call Dr, Fayetteville, NC 28314. open to a discounted cash, as-is offer, fast cash close, short feasibility window? Where can I email the written terms? Thanks so much!</t>
+          <t>Hello AMANDA. I'm Charles with Paragon Government Solutions, and I'm a cash investor looking at 1009 Bugle Call Dr, Fayetteville, NC 28314. Open to a discounted cash, as-is offer, fast cash close, short feasibility window? Where can I email the written terms? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -4697,7 +4697,7 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>Hi AMY — Charles Pleasant, Paragon Government Solutions. I came across 7092 Pantego Dr, Fayetteville, NC 28314 and buy cash. would the owner entertain a cash as-is offer with quick close and a short inspection. Where should I send the offer in writing? Thanks much!</t>
+          <t>Hi AMY — Charles Pleasant, Paragon Government Solutions. I came across 7092 Pantego Dr, Fayetteville, NC 28314 and buy cash. Would the owner entertain a cash as-is offer with quick close and a short inspection. Where should I send the offer in writing? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -4722,7 +4722,7 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>Hello Andre — Charles here with Paragon Government Solutions. I'm reaching out about 19447 Sunset St, Detroit, MI 48234. is the seller open to a cash as-is offer with quick close and a short inspection. Best email for the formal offer? Thanks!</t>
+          <t>Hello Andre — Charles here with Paragon Government Solutions. I'm reaching out about 19447 Sunset St, Detroit, MI 48234. Is the seller open to a cash as-is offer with quick close and a short inspection. Best email for the formal offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -4772,7 +4772,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>Hi Angel. this is Charles Pleasant with Paragon Government Solutions, and I came across 7606 Blessing Ave, Austin, TX 78752 and buy cash. would the seller consider a cash, as-is offer, a quick clean close and short due diligence? What's a good email for the written offer? Appreciate it!</t>
+          <t>Hi Angel. This is Charles Pleasant with Paragon Government Solutions, and I came across 7606 Blessing Ave, Austin, TX 78752 and buy cash. Would the seller consider a cash, as-is offer, a quick clean close and short due diligence? What's a good email for the written offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>Hello Angela — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 16 Carroll St, Trenton, NJ 08609. any chance the seller would take a cash, as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Thanks so much!</t>
+          <t>Hello Angela — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 16 Carroll St, Trenton, NJ 08609. Any chance the seller would take a cash, as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -4947,7 +4947,7 @@
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>Hi there ANTHONY. Charles here with Paragon Government Solutions, and I came across 2917 PARR Court E, Jacksonville, FL 32216 and buy cash. would the seller consider a cash, as-is offer, close quickly, short inspection period? What email should I send the written offer to? Much appreciated!</t>
+          <t>Hi there ANTHONY. Charles here with Paragon Government Solutions, and I came across 2917 PARR Court E, Jacksonville, FL 32216 and buy cash. Would the seller consider a cash, as-is offer, close quickly, short inspection period? What email should I send the written offer to? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -4997,7 +4997,7 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>Good day ANTOINETTE — Charles here with Paragon Government Solutions. I'm interested in buying 9419 SCADLOCKE Road, Jacksonville, FL 32208 for cash. is the seller open to a cash as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Thanks much!</t>
+          <t>Good day ANTOINETTE — Charles here with Paragon Government Solutions. I'm interested in buying 9419 SCADLOCKE Road, Jacksonville, FL 32208 for cash. Is the seller open to a cash as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -5022,7 +5022,7 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>Hey April — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 6510 Portsmouth Dr, Fayetteville, NC 28314. is the seller open to a cash as-is offer with a quick clean close and short due diligence. What's the best email to send it to? Appreciate it!</t>
+          <t>Hey April — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 6510 Portsmouth Dr, Fayetteville, NC 28314. Is the seller open to a cash as-is offer with a quick clean close and short due diligence. What's the best email to send it to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -5047,7 +5047,7 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>Good day APRYL — my name's Charles Pleasant, Paragon Government Solutions. I came across 2225 THIERVY Drive, Jacksonville, FL 32210 and buy cash. is the seller open to a cash as-is offer with close quickly, short inspection period. What's a good email for the written offer? Thanks!</t>
+          <t>Good day APRYL — my name's Charles Pleasant, Paragon Government Solutions. I came across 2225 THIERVY Drive, Jacksonville, FL 32210 and buy cash. Is the seller open to a cash as-is offer with close quickly, short inspection period. What's a good email for the written offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -5097,7 +5097,7 @@
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>Hey Arianna. my name's Charles Pleasant, Paragon Government Solutions, and I came across 4153 Concord St, Detroit, MI 48207 and buy cash. would the seller consider a cash, as-is offer, fast close with a brief inspection window? What's a good email for the written offer? Thanks much!</t>
+          <t>Hey Arianna. My name's Charles Pleasant, Paragon Government Solutions, and I came across 4153 Concord St, Detroit, MI 48207 and buy cash. Would the seller consider a cash, as-is offer, fast close with a brief inspection window? What's a good email for the written offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -5172,7 +5172,7 @@
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>Hello ARMANDO — Charles here with Paragon Government Solutions. I'm a cash investor looking at 153 Knapp Ave, Hamilton, NJ 08610. could the seller look at a cash, as-is offer with fast cash close, short feasibility window. What email should I send the written offer to? Thank you!</t>
+          <t>Hello ARMANDO — Charles here with Paragon Government Solutions. I'm a cash investor looking at 153 Knapp Ave, Hamilton, NJ 08610. Could the seller look at a cash, as-is offer with fast cash close, short feasibility window. What email should I send the written offer to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -5222,7 +5222,7 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>Hey Ashley — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 3879 W 21st St, Cleveland, OH 44109. any chance the seller would take a cash, as-is offer with quick close and a short inspection. What's the best email to send it to? Thank you!</t>
+          <t>Hey Ashley — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 3879 W 21st St, Cleveland, OH 44109. Any chance the seller would take a cash, as-is offer with quick close and a short inspection. What's the best email to send it to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -5247,7 +5247,7 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>Hello Ashley — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 414 Angel Grove Ln, Columbia, SC 29210. open to a discounted cash, as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Much appreciated!</t>
+          <t>Hello Ashley — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 414 Angel Grove Ln, Columbia, SC 29210. Open to a discounted cash, as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -5272,7 +5272,7 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>Hi Ashley. my name's Charles Pleasant, Paragon Government Solutions, and I came across 1008 Walnut Ave, Baltimore, MD 21229 and buy cash. is the seller open to a cash as-is offer, fast close with a brief inspection window? Where can I email the written terms? Much appreciated!</t>
+          <t>Hi Ashley. My name's Charles Pleasant, Paragon Government Solutions, and I came across 1008 Walnut Ave, Baltimore, MD 21229 and buy cash. Is the seller open to a cash as-is offer, fast close with a brief inspection window? Where can I email the written terms? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -5297,7 +5297,7 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>Hi Ashley — my name's Charles Pleasant, Paragon Government Solutions. I'm reaching out about 19261 Mitchell St, Detroit, MI 48234. would the seller consider a cash, as-is offer with fast cash close, short feasibility window. Best email for the formal offer? Thanks so much!</t>
+          <t>Hi Ashley — my name's Charles Pleasant, Paragon Government Solutions. I'm reaching out about 19261 Mitchell St, Detroit, MI 48234. Would the seller consider a cash, as-is offer with fast cash close, short feasibility window. Best email for the formal offer? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -5372,7 +5372,7 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>Hey Babajide — I'm Charles with Paragon Government Solutions. I came across 317 E 134th St, Chicago, IL 60827 and buy cash. is the seller open to a cash as-is offer with a quick clean close and short due diligence. Where can I email the written terms? Thanks much!</t>
+          <t>Hey Babajide — I'm Charles with Paragon Government Solutions. I came across 317 E 134th St, Chicago, IL 60827 and buy cash. Is the seller open to a cash as-is offer with a quick clean close and short due diligence. Where can I email the written terms? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -5397,7 +5397,7 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>Hi Bailee. Charles here with Paragon Government Solutions, and I'm a cash investor looking at 11144 Sanford St, Detroit, MI 48205. would the seller consider a cash, as-is offer, fast close with a brief inspection window? Where can I email the written terms? Thanks so much!</t>
+          <t>Hi Bailee. Charles here with Paragon Government Solutions, and I'm a cash investor looking at 11144 Sanford St, Detroit, MI 48205. Would the seller consider a cash, as-is offer, fast close with a brief inspection window? Where can I email the written terms? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -5422,7 +5422,7 @@
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>Hello Barbara — Charles here with Paragon Government Solutions. I'm a cash investor looking at 2336 Albert St, Alexandria, LA 71301. would the seller consider a cash, as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Much appreciated!</t>
+          <t>Hello Barbara — Charles here with Paragon Government Solutions. I'm a cash investor looking at 2336 Albert St, Alexandria, LA 71301. Would the seller consider a cash, as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -5447,7 +5447,7 @@
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>Hey BARBARA — my name's Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 1603 W 14TH Street, Jacksonville, FL 32209. open to a discounted cash, as-is offer with fast cash close, short feasibility window. Where should I send the offer in writing? Thank you!</t>
+          <t>Hey BARBARA — my name's Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 1603 W 14TH Street, Jacksonville, FL 32209. Open to a discounted cash, as-is offer with fast cash close, short feasibility window. Where should I send the offer in writing? Thank you!</t>
         </is>
       </c>
     </row>
@@ -5522,7 +5522,7 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>Hello Belle — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 413 Seton Hall Dr, Columbia, SC 29223. could the seller look at a cash, as-is offer with a quick clean close and short due diligence. Best email for the formal offer? Thanks!</t>
+          <t>Hello Belle — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 413 Seton Hall Dr, Columbia, SC 29223. Could the seller look at a cash, as-is offer with a quick clean close and short due diligence. Best email for the formal offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -5547,7 +5547,7 @@
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>Hi Benjamin — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 1005 Wildwood Ave, Columbia, SC 29203. any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. Where should I send the offer in writing? Much appreciated!</t>
+          <t>Hi Benjamin — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 1005 Wildwood Ave, Columbia, SC 29203. Any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. Where should I send the offer in writing? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -5697,7 +5697,7 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>Hi Brandon. Charles here with Paragon Government Solutions, and I'm interested in buying 15237 Carlisle St, Detroit, MI 48205 for cash. is the seller open to a cash as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Thanks!</t>
+          <t>Hi Brandon. Charles here with Paragon Government Solutions, and I'm interested in buying 15237 Carlisle St, Detroit, MI 48205 for cash. Is the seller open to a cash as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -5747,7 +5747,7 @@
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>Hey Brian. I'm Charles with Paragon Government Solutions, and I'm a cash buyer interested in 30 Ward Ct, Columbia, SC 29223. would the seller consider a cash, as-is offer, fast close with a brief inspection window? Best email for the formal offer? Thanks!</t>
+          <t>Hey Brian. I'm Charles with Paragon Government Solutions, and I'm a cash buyer interested in 30 Ward Ct, Columbia, SC 29223. Would the seller consider a cash, as-is offer, fast close with a brief inspection window? Best email for the formal offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -5772,7 +5772,7 @@
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>Hi there Brian. Charles here with Paragon Government Solutions, and I'm a cash buyer interested in 1648 Tampa Bay Dr, Dallas, TX 75217. would the seller consider a cash, as-is offer, quick close and a short inspection? What's the best email to send it to? Much appreciated!</t>
+          <t>Hi there Brian. Charles here with Paragon Government Solutions, and I'm a cash buyer interested in 1648 Tampa Bay Dr, Dallas, TX 75217. Would the seller consider a cash, as-is offer, quick close and a short inspection? What's the best email to send it to? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -5797,7 +5797,7 @@
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>Hi Brianna — my name's Charles Pleasant, Paragon Government Solutions. I'm interested in buying 6015 N 32nd Dr, Phoenix, AZ 85017 for cash. any chance the seller would take a cash, as-is offer with fast close with a brief inspection window. Where should I send the offer in writing? Thanks!</t>
+          <t>Hi Brianna — my name's Charles Pleasant, Paragon Government Solutions. I'm interested in buying 6015 N 32nd Dr, Phoenix, AZ 85017 for cash. Any chance the seller would take a cash, as-is offer with fast close with a brief inspection window. Where should I send the offer in writing? Thanks!</t>
         </is>
       </c>
     </row>
@@ -5897,7 +5897,7 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>Bryton, hi — Charles here with Paragon Government Solutions. I'd like to put in a cash offer on 8215 Leather Market St, Houston, TX 77064. any chance the seller would take a cash, as-is offer with a quick clean close and short due diligence. Where should I send the offer in writing? Thanks so much!</t>
+          <t>Bryton, hi — Charles here with Paragon Government Solutions. I'd like to put in a cash offer on 8215 Leather Market St, Houston, TX 77064. Any chance the seller would take a cash, as-is offer with a quick clean close and short due diligence. Where should I send the offer in writing? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -5972,7 +5972,7 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>Hi Carly. my name's Charles Pleasant, Paragon Government Solutions, and I'm a cash investor looking at 10316 Ridge Oak St, Dallas, TX 75227. any chance the seller would take a cash, as-is offer, quick close and a short inspection? Best email for the formal offer? Much appreciated!</t>
+          <t>Hi Carly. My name's Charles Pleasant, Paragon Government Solutions, and I'm a cash investor looking at 10316 Ridge Oak St, Dallas, TX 75227. Any chance the seller would take a cash, as-is offer, quick close and a short inspection? Best email for the formal offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -6022,7 +6022,7 @@
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>Hi Carmen. Charles here with Paragon Government Solutions, and I'm a cash investor looking at 7216 OAKWOOD Drive, Jacksonville, FL 32211. is the seller open to a cash as-is offer, close quickly, short inspection period? What email should I send the written offer to? Appreciate it!</t>
+          <t>Hi Carmen. Charles here with Paragon Government Solutions, and I'm a cash investor looking at 7216 OAKWOOD Drive, Jacksonville, FL 32211. Is the seller open to a cash as-is offer, close quickly, short inspection period? What email should I send the written offer to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -6072,7 +6072,7 @@
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>Good day Carolinas — I'm Charles with Paragon Government Solutions. I'm a cash buyer interested in 4723 Linden St, Columbia, SC 29203. would the seller consider a cash, as-is offer with fast close with a brief inspection window. Best email for the formal offer? Thanks much!</t>
+          <t>Good day Carolinas — I'm Charles with Paragon Government Solutions. I'm a cash buyer interested in 4723 Linden St, Columbia, SC 29203. Would the seller consider a cash, as-is offer with fast close with a brief inspection window. Best email for the formal offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -6097,7 +6097,7 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>Carolyn, hi. my name's Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 7201 S Vernon Ave, Chicago, IL 60619. would the seller consider a cash, as-is offer, a quick clean close and short due diligence? What email should I send the written offer to? Thank you!</t>
+          <t>Carolyn, hi. My name's Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 7201 S Vernon Ave, Chicago, IL 60619. Would the seller consider a cash, as-is offer, a quick clean close and short due diligence? What email should I send the written offer to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -6172,7 +6172,7 @@
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>Carrie, hi. I'm Charles with Paragon Government Solutions, and I'm a cash investor looking at 1663 W 30th St, Jacksonville, FL 32209. would the owner entertain a cash as-is offer, a quick clean close and short due diligence? What's a good email for the written offer? Thanks!</t>
+          <t>Carrie, hi. I'm Charles with Paragon Government Solutions, and I'm a cash investor looking at 1663 W 30th St, Jacksonville, FL 32209. Would the owner entertain a cash as-is offer, a quick clean close and short due diligence? What's a good email for the written offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -6197,7 +6197,7 @@
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>Hello Carrie — this is Charles Pleasant with Paragon Government Solutions. I came across 4243 Mandel Dr, Columbia, SC 29210 and buy cash. could the seller look at a cash, as-is offer with quick close and a short inspection. What's the best email to send it to? Appreciate it!</t>
+          <t>Hello Carrie — this is Charles Pleasant with Paragon Government Solutions. I came across 4243 Mandel Dr, Columbia, SC 29210 and buy cash. Could the seller look at a cash, as-is offer with quick close and a short inspection. What's the best email to send it to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -6222,7 +6222,7 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>Hi Caryn — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 10017 Morocco Rd, Houston, TX 77041. any chance the seller would take a cash, as-is offer with quick close and a short inspection. Best email for the formal offer? Thanks much!</t>
+          <t>Hi Caryn — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 10017 Morocco Rd, Houston, TX 77041. Any chance the seller would take a cash, as-is offer with quick close and a short inspection. Best email for the formal offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -6247,7 +6247,7 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>Hi there Casey — Charles here with Paragon Government Solutions. I came across 3414 Maybank St, Columbia, SC 29204 and buy cash. could the seller look at a cash, as-is offer with a quick clean close and short due diligence. Where should I send the offer in writing? Thanks much!</t>
+          <t>Hi there Casey — Charles here with Paragon Government Solutions. I came across 3414 Maybank St, Columbia, SC 29204 and buy cash. Could the seller look at a cash, as-is offer with a quick clean close and short due diligence. Where should I send the offer in writing? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -6347,7 +6347,7 @@
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>Hey CC — Charles Pleasant, Paragon Government Solutions. I'm reaching out about 5418 MINOSA Court, Jacksonville, FL 32209. could the seller look at a cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Thanks much!</t>
+          <t>Hey CC — Charles Pleasant, Paragon Government Solutions. I'm reaching out about 5418 MINOSA Court, Jacksonville, FL 32209. Could the seller look at a cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -6397,7 +6397,7 @@
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>Good day Century — Charles Pleasant, Paragon Government Solutions. I'm reaching out about 1033 Glencroft Drive, Columbia, SC 29210. open to a discounted cash, as-is offer with close quickly, short inspection period. Where can I email the written terms? Thanks so much!</t>
+          <t>Good day Century — Charles Pleasant, Paragon Government Solutions. I'm reaching out about 1033 Glencroft Drive, Columbia, SC 29210. Open to a discounted cash, as-is offer with close quickly, short inspection period. Where can I email the written terms? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6447,7 @@
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>Hey Cerita. Charles here with Paragon Government Solutions, and I'd like to put in a cash offer on 528 1st St SW, Birmingham, AL 35211. open to a discounted cash, as-is offer, a quick clean close and short due diligence? Where can I email the written terms? Thanks so much!</t>
+          <t>Hey Cerita. Charles here with Paragon Government Solutions, and I'd like to put in a cash offer on 528 1st St SW, Birmingham, AL 35211. Open to a discounted cash, as-is offer, a quick clean close and short due diligence? Where can I email the written terms? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -6472,7 +6472,7 @@
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>Hi Chad. Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 2426 Dora Ave NW, Albuquerque, NM 87104 for cash. any chance the seller would take a cash, as-is offer, fast cash close, short feasibility window? Best email for the formal offer? Thank you!</t>
+          <t>Hi Chad. Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 2426 Dora Ave NW, Albuquerque, NM 87104 for cash. Any chance the seller would take a cash, as-is offer, fast cash close, short feasibility window? Best email for the formal offer? Thank you!</t>
         </is>
       </c>
     </row>
@@ -6572,7 +6572,7 @@
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>Good day Charles. Charles here with Paragon Government Solutions, and I'm a cash buyer interested in 334 Carver St, Lafayette, LA 70501. would the owner entertain a cash as-is offer, a quick clean close and short due diligence? What's a good email for the written offer? Thanks so much!</t>
+          <t>Good day Charles. Charles here with Paragon Government Solutions, and I'm a cash buyer interested in 334 Carver St, Lafayette, LA 70501. Would the owner entertain a cash as-is offer, a quick clean close and short due diligence? What's a good email for the written offer? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -6622,7 +6622,7 @@
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>Hello CHERYL. Charles here with Paragon Government Solutions, and I'm interested in buying 9711 SKYDIVE Court, Jacksonville, FL 32221 for cash. open to a discounted cash, as-is offer, close quickly, short inspection period? Where should I send the offer in writing? Appreciate it!</t>
+          <t>Hello CHERYL. Charles here with Paragon Government Solutions, and I'm interested in buying 9711 SKYDIVE Court, Jacksonville, FL 32221 for cash. Open to a discounted cash, as-is offer, close quickly, short inspection period? Where should I send the offer in writing? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -6647,7 +6647,7 @@
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>Hello Chip — Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 329 Shagbark Ave, Columbia, SC 29209. is the seller open to a cash as-is offer with fast close with a brief inspection window. What's the best email to send it to? Thanks much!</t>
+          <t>Hello Chip — Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 329 Shagbark Ave, Columbia, SC 29209. Is the seller open to a cash as-is offer with fast close with a brief inspection window. What's the best email to send it to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -6672,7 +6672,7 @@
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>Hi Chip. Charles here with Paragon Government Solutions, and I'm a cash investor looking at 329 Shagbark Ave, Columbia, SC 29209. any chance the seller would take a cash, as-is offer, a quick clean close and short due diligence? Best email for the formal offer? Thanks!</t>
+          <t>Hi Chip. Charles here with Paragon Government Solutions, and I'm a cash investor looking at 329 Shagbark Ave, Columbia, SC 29209. Any chance the seller would take a cash, as-is offer, a quick clean close and short due diligence? Best email for the formal offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -6747,7 +6747,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>Hey Chris — I'm Charles with Paragon Government Solutions. I'm a cash buyer interested in 3405 Gwynns Falls Pkwy, Baltimore, MD 21216. could the seller look at a cash, as-is offer with quick close and a short inspection. Where should I send the offer in writing? Thanks much!</t>
+          <t>Hey Chris — I'm Charles with Paragon Government Solutions. I'm a cash buyer interested in 3405 Gwynns Falls Pkwy, Baltimore, MD 21216. Could the seller look at a cash, as-is offer with quick close and a short inspection. Where should I send the offer in writing? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -6797,7 +6797,7 @@
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>Hi there Chris — Charles here with Paragon Government Solutions. I'm a cash buyer interested in 3804 Park Heights Ave, Baltimore, MD 21215. open to a discounted cash, as-is offer with fast close with a brief inspection window. Best email for the formal offer? Thanks much!</t>
+          <t>Hi there Chris — Charles here with Paragon Government Solutions. I'm a cash buyer interested in 3804 Park Heights Ave, Baltimore, MD 21215. Open to a discounted cash, as-is offer with fast close with a brief inspection window. Best email for the formal offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -6872,7 +6872,7 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>Hi there Christine — I'm Charles with Paragon Government Solutions. I'm reaching out about 2633 W Grand Blvd, Detroit, MI 48208. any chance the seller would take a cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Thanks!</t>
+          <t>Hi there Christine — I'm Charles with Paragon Government Solutions. I'm reaching out about 2633 W Grand Blvd, Detroit, MI 48208. Any chance the seller would take a cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Thanks!</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>CHRISTOPHER, hi. my name's Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 1404 Valencia Dr, Fayetteville, NC 28303. could the seller look at a cash, as-is offer, quick close and a short inspection? Where should I send the offer in writing? Thanks so much!</t>
+          <t>CHRISTOPHER, hi. My name's Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 1404 Valencia Dr, Fayetteville, NC 28303. Could the seller look at a cash, as-is offer, quick close and a short inspection? Where should I send the offer in writing? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -6947,7 +6947,7 @@
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>Good day Chuck — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 711 S Montclair Ave, Dallas, TX 75208. is the seller open to a cash as-is offer with fast close with a brief inspection window. What's a good email for the written offer? Thanks so much!</t>
+          <t>Good day Chuck — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 711 S Montclair Ave, Dallas, TX 75208. Is the seller open to a cash as-is offer with fast close with a brief inspection window. What's a good email for the written offer? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -6972,7 +6972,7 @@
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>Cindy, hi — I'm Charles with Paragon Government Solutions. I'm interested in buying 2237 Kingswood Dr, Columbia, SC 29205 for cash. could the seller look at a cash, as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Thanks much!</t>
+          <t>Cindy, hi — I'm Charles with Paragon Government Solutions. I'm interested in buying 2237 Kingswood Dr, Columbia, SC 29205 for cash. Could the seller look at a cash, as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -7022,7 +7022,7 @@
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>Cindy, hi. Charles here with Paragon Government Solutions, and I'm a cash buyer interested in 1703 Alba Dr, Columbia, SC 29209. would the seller consider a cash, as-is offer, a quick clean close and short due diligence? What's the best email to send it to? Thanks much!</t>
+          <t>Cindy, hi. Charles here with Paragon Government Solutions, and I'm a cash buyer interested in 1703 Alba Dr, Columbia, SC 29209. Would the seller consider a cash, as-is offer, a quick clean close and short due diligence? What's the best email to send it to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -7072,7 +7072,7 @@
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>Hi there Clarence — Charles here with Paragon Government Solutions. I'm a cash investor looking at 7707 Candlegreen Ln, Houston, TX 77071. would the owner entertain a cash as-is offer with close quickly, short inspection period. What's a good email for the written offer? Appreciate it!</t>
+          <t>Hi there Clarence — Charles here with Paragon Government Solutions. I'm a cash investor looking at 7707 Candlegreen Ln, Houston, TX 77071. Would the owner entertain a cash as-is offer with close quickly, short inspection period. What's a good email for the written offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -7097,7 +7097,7 @@
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>Hey Claudia. I'm Charles with Paragon Government Solutions, and I'm interested in buying 20495 Mendota St, Detroit, MI 48221 for cash. any chance the seller would take a cash, as-is offer, quick close and a short inspection? Where can I email the written terms? Thank you!</t>
+          <t>Hey Claudia. I'm Charles with Paragon Government Solutions, and I'm interested in buying 20495 Mendota St, Detroit, MI 48221 for cash. Any chance the seller would take a cash, as-is offer, quick close and a short inspection? Where can I email the written terms? Thank you!</t>
         </is>
       </c>
     </row>
@@ -7122,7 +7122,7 @@
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>Hi Clay — this is Charles Pleasant with Paragon Government Solutions. I came across 1522 W Taylor St, Phoenix, AZ 85007 and buy cash. is the seller open to a cash as-is offer with fast cash close, short feasibility window. Best email for the formal offer? Much appreciated!</t>
+          <t>Hi Clay — this is Charles Pleasant with Paragon Government Solutions. I came across 1522 W Taylor St, Phoenix, AZ 85007 and buy cash. Is the seller open to a cash as-is offer with fast cash close, short feasibility window. Best email for the formal offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -7147,7 +7147,7 @@
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>Good day Cliff. my name's Charles Pleasant, Paragon Government Solutions, and I'm a cash buyer interested in 11604 Tuscora Ave, Cleveland, OH 44108. would the owner entertain a cash as-is offer, fast cash close, short feasibility window? What email should I send the written offer to? Thanks!</t>
+          <t>Good day Cliff. My name's Charles Pleasant, Paragon Government Solutions, and I'm a cash buyer interested in 11604 Tuscora Ave, Cleveland, OH 44108. Would the owner entertain a cash as-is offer, fast cash close, short feasibility window? What email should I send the written offer to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -7172,7 +7172,7 @@
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>Hi there Coby — Charles Pleasant, Paragon Government Solutions. I'm reaching out about 5906 Bower Ave, Cleveland, OH 44127. any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. What's the best email to send it to? Thanks!</t>
+          <t>Hi there Coby — Charles Pleasant, Paragon Government Solutions. I'm reaching out about 5906 Bower Ave, Cleveland, OH 44127. Any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. What's the best email to send it to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -7247,7 +7247,7 @@
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>Colleen, hi — I'm Charles with Paragon Government Solutions. I'm a cash buyer interested in 3945 Liberty Ave, Pittsburgh, PA 15224. any chance the seller would take a cash, as-is offer with fast close with a brief inspection window. What's the best email to send it to? Much appreciated!</t>
+          <t>Colleen, hi — I'm Charles with Paragon Government Solutions. I'm a cash buyer interested in 3945 Liberty Ave, Pittsburgh, PA 15224. Any chance the seller would take a cash, as-is offer with fast close with a brief inspection window. What's the best email to send it to? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -7272,7 +7272,7 @@
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>Hello Comeiko. Charles Pleasant, Paragon Government Solutions, and I'm a cash investor looking at 4971 Brigadoon Ln, Dallas, TX 75216. could the seller look at a cash, as-is offer, fast close with a brief inspection window? What's the best email to send it to? Thank you!</t>
+          <t>Hello Comeiko. Charles Pleasant, Paragon Government Solutions, and I'm a cash investor looking at 4971 Brigadoon Ln, Dallas, TX 75216. Could the seller look at a cash, as-is offer, fast close with a brief inspection window? What's the best email to send it to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -7347,7 +7347,7 @@
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>Hey Conor — this is Charles Pleasant with Paragon Government Solutions. I'm interested in buying 937 Avenue S, Birmingham, AL 35214 for cash. is the seller open to a cash as-is offer with a quick clean close and short due diligence. What email should I send the written offer to? Thank you!</t>
+          <t>Hey Conor — this is Charles Pleasant with Paragon Government Solutions. I'm interested in buying 937 Avenue S, Birmingham, AL 35214 for cash. Is the seller open to a cash as-is offer with a quick clean close and short due diligence. What email should I send the written offer to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -7422,7 +7422,7 @@
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>Hi Cory — I'm Charles with Paragon Government Solutions. I'm reaching out about 5747 Easthampton Dr Unit D, Houston, TX 77039. would the owner entertain a cash as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Thanks much!</t>
+          <t>Hi Cory — I'm Charles with Paragon Government Solutions. I'm reaching out about 5747 Easthampton Dr Unit D, Houston, TX 77039. Would the owner entertain a cash as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -7447,7 +7447,7 @@
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>Hello Crystal — Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 4010 Copeland St, Dallas, TX 75210. open to a discounted cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Thanks much!</t>
+          <t>Hello Crystal — Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 4010 Copeland St, Dallas, TX 75210. Open to a discounted cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -7522,7 +7522,7 @@
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>Good day D.R. — my name's Charles Pleasant, Paragon Government Solutions. I'm interested in buying Ledoux Plan, Trivento, Baker, LA 70714 for cash. any chance the seller would take a cash, as-is offer with a quick clean close and short due diligence. Where should I send the offer in writing? Thanks!</t>
+          <t>Good day D.R. — my name's Charles Pleasant, Paragon Government Solutions. I'm interested in buying Ledoux Plan, Trivento, Baker, LA 70714 for cash. Any chance the seller would take a cash, as-is offer with a quick clean close and short due diligence. Where should I send the offer in writing? Thanks!</t>
         </is>
       </c>
     </row>
@@ -7547,7 +7547,7 @@
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>Hi D.R. — I'm Charles with Paragon Government Solutions. I came across Ledoux Plan, Zachary Trails at Meadow View, Zachary, LA 70791 and buy cash. any chance the seller would take a cash, as-is offer with close quickly, short inspection period. What's a good email for the written offer? Appreciate it!</t>
+          <t>Hi D.R. — I'm Charles with Paragon Government Solutions. I came across Ledoux Plan, Zachary Trails at Meadow View, Zachary, LA 70791 and buy cash. Any chance the seller would take a cash, as-is offer with close quickly, short inspection period. What's a good email for the written offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -7572,7 +7572,7 @@
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t>Good day Daisy. this is Charles Pleasant with Paragon Government Solutions, and I'm a cash buyer interested in 4534 S Honore St, Chicago, IL 60609. would the owner entertain a cash as-is offer, close quickly, short inspection period? Where should I send the offer in writing? Thanks so much!</t>
+          <t>Good day Daisy. This is Charles Pleasant with Paragon Government Solutions, and I'm a cash buyer interested in 4534 S Honore St, Chicago, IL 60609. Would the owner entertain a cash as-is offer, close quickly, short inspection period? Where should I send the offer in writing? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -7597,7 +7597,7 @@
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>Hi there Dan. I'm Charles with Paragon Government Solutions, and I came across 1401 Kirby St NE, Albuquerque, NM 87112 and buy cash. could the seller look at a cash, as-is offer, quick close and a short inspection? Best email for the formal offer? Much appreciated!</t>
+          <t>Hi there Dan. I'm Charles with Paragon Government Solutions, and I came across 1401 Kirby St NE, Albuquerque, NM 87112 and buy cash. Could the seller look at a cash, as-is offer, quick close and a short inspection? Best email for the formal offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -7647,7 +7647,7 @@
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>Hi Dana — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 11831 Bee Ln, Houston, TX 77067. would the owner entertain a cash as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Thank you!</t>
+          <t>Hi Dana — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 11831 Bee Ln, Houston, TX 77067. Would the owner entertain a cash as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -7697,7 +7697,7 @@
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>Good day DANIEL. my name's Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 22 MONTE Street, Jacksonville, FL 32254 for cash. is the seller open to a cash as-is offer, close quickly, short inspection period? Where can I email the written terms? Thanks much!</t>
+          <t>Good day DANIEL. My name's Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 22 MONTE Street, Jacksonville, FL 32254 for cash. Is the seller open to a cash as-is offer, close quickly, short inspection period? Where can I email the written terms? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -7722,7 +7722,7 @@
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>Hello Daniel — this is Charles Pleasant with Paragon Government Solutions. I'm reaching out about 20489 Andover St, Highland Park, MI 48203. would the seller consider a cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Thank you!</t>
+          <t>Hello Daniel — this is Charles Pleasant with Paragon Government Solutions. I'm reaching out about 20489 Andover St, Highland Park, MI 48203. Would the seller consider a cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Thank you!</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>Hi Danielle — Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 18281 Lancashire St, Detroit, MI 48223. would the owner entertain a cash as-is offer with close quickly, short inspection period. What's a good email for the written offer? Appreciate it!</t>
+          <t>Hi Danielle — Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 18281 Lancashire St, Detroit, MI 48223. Would the owner entertain a cash as-is offer with close quickly, short inspection period. What's a good email for the written offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -7822,7 +7822,7 @@
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>Hi Darius. Charles here with Paragon Government Solutions, and I'm reaching out about 1825 N 17th St, Baton Rouge, LA 70802. is the seller open to a cash as-is offer, close quickly, short inspection period? What's a good email for the written offer? Thanks so much!</t>
+          <t>Hi Darius. Charles here with Paragon Government Solutions, and I'm reaching out about 1825 N 17th St, Baton Rouge, LA 70802. Is the seller open to a cash as-is offer, close quickly, short inspection period? What's a good email for the written offer? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -7847,7 +7847,7 @@
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>Hi Darrin — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 3507 E SANDRA Terrace, Phoenix, AZ 85032. could the seller look at a cash, as-is offer with fast close with a brief inspection window. Where should I send the offer in writing? Appreciate it!</t>
+          <t>Hi Darrin — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 3507 E SANDRA Terrace, Phoenix, AZ 85032. Could the seller look at a cash, as-is offer with fast close with a brief inspection window. Where should I send the offer in writing? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -7997,7 +7997,7 @@
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>Hi there David — Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 116 Larchwood Dr, Columbia, SC 29203. would the seller consider a cash, as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Much appreciated!</t>
+          <t>Hi there David — Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 116 Larchwood Dr, Columbia, SC 29203. Would the seller consider a cash, as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -8047,7 +8047,7 @@
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>Good day David — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 712 Thaxton Ave SE, Albuquerque, NM 87102. would the owner entertain a cash as-is offer with close quickly, short inspection period. Best email for the formal offer? Appreciate it!</t>
+          <t>Good day David — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 712 Thaxton Ave SE, Albuquerque, NM 87102. Would the owner entertain a cash as-is offer with close quickly, short inspection period. Best email for the formal offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -8072,7 +8072,7 @@
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>David, hi — Charles here with Paragon Government Solutions. I'm a cash buyer interested in 6 Crescent Ln, Columbia, SC 29212. any chance the seller would take a cash, as-is offer with quick close and a short inspection. What's the best email to send it to? Thanks!</t>
+          <t>David, hi — Charles here with Paragon Government Solutions. I'm a cash buyer interested in 6 Crescent Ln, Columbia, SC 29212. Any chance the seller would take a cash, as-is offer with quick close and a short inspection. What's the best email to send it to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -8097,7 +8097,7 @@
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>Hi David. my name's Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 139 Spruce St, Bakersfield, CA 93304 for cash. would the owner entertain a cash as-is offer, fast close with a brief inspection window? What's a good email for the written offer? Thanks much!</t>
+          <t>Hi David. My name's Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 139 Spruce St, Bakersfield, CA 93304 for cash. Would the owner entertain a cash as-is offer, fast close with a brief inspection window? What's a good email for the written offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -8122,7 +8122,7 @@
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>Hey David. I'm Charles with Paragon Government Solutions, and I'd like to put in a cash offer on 2631 Mike St, Dallas, TX 75212. could the seller look at a cash, as-is offer, a quick clean close and short due diligence? Where should I send the offer in writing? Thanks so much!</t>
+          <t>Hey David. I'm Charles with Paragon Government Solutions, and I'd like to put in a cash offer on 2631 Mike St, Dallas, TX 75212. Could the seller look at a cash, as-is offer, a quick clean close and short due diligence? Where should I send the offer in writing? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -8147,7 +8147,7 @@
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>Hi David. Charles here with Paragon Government Solutions, and I'm reaching out about 19182 Hickory St, Detroit, MI 48205. could the seller look at a cash, as-is offer, fast close with a brief inspection window? What's a good email for the written offer? Thank you!</t>
+          <t>Hi David. Charles here with Paragon Government Solutions, and I'm reaching out about 19182 Hickory St, Detroit, MI 48205. Could the seller look at a cash, as-is offer, fast close with a brief inspection window? What's a good email for the written offer? Thank you!</t>
         </is>
       </c>
     </row>
@@ -8172,7 +8172,7 @@
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>DAVID, hi. this is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 311 Glen Canyon Dr, Fayetteville, NC 28303. would the owner entertain a cash as-is offer, close quickly, short inspection period? Where can I email the written terms? Thank you!</t>
+          <t>DAVID, hi. This is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 311 Glen Canyon Dr, Fayetteville, NC 28303. Would the owner entertain a cash as-is offer, close quickly, short inspection period? Where can I email the written terms? Thank you!</t>
         </is>
       </c>
     </row>
@@ -8247,7 +8247,7 @@
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>Hi there Dean — my name's Charles Pleasant, Paragon Government Solutions. I came across 3497 W 46th St, Cleveland, OH 44102 and buy cash. would the owner entertain a cash as-is offer with close quickly, short inspection period. Best email for the formal offer? Thanks!</t>
+          <t>Hi there Dean — my name's Charles Pleasant, Paragon Government Solutions. I came across 3497 W 46th St, Cleveland, OH 44102 and buy cash. Would the owner entertain a cash as-is offer with close quickly, short inspection period. Best email for the formal offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -8322,7 +8322,7 @@
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>Hello Deborah — Charles here with Paragon Government Solutions. I'm interested in buying 10147 S State St, Chicago, IL 60628 for cash. could the seller look at a cash, as-is offer with a quick clean close and short due diligence. Where should I send the offer in writing? Thank you!</t>
+          <t>Hello Deborah — Charles here with Paragon Government Solutions. I'm interested in buying 10147 S State St, Chicago, IL 60628 for cash. Could the seller look at a cash, as-is offer with a quick clean close and short due diligence. Where should I send the offer in writing? Thank you!</t>
         </is>
       </c>
     </row>
@@ -8347,7 +8347,7 @@
       </c>
       <c r="F317" t="inlineStr">
         <is>
-          <t>Good day DEIRDRA. Charles here with Paragon Government Solutions, and I'm interested in buying 6818 MERRILL Court, Jacksonville, FL 32211 for cash. open to a discounted cash, as-is offer, fast cash close, short feasibility window? What's a good email for the written offer? Much appreciated!</t>
+          <t>Good day DEIRDRA. Charles here with Paragon Government Solutions, and I'm interested in buying 6818 MERRILL Court, Jacksonville, FL 32211 for cash. Open to a discounted cash, as-is offer, fast cash close, short feasibility window? What's a good email for the written offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -8372,7 +8372,7 @@
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t>Hi Demetria — Charles here with Paragon Government Solutions. I'd like to put in a cash offer on 6511 Brook Ave, Baltimore, MD 21206. is the seller open to a cash as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Thanks much!</t>
+          <t>Hi Demetria — Charles here with Paragon Government Solutions. I'd like to put in a cash offer on 6511 Brook Ave, Baltimore, MD 21206. Is the seller open to a cash as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -8397,7 +8397,7 @@
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>Hello Dena — I'm Charles with Paragon Government Solutions. I came across 301 Squire Rd, Columbia, SC 29223 and buy cash. would the owner entertain a cash as-is offer with fast close with a brief inspection window. Where should I send the offer in writing? Much appreciated!</t>
+          <t>Hello Dena — I'm Charles with Paragon Government Solutions. I came across 301 Squire Rd, Columbia, SC 29223 and buy cash. Would the owner entertain a cash as-is offer with fast close with a brief inspection window. Where should I send the offer in writing? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -8472,7 +8472,7 @@
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>Hi there Deven — Charles Pleasant, Paragon Government Solutions. I'm interested in buying 7700 S Lowe Ave, Chicago, IL 60620 for cash. could the seller look at a cash, as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Much appreciated!</t>
+          <t>Hi there Deven — Charles Pleasant, Paragon Government Solutions. I'm interested in buying 7700 S Lowe Ave, Chicago, IL 60620 for cash. Could the seller look at a cash, as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -8522,7 +8522,7 @@
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>Hello Dexter — this is Charles Pleasant with Paragon Government Solutions. I'm interested in buying 639 E 90th Pl, Chicago, IL 60619 for cash. is the seller open to a cash as-is offer with close quickly, short inspection period. Best email for the formal offer? Thank you!</t>
+          <t>Hello Dexter — this is Charles Pleasant with Paragon Government Solutions. I'm interested in buying 639 E 90th Pl, Chicago, IL 60619 for cash. Is the seller open to a cash as-is offer with close quickly, short inspection period. Best email for the formal offer? Thank you!</t>
         </is>
       </c>
     </row>
@@ -8547,7 +8547,7 @@
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>Diana, hi. my name's Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 18968 E Northlawn St E, Detroit, MI 48221. is the seller open to a cash as-is offer, quick close and a short inspection? What's the best email to send it to? Much appreciated!</t>
+          <t>Diana, hi. My name's Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 18968 E Northlawn St E, Detroit, MI 48221. Is the seller open to a cash as-is offer, quick close and a short inspection? What's the best email to send it to? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -8572,7 +8572,7 @@
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>Diane, hi — I'm Charles with Paragon Government Solutions. I'm a cash buyer interested in 2024 Elmridge Rd, Columbia, SC 29209. would the seller consider a cash, as-is offer with close quickly, short inspection period. What email should I send the written offer to? Thanks much!</t>
+          <t>Diane, hi — I'm Charles with Paragon Government Solutions. I'm a cash buyer interested in 2024 Elmridge Rd, Columbia, SC 29209. Would the seller consider a cash, as-is offer with close quickly, short inspection period. What email should I send the written offer to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -8597,7 +8597,7 @@
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>Hi there DMITRIY. Charles here with Paragon Government Solutions, and I'm interested in buying 5527 MAXINE Drive, Jacksonville, FL 32277 for cash. is the seller open to a cash as-is offer, fast cash close, short feasibility window? What's a good email for the written offer? Thank you!</t>
+          <t>Hi there DMITRIY. Charles here with Paragon Government Solutions, and I'm interested in buying 5527 MAXINE Drive, Jacksonville, FL 32277 for cash. Is the seller open to a cash as-is offer, fast cash close, short feasibility window? What's a good email for the written offer? Thank you!</t>
         </is>
       </c>
     </row>
@@ -8647,7 +8647,7 @@
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>Good day Donna. Charles here with Paragon Government Solutions, and I'm a cash investor looking at 8529 S May St, Chicago, IL 60620. would the seller consider a cash, as-is offer, quick close and a short inspection? Best email for the formal offer? Much appreciated!</t>
+          <t>Good day Donna. Charles here with Paragon Government Solutions, and I'm a cash investor looking at 8529 S May St, Chicago, IL 60620. Would the seller consider a cash, as-is offer, quick close and a short inspection? Best email for the formal offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -8722,7 +8722,7 @@
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>Hello Douglas. this is Charles Pleasant with Paragon Government Solutions, and I'm a cash investor looking at 7111 Bart Hollow, San Antonio, TX 78250. is the seller open to a cash as-is offer, quick close and a short inspection? Where should I send the offer in writing? Thank you!</t>
+          <t>Hello Douglas. This is Charles Pleasant with Paragon Government Solutions, and I'm a cash investor looking at 7111 Bart Hollow, San Antonio, TX 78250. Is the seller open to a cash as-is offer, quick close and a short inspection? Where should I send the offer in writing? Thank you!</t>
         </is>
       </c>
     </row>
@@ -8747,7 +8747,7 @@
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>Hi Doxie — Charles here with Paragon Government Solutions. I'd like to put in a cash offer on 987 E 129th St, Cleveland, OH 44108. would the owner entertain a cash as-is offer with fast cash close, short feasibility window. Where should I send the offer in writing? Appreciate it!</t>
+          <t>Hi Doxie — Charles here with Paragon Government Solutions. I'd like to put in a cash offer on 987 E 129th St, Cleveland, OH 44108. Would the owner entertain a cash as-is offer with fast cash close, short feasibility window. Where should I send the offer in writing? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -8797,7 +8797,7 @@
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>Good day Drew. Charles Pleasant, Paragon Government Solutions, and I came across 4137 W 157th St, Cleveland, OH 44135 and buy cash. any chance the seller would take a cash, as-is offer, a quick clean close and short due diligence? Best email for the formal offer? Thanks much!</t>
+          <t>Good day Drew. Charles Pleasant, Paragon Government Solutions, and I came across 4137 W 157th St, Cleveland, OH 44135 and buy cash. Any chance the seller would take a cash, as-is offer, a quick clean close and short due diligence? Best email for the formal offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -8872,7 +8872,7 @@
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t>Hello DWAYNE — Charles here with Paragon Government Solutions. I came across 5919 SONORA Drive W, Jacksonville, FL 32244 and buy cash. is the seller open to a cash as-is offer with fast close with a brief inspection window. Where should I send the offer in writing? Thanks much!</t>
+          <t>Hello DWAYNE — Charles here with Paragon Government Solutions. I came across 5919 SONORA Drive W, Jacksonville, FL 32244 and buy cash. Is the seller open to a cash as-is offer with fast close with a brief inspection window. Where should I send the offer in writing? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -8922,7 +8922,7 @@
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t>Edgardo, hi — I'm Charles with Paragon Government Solutions. I'd like to put in a cash offer on 7949 S Manistee Ave, Chicago, IL 60617. open to a discounted cash, as-is offer with quick close and a short inspection. Where should I send the offer in writing? Thanks!</t>
+          <t>Edgardo, hi — I'm Charles with Paragon Government Solutions. I'd like to put in a cash offer on 7949 S Manistee Ave, Chicago, IL 60617. Open to a discounted cash, as-is offer with quick close and a short inspection. Where should I send the offer in writing? Thanks!</t>
         </is>
       </c>
     </row>
@@ -8997,7 +8997,7 @@
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t>Edward, hi — Charles here with Paragon Government Solutions. I'm a cash investor looking at 217 S Shields Rd, Columbia, SC 29223. open to a discounted cash, as-is offer with fast close with a brief inspection window. Where should I send the offer in writing? Thanks so much!</t>
+          <t>Edward, hi — Charles here with Paragon Government Solutions. I'm a cash investor looking at 217 S Shields Rd, Columbia, SC 29223. Open to a discounted cash, as-is offer with fast close with a brief inspection window. Where should I send the offer in writing? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -9022,7 +9022,7 @@
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t>Edward, hi — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 6633 Sandstone St, Houston, TX 77074. would the owner entertain a cash as-is offer with a quick clean close and short due diligence. What email should I send the written offer to? Thanks much!</t>
+          <t>Edward, hi — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 6633 Sandstone St, Houston, TX 77074. Would the owner entertain a cash as-is offer with a quick clean close and short due diligence. What email should I send the written offer to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -9047,7 +9047,7 @@
       </c>
       <c r="F345" t="inlineStr">
         <is>
-          <t>Good day Edward — Charles here with Paragon Government Solutions. I'm reaching out about 13 Winding Way, Trenton, NJ 08620. would the seller consider a cash, as-is offer with close quickly, short inspection period. What's a good email for the written offer? Thanks!</t>
+          <t>Good day Edward — Charles here with Paragon Government Solutions. I'm reaching out about 13 Winding Way, Trenton, NJ 08620. Would the seller consider a cash, as-is offer with close quickly, short inspection period. What's a good email for the written offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -9072,7 +9072,7 @@
       </c>
       <c r="F346" t="inlineStr">
         <is>
-          <t>Hi Edwin — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 19338 Teppert St, Detroit, MI 48234. open to a discounted cash, as-is offer with fast close with a brief inspection window. What's the best email to send it to? Thanks!</t>
+          <t>Hi Edwin — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 19338 Teppert St, Detroit, MI 48234. Open to a discounted cash, as-is offer with fast close with a brief inspection window. What's the best email to send it to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -9097,7 +9097,7 @@
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>Good day Eileen — Charles Pleasant, Paragon Government Solutions. I'm reaching out about 10121 Jasper Ave, Cleveland, OH 44111. open to a discounted cash, as-is offer with a quick clean close and short due diligence. Where should I send the offer in writing? Much appreciated!</t>
+          <t>Good day Eileen — Charles Pleasant, Paragon Government Solutions. I'm reaching out about 10121 Jasper Ave, Cleveland, OH 44111. Open to a discounted cash, as-is offer with a quick clean close and short due diligence. Where should I send the offer in writing? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -9322,7 +9322,7 @@
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t>Hi there Erick. Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 18710 McCormick St, Detroit, MI 48224. open to a discounted cash, as-is offer, a quick clean close and short due diligence? Where should I send the offer in writing? Thanks much!</t>
+          <t>Hi there Erick. Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 18710 McCormick St, Detroit, MI 48224. Open to a discounted cash, as-is offer, a quick clean close and short due diligence? Where should I send the offer in writing? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -9347,7 +9347,7 @@
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t>Hi there Esmeralda. Charles here with Paragon Government Solutions, and I'm a cash investor looking at 105 Dresden St, Houston, TX 77012. is the seller open to a cash as-is offer, fast cash close, short feasibility window? What's the best email to send it to? Much appreciated!</t>
+          <t>Hi there Esmeralda. Charles here with Paragon Government Solutions, and I'm a cash investor looking at 105 Dresden St, Houston, TX 77012. Is the seller open to a cash as-is offer, fast cash close, short feasibility window? What's the best email to send it to? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -9372,7 +9372,7 @@
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t>Hi Eve — this is Charles Pleasant with Paragon Government Solutions. I came across 11224 S Stewart Ave, Chicago, IL 60628 and buy cash. is the seller open to a cash as-is offer with a quick clean close and short due diligence. Best email for the formal offer? Much appreciated!</t>
+          <t>Hi Eve — this is Charles Pleasant with Paragon Government Solutions. I came across 11224 S Stewart Ave, Chicago, IL 60628 and buy cash. Is the seller open to a cash as-is offer with a quick clean close and short due diligence. Best email for the formal offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -9422,7 +9422,7 @@
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t>Fadie, hi. Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 6324 Annland St, Detroit, MI 48204. any chance the seller would take a cash, as-is offer, fast cash close, short feasibility window? Best email for the formal offer? Thank you!</t>
+          <t>Fadie, hi. Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 6324 Annland St, Detroit, MI 48204. Any chance the seller would take a cash, as-is offer, fast cash close, short feasibility window? Best email for the formal offer? Thank you!</t>
         </is>
       </c>
     </row>
@@ -9472,7 +9472,7 @@
       </c>
       <c r="F362" t="inlineStr">
         <is>
-          <t>Hello Felicia. Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 6953 S Elizabeth St, Chicago, IL 60636 for cash. is the seller open to a cash as-is offer, close quickly, short inspection period? What's the best email to send it to? Thank you!</t>
+          <t>Hello Felicia. Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 6953 S Elizabeth St, Chicago, IL 60636 for cash. Is the seller open to a cash as-is offer, close quickly, short inspection period? What's the best email to send it to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -9522,7 +9522,7 @@
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t>Good day Francisco — I'm Charles with Paragon Government Solutions. I'd like to put in a cash offer on 921 S 3RD Avenue, Phoenix, AZ 85003. open to a discounted cash, as-is offer with fast cash close, short feasibility window. What's the best email to send it to? Thank you!</t>
+          <t>Good day Francisco — I'm Charles with Paragon Government Solutions. I'd like to put in a cash offer on 921 S 3RD Avenue, Phoenix, AZ 85003. Open to a discounted cash, as-is offer with fast cash close, short feasibility window. What's the best email to send it to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -9547,7 +9547,7 @@
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>Francisco, hi. I'm Charles with Paragon Government Solutions, and I'm interested in buying 11432 S Wentworth Ave, Chicago, IL 60628 for cash. any chance the seller would take a cash, as-is offer, quick close and a short inspection? What's the best email to send it to? Thanks!</t>
+          <t>Francisco, hi. I'm Charles with Paragon Government Solutions, and I'm interested in buying 11432 S Wentworth Ave, Chicago, IL 60628 for cash. Any chance the seller would take a cash, as-is offer, quick close and a short inspection? What's the best email to send it to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -9647,7 +9647,7 @@
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t>Frank, hi. this is Charles Pleasant with Paragon Government Solutions, and I'd like to put in a cash offer on 7800 S Kimbark Ave, Chicago, IL 60619. open to a discounted cash, as-is offer, close quickly, short inspection period? Best email for the formal offer? Thanks much!</t>
+          <t>Frank, hi. This is Charles Pleasant with Paragon Government Solutions, and I'd like to put in a cash offer on 7800 S Kimbark Ave, Chicago, IL 60619. Open to a discounted cash, as-is offer, close quickly, short inspection period? Best email for the formal offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -9722,7 +9722,7 @@
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t>Hi Gabe — I'm Charles with Paragon Government Solutions. I came across 9601 Silk Ave, Cleveland, OH 44102 and buy cash. open to a discounted cash, as-is offer with quick close and a short inspection. What's the best email to send it to? Thanks!</t>
+          <t>Hi Gabe — I'm Charles with Paragon Government Solutions. I came across 9601 Silk Ave, Cleveland, OH 44102 and buy cash. Open to a discounted cash, as-is offer with quick close and a short inspection. What's the best email to send it to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -9797,7 +9797,7 @@
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>Hey GARY. Charles Pleasant, Paragon Government Solutions, and I'm a cash buyer interested in 113 Starhill Ave, Fayetteville, NC 28303. open to a discounted cash, as-is offer, close quickly, short inspection period? What email should I send the written offer to? Thanks so much!</t>
+          <t>Hey GARY. Charles Pleasant, Paragon Government Solutions, and I'm a cash buyer interested in 113 Starhill Ave, Fayetteville, NC 28303. Open to a discounted cash, as-is offer, close quickly, short inspection period? What email should I send the written offer to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -9822,7 +9822,7 @@
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t>Hi Gaymon — this is Charles Pleasant with Paragon Government Solutions. I came across 113 Salusbury Ln, Columbia, SC 29229 and buy cash. would the seller consider a cash, as-is offer with fast cash close, short feasibility window. Where can I email the written terms? Appreciate it!</t>
+          <t>Hi Gaymon — this is Charles Pleasant with Paragon Government Solutions. I came across 113 Salusbury Ln, Columbia, SC 29229 and buy cash. Would the seller consider a cash, as-is offer with fast cash close, short feasibility window. Where can I email the written terms? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -9872,7 +9872,7 @@
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t>Hey Gene — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 192 Dunham Rd, Columbia, SC 29209. would the owner entertain a cash as-is offer with fast cash close, short feasibility window. What's the best email to send it to? Thanks!</t>
+          <t>Hey Gene — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 192 Dunham Rd, Columbia, SC 29209. Would the owner entertain a cash as-is offer with fast cash close, short feasibility window. What's the best email to send it to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -9947,7 +9947,7 @@
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t>Gerilet, hi — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 5147 BROKEN ARROW Drive N, Jacksonville, FL 32244. would the seller consider a cash, as-is offer with close quickly, short inspection period. What's a good email for the written offer? Appreciate it!</t>
+          <t>Gerilet, hi — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 5147 BROKEN ARROW Drive N, Jacksonville, FL 32244. Would the seller consider a cash, as-is offer with close quickly, short inspection period. What's a good email for the written offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -9972,7 +9972,7 @@
       </c>
       <c r="F382" t="inlineStr">
         <is>
-          <t>Hi Gershon. Charles Pleasant, Paragon Government Solutions, and I'm a cash buyer interested in 8005 S Campbell Ave, Chicago, IL 60652. is the seller open to a cash as-is offer, fast close with a brief inspection window? Best email for the formal offer? Appreciate it!</t>
+          <t>Hi Gershon. Charles Pleasant, Paragon Government Solutions, and I'm a cash buyer interested in 8005 S Campbell Ave, Chicago, IL 60652. Is the seller open to a cash as-is offer, fast close with a brief inspection window? Best email for the formal offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -9997,7 +9997,7 @@
       </c>
       <c r="F383" t="inlineStr">
         <is>
-          <t>Hi there Gina — Charles Pleasant, Paragon Government Solutions. I came across 2640 Ridgely St, Baltimore, MD 21230 and buy cash. open to a discounted cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Thanks so much!</t>
+          <t>Hi there Gina — Charles Pleasant, Paragon Government Solutions. I came across 2640 Ridgely St, Baltimore, MD 21230 and buy cash. Open to a discounted cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -10022,7 +10022,7 @@
       </c>
       <c r="F384" t="inlineStr">
         <is>
-          <t>Gino, hi. this is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 78 Liberty St, Trenton, NJ 08611. is the seller open to a cash as-is offer, a quick clean close and short due diligence? What's a good email for the written offer? Thank you!</t>
+          <t>Gino, hi. This is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 78 Liberty St, Trenton, NJ 08611. Is the seller open to a cash as-is offer, a quick clean close and short due diligence? What's a good email for the written offer? Thank you!</t>
         </is>
       </c>
     </row>
@@ -10072,7 +10072,7 @@
       </c>
       <c r="F386" t="inlineStr">
         <is>
-          <t>Hey Glen — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 3194 W 95th St, Cleveland, OH 44102. any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Thank you!</t>
+          <t>Hey Glen — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 3194 W 95th St, Cleveland, OH 44102. Any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Thank you!</t>
         </is>
       </c>
     </row>
@@ -10097,7 +10097,7 @@
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t>Hi GLEN. I'm Charles with Paragon Government Solutions, and I'd like to put in a cash offer on 8456 BOYSENBERRY Lane W, Jacksonville, FL 32244. would the seller consider a cash, as-is offer, fast cash close, short feasibility window? What's the best email to send it to? Thanks much!</t>
+          <t>Hi GLEN. I'm Charles with Paragon Government Solutions, and I'd like to put in a cash offer on 8456 BOYSENBERRY Lane W, Jacksonville, FL 32244. Would the seller consider a cash, as-is offer, fast cash close, short feasibility window? What's the best email to send it to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -10122,7 +10122,7 @@
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t>Hi there Gonzalo. I'm Charles with Paragon Government Solutions, and I came across 725 W SOUTHGATE Avenue W, Phoenix, AZ 85041 and buy cash. is the seller open to a cash as-is offer, fast close with a brief inspection window? Where can I email the written terms? Thank you!</t>
+          <t>Hi there Gonzalo. I'm Charles with Paragon Government Solutions, and I came across 725 W SOUTHGATE Avenue W, Phoenix, AZ 85041 and buy cash. Is the seller open to a cash as-is offer, fast close with a brief inspection window? Where can I email the written terms? Thank you!</t>
         </is>
       </c>
     </row>
@@ -10172,7 +10172,7 @@
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t>Gracie, hi. this is Charles Pleasant with Paragon Government Solutions, and I'm a cash investor looking at 4015 Shadrack Dr, Dallas, TX 75212. would the seller consider a cash, as-is offer, quick close and a short inspection? Best email for the formal offer? Thank you!</t>
+          <t>Gracie, hi. This is Charles Pleasant with Paragon Government Solutions, and I'm a cash investor looking at 4015 Shadrack Dr, Dallas, TX 75212. Would the seller consider a cash, as-is offer, quick close and a short inspection? Best email for the formal offer? Thank you!</t>
         </is>
       </c>
     </row>
@@ -10197,7 +10197,7 @@
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>Hi Grant — Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 1709 Jeffrey Bryan Dr, Charlotte, NC 28213. could the seller look at a cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Appreciate it!</t>
+          <t>Hi Grant — Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 1709 Jeffrey Bryan Dr, Charlotte, NC 28213. Could the seller look at a cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -10222,7 +10222,7 @@
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t>Hi Grazyna — Charles Pleasant, Paragon Government Solutions. I came across 3709 W 66th Pl, Chicago, IL 60629 and buy cash. is the seller open to a cash as-is offer with quick close and a short inspection. What's the best email to send it to? Thanks so much!</t>
+          <t>Hi Grazyna — Charles Pleasant, Paragon Government Solutions. I came across 3709 W 66th Pl, Chicago, IL 60629 and buy cash. Is the seller open to a cash as-is offer with quick close and a short inspection. What's the best email to send it to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -10272,7 +10272,7 @@
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t>Hi there Gregory. my name's Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 10535 S Peoria St, Chicago, IL 60643. is the seller open to a cash as-is offer, close quickly, short inspection period? Where should I send the offer in writing? Appreciate it!</t>
+          <t>Hi there Gregory. My name's Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 10535 S Peoria St, Chicago, IL 60643. Is the seller open to a cash as-is offer, close quickly, short inspection period? Where should I send the offer in writing? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -10297,7 +10297,7 @@
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t>Hey Gregory — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 19358 Teppert St, Detroit, MI 48234. open to a discounted cash, as-is offer with fast cash close, short feasibility window. Where can I email the written terms? Much appreciated!</t>
+          <t>Hey Gregory — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 19358 Teppert St, Detroit, MI 48234. Open to a discounted cash, as-is offer with fast cash close, short feasibility window. Where can I email the written terms? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -10397,7 +10397,7 @@
       </c>
       <c r="F399" t="inlineStr">
         <is>
-          <t>Hey Hannah — Charles here with Paragon Government Solutions. I'm a cash investor looking at 232 Fernview Dr, Columbia, SC 29229. any chance the seller would take a cash, as-is offer with fast close with a brief inspection window. Where can I email the written terms? Thanks much!</t>
+          <t>Hey Hannah — Charles here with Paragon Government Solutions. I'm a cash investor looking at 232 Fernview Dr, Columbia, SC 29229. Any chance the seller would take a cash, as-is offer with fast close with a brief inspection window. Where can I email the written terms? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -10547,7 +10547,7 @@
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t>Hey Heather. Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 5235 Cumberland Cove Dr, Baton Rouge, LA 70817 for cash. any chance the seller would take a cash, as-is offer, close quickly, short inspection period? What's a good email for the written offer? Much appreciated!</t>
+          <t>Hey Heather. Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 5235 Cumberland Cove Dr, Baton Rouge, LA 70817 for cash. Any chance the seller would take a cash, as-is offer, close quickly, short inspection period? What's a good email for the written offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -10597,7 +10597,7 @@
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t>Heather, hi. I'm Charles with Paragon Government Solutions, and I came across 1802 E Campo Bello Drive #92, Phoenix, AZ 85022 and buy cash. would the seller consider a cash, as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Thanks much!</t>
+          <t>Heather, hi. I'm Charles with Paragon Government Solutions, and I came across 1802 E Campo Bello Drive #92, Phoenix, AZ 85022 and buy cash. Would the seller consider a cash, as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -10647,7 +10647,7 @@
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t>HENRY, hi. this is Charles Pleasant with Paragon Government Solutions, and I'm a cash investor looking at 27 W 44TH Street, Jacksonville, FL 32208. could the seller look at a cash, as-is offer, fast close with a brief inspection window? Best email for the formal offer? Thanks much!</t>
+          <t>HENRY, hi. This is Charles Pleasant with Paragon Government Solutions, and I'm a cash investor looking at 27 W 44TH Street, Jacksonville, FL 32208. Could the seller look at a cash, as-is offer, fast close with a brief inspection window? Best email for the formal offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -10672,7 +10672,7 @@
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t>Hi there Henry — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 6603 S Oakley Ave, Chicago, IL 60636. would the seller consider a cash, as-is offer with quick close and a short inspection. What's a good email for the written offer? Much appreciated!</t>
+          <t>Hi there Henry — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 6603 S Oakley Ave, Chicago, IL 60636. Would the seller consider a cash, as-is offer with quick close and a short inspection. What's a good email for the written offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -10722,7 +10722,7 @@
       </c>
       <c r="F412" t="inlineStr">
         <is>
-          <t>Hi Hilda. Charles here with Paragon Government Solutions, and I'm reaching out about 1401 El Sereno Dr, Bakersfield, CA 93304. could the seller look at a cash, as-is offer, quick close and a short inspection? Where can I email the written terms? Much appreciated!</t>
+          <t>Hi Hilda. Charles here with Paragon Government Solutions, and I'm reaching out about 1401 El Sereno Dr, Bakersfield, CA 93304. Could the seller look at a cash, as-is offer, quick close and a short inspection? Where can I email the written terms? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -10747,7 +10747,7 @@
       </c>
       <c r="F413" t="inlineStr">
         <is>
-          <t>Ian, hi. Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 19479 Spencer St, Detroit, MI 48234. open to a discounted cash, as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Thanks much!</t>
+          <t>Ian, hi. Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 19479 Spencer St, Detroit, MI 48234. Open to a discounted cash, as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -10772,7 +10772,7 @@
       </c>
       <c r="F414" t="inlineStr">
         <is>
-          <t>Ijella, hi. I'm Charles with Paragon Government Solutions, and I'd like to put in a cash offer on 9627 Scotswood Dr, Baton Rouge, LA 70818. open to a discounted cash, as-is offer, quick close and a short inspection? What's a good email for the written offer? Thanks!</t>
+          <t>Ijella, hi. I'm Charles with Paragon Government Solutions, and I'd like to put in a cash offer on 9627 Scotswood Dr, Baton Rouge, LA 70818. Open to a discounted cash, as-is offer, quick close and a short inspection? What's a good email for the written offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -10797,7 +10797,7 @@
       </c>
       <c r="F415" t="inlineStr">
         <is>
-          <t>Hey Ingrid — Charles Pleasant, Paragon Government Solutions. I came across 842 Meridian Ave, Lakeland, FL 33801 and buy cash. open to a discounted cash, as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Thanks so much!</t>
+          <t>Hey Ingrid — Charles Pleasant, Paragon Government Solutions. I came across 842 Meridian Ave, Lakeland, FL 33801 and buy cash. Open to a discounted cash, as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -10822,7 +10822,7 @@
       </c>
       <c r="F416" t="inlineStr">
         <is>
-          <t>Hi there IRAN — Charles here with Paragon Government Solutions. I'm interested in buying 2501 DOBY Street, Jacksonville, FL 32209 for cash. open to a discounted cash, as-is offer with a quick clean close and short due diligence. Where can I email the written terms? Thank you!</t>
+          <t>Hi there IRAN — Charles here with Paragon Government Solutions. I'm interested in buying 2501 DOBY Street, Jacksonville, FL 32209 for cash. Open to a discounted cash, as-is offer with a quick clean close and short due diligence. Where can I email the written terms? Thank you!</t>
         </is>
       </c>
     </row>
@@ -10847,7 +10847,7 @@
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t>Hello Iris — this is Charles Pleasant with Paragon Government Solutions. I came across 189 Mercer St, Hamilton, NJ 08690 and buy cash. would the owner entertain a cash as-is offer with close quickly, short inspection period. What email should I send the written offer to? Appreciate it!</t>
+          <t>Hello Iris — this is Charles Pleasant with Paragon Government Solutions. I came across 189 Mercer St, Hamilton, NJ 08690 and buy cash. Would the owner entertain a cash as-is offer with close quickly, short inspection period. What email should I send the written offer to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -10902,7 +10902,7 @@
       </c>
       <c r="F419" t="inlineStr">
         <is>
-          <t>Hey Jack. my name's Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 905 Ann Ave, Dallas, TX 75223 for cash. is the seller open to a cash as-is offer, quick close and a short inspection? Best email for the formal offer? Thank you!</t>
+          <t>Hey Jack. My name's Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 905 Ann Ave, Dallas, TX 75223 for cash. Is the seller open to a cash as-is offer, quick close and a short inspection? Best email for the formal offer? Thank you!</t>
         </is>
       </c>
     </row>
@@ -10927,7 +10927,7 @@
       </c>
       <c r="F420" t="inlineStr">
         <is>
-          <t>Jacob, hi — my name's Charles Pleasant, Paragon Government Solutions. I'm interested in buying 17360 Greenlawn St, Detroit, MI 48221 for cash. any chance the seller would take a cash, as-is offer with quick close and a short inspection. Where can I email the written terms? Thanks!</t>
+          <t>Jacob, hi — my name's Charles Pleasant, Paragon Government Solutions. I'm interested in buying 17360 Greenlawn St, Detroit, MI 48221 for cash. Any chance the seller would take a cash, as-is offer with quick close and a short inspection. Where can I email the written terms? Thanks!</t>
         </is>
       </c>
     </row>
@@ -11052,7 +11052,7 @@
       </c>
       <c r="F425" t="inlineStr">
         <is>
-          <t>Hello JAMES — Charles Pleasant, Paragon Government Solutions. I came across 2203 SHERRINGTON Street, Jacksonville, FL 32209 and buy cash. would the seller consider a cash, as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Thanks much!</t>
+          <t>Hello JAMES — Charles Pleasant, Paragon Government Solutions. I came across 2203 SHERRINGTON Street, Jacksonville, FL 32209 and buy cash. Would the seller consider a cash, as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -11077,7 +11077,7 @@
       </c>
       <c r="F426" t="inlineStr">
         <is>
-          <t>Hi James — Charles here with Paragon Government Solutions. I'd like to put in a cash offer on 9433 S Michigan Ave, Chicago, IL 60619. is the seller open to a cash as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Thanks much!</t>
+          <t>Hi James — Charles here with Paragon Government Solutions. I'd like to put in a cash offer on 9433 S Michigan Ave, Chicago, IL 60619. Is the seller open to a cash as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -11127,7 +11127,7 @@
       </c>
       <c r="F428" t="inlineStr">
         <is>
-          <t>Hi there James. Charles Pleasant, Paragon Government Solutions, and I'm a cash buyer interested in 9261 Camley St, Detroit, MI 48224. open to a discounted cash, as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Thanks!</t>
+          <t>Hi there James. Charles Pleasant, Paragon Government Solutions, and I'm a cash buyer interested in 9261 Camley St, Detroit, MI 48224. Open to a discounted cash, as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -11177,7 +11177,7 @@
       </c>
       <c r="F430" t="inlineStr">
         <is>
-          <t>Hello Jami — this is Charles Pleasant with Paragon Government Solutions. I came across 10339 Limestone Dr, Dallas, TX 75217 and buy cash. is the seller open to a cash as-is offer with quick close and a short inspection. What email should I send the written offer to? Thanks so much!</t>
+          <t>Hello Jami — this is Charles Pleasant with Paragon Government Solutions. I came across 10339 Limestone Dr, Dallas, TX 75217 and buy cash. Is the seller open to a cash as-is offer with quick close and a short inspection. What email should I send the written offer to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="F431" t="inlineStr">
         <is>
-          <t>Hey Jamie — Charles Pleasant, Paragon Government Solutions. I'm reaching out about 3010 Hartwick Rd, Houston, TX 77093. would the owner entertain a cash as-is offer with fast cash close, short feasibility window. Where can I email the written terms? Thanks much!</t>
+          <t>Hey Jamie — Charles Pleasant, Paragon Government Solutions. I'm reaching out about 3010 Hartwick Rd, Houston, TX 77093. Would the owner entertain a cash as-is offer with fast cash close, short feasibility window. Where can I email the written terms? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -11227,7 +11227,7 @@
       </c>
       <c r="F432" t="inlineStr">
         <is>
-          <t>Hi there Jamie — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 2229 W 60th St, Indianapolis, IN 46228. would the seller consider a cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Thanks so much!</t>
+          <t>Hi there Jamie — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 2229 W 60th St, Indianapolis, IN 46228. Would the seller consider a cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -11252,7 +11252,7 @@
       </c>
       <c r="F433" t="inlineStr">
         <is>
-          <t>Hi Jamila — my name's Charles Pleasant, Paragon Government Solutions. I'm reaching out about 12607 Oakfield Ave, Cleveland, OH 44105. would the seller consider a cash, as-is offer with quick close and a short inspection. Where should I send the offer in writing? Thanks!</t>
+          <t>Hi Jamila — my name's Charles Pleasant, Paragon Government Solutions. I'm reaching out about 12607 Oakfield Ave, Cleveland, OH 44105. Would the seller consider a cash, as-is offer with quick close and a short inspection. Where should I send the offer in writing? Thanks!</t>
         </is>
       </c>
     </row>
@@ -11277,7 +11277,7 @@
       </c>
       <c r="F434" t="inlineStr">
         <is>
-          <t>Good day Janina. this is Charles Pleasant with Paragon Government Solutions, and I'm a cash buyer interested in 7324 S Blackstone Ave, Chicago, IL 60619. would the seller consider a cash, as-is offer, close quickly, short inspection period? Best email for the formal offer? Appreciate it!</t>
+          <t>Good day Janina. This is Charles Pleasant with Paragon Government Solutions, and I'm a cash buyer interested in 7324 S Blackstone Ave, Chicago, IL 60619. Would the seller consider a cash, as-is offer, close quickly, short inspection period? Best email for the formal offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -11352,7 +11352,7 @@
       </c>
       <c r="F437" t="inlineStr">
         <is>
-          <t>Jason, hi. I'm Charles with Paragon Government Solutions, and I'm interested in buying 1009 Poplar Grove St, Baltimore, MD 21216 for cash. open to a discounted cash, as-is offer, close quickly, short inspection period? What email should I send the written offer to? Thanks!</t>
+          <t>Jason, hi. I'm Charles with Paragon Government Solutions, and I'm interested in buying 1009 Poplar Grove St, Baltimore, MD 21216 for cash. Open to a discounted cash, as-is offer, close quickly, short inspection period? What email should I send the written offer to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -11402,7 +11402,7 @@
       </c>
       <c r="F439" t="inlineStr">
         <is>
-          <t>Hi Jason. my name's Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 2600 Brookside Dr APT 41, Bakersfield, CA 93311. would the owner entertain a cash as-is offer, fast close with a brief inspection window? Best email for the formal offer? Appreciate it!</t>
+          <t>Hi Jason. My name's Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 2600 Brookside Dr APT 41, Bakersfield, CA 93311. Would the owner entertain a cash as-is offer, fast close with a brief inspection window? Best email for the formal offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -11427,7 +11427,7 @@
       </c>
       <c r="F440" t="inlineStr">
         <is>
-          <t>Hey Jason — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 106 N Briscoe Blvd, Dallas, TX 75211. open to a discounted cash, as-is offer with a quick clean close and short due diligence. What email should I send the written offer to? Much appreciated!</t>
+          <t>Hey Jason — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 106 N Briscoe Blvd, Dallas, TX 75211. Open to a discounted cash, as-is offer with a quick clean close and short due diligence. What email should I send the written offer to? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -11452,7 +11452,7 @@
       </c>
       <c r="F441" t="inlineStr">
         <is>
-          <t>Hello Jason. this is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 1921 W WHITTON Avenue, Phoenix, AZ 85015. would the owner entertain a cash as-is offer, quick close and a short inspection? What's the best email to send it to? Thanks much!</t>
+          <t>Hello Jason. This is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 1921 W WHITTON Avenue, Phoenix, AZ 85015. Would the owner entertain a cash as-is offer, quick close and a short inspection? What's the best email to send it to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -11502,7 +11502,7 @@
       </c>
       <c r="F443" t="inlineStr">
         <is>
-          <t>Jay, hi — I'm Charles with Paragon Government Solutions. I came across 4909 Falls St, Houston, TX 77026 and buy cash. could the seller look at a cash, as-is offer with fast cash close, short feasibility window. What email should I send the written offer to? Thanks so much!</t>
+          <t>Jay, hi — I'm Charles with Paragon Government Solutions. I came across 4909 Falls St, Houston, TX 77026 and buy cash. Could the seller look at a cash, as-is offer with fast cash close, short feasibility window. What email should I send the written offer to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -11527,7 +11527,7 @@
       </c>
       <c r="F444" t="inlineStr">
         <is>
-          <t>Hi JC — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 5009 W Chicago Ave, Chicago, IL 60651. open to a discounted cash, as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Thank you!</t>
+          <t>Hi JC — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 5009 W Chicago Ave, Chicago, IL 60651. Open to a discounted cash, as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Thank you!</t>
         </is>
       </c>
     </row>
@@ -11552,7 +11552,7 @@
       </c>
       <c r="F445" t="inlineStr">
         <is>
-          <t>JD, hi. Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 6810 Satchel Ford Rd, Columbia, SC 29206. open to a discounted cash, as-is offer, quick close and a short inspection? What email should I send the written offer to? Thanks much!</t>
+          <t>JD, hi. Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 6810 Satchel Ford Rd, Columbia, SC 29206. Open to a discounted cash, as-is offer, quick close and a short inspection? What email should I send the written offer to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -11602,7 +11602,7 @@
       </c>
       <c r="F447" t="inlineStr">
         <is>
-          <t>Hey Jeff — this is Charles Pleasant with Paragon Government Solutions. I'm interested in buying 3218 College St, Slidell, LA 70458 for cash. is the seller open to a cash as-is offer with close quickly, short inspection period. Where can I email the written terms? Thank you!</t>
+          <t>Hey Jeff — this is Charles Pleasant with Paragon Government Solutions. I'm interested in buying 3218 College St, Slidell, LA 70458 for cash. Is the seller open to a cash as-is offer with close quickly, short inspection period. Where can I email the written terms? Thank you!</t>
         </is>
       </c>
     </row>
@@ -11702,7 +11702,7 @@
       </c>
       <c r="F451" t="inlineStr">
         <is>
-          <t>Jeffrey, hi. my name's Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 8622 Othello St, Houston, TX 77029 for cash. would the owner entertain a cash as-is offer, close quickly, short inspection period? What email should I send the written offer to? Thank you!</t>
+          <t>Jeffrey, hi. My name's Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 8622 Othello St, Houston, TX 77029 for cash. Would the owner entertain a cash as-is offer, close quickly, short inspection period? What email should I send the written offer to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -11902,7 +11902,7 @@
       </c>
       <c r="F459" t="inlineStr">
         <is>
-          <t>Good day Jerry. this is Charles Pleasant with Paragon Government Solutions, and I'm a cash investor looking at 3012 Skyview Dr, Lakeland, FL 33801. open to a discounted cash, as-is offer, close quickly, short inspection period? What email should I send the written offer to? Appreciate it!</t>
+          <t>Good day Jerry. This is Charles Pleasant with Paragon Government Solutions, and I'm a cash investor looking at 3012 Skyview Dr, Lakeland, FL 33801. Open to a discounted cash, as-is offer, close quickly, short inspection period? What email should I send the written offer to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -11977,7 +11977,7 @@
       </c>
       <c r="F462" t="inlineStr">
         <is>
-          <t>Hello Jessica. I'm Charles with Paragon Government Solutions, and I'd like to put in a cash offer on 3929 Trotter Rd, Columbia, SC 29209. would the owner entertain a cash as-is offer, fast close with a brief inspection window? What's the best email to send it to? Much appreciated!</t>
+          <t>Hello Jessica. I'm Charles with Paragon Government Solutions, and I'd like to put in a cash offer on 3929 Trotter Rd, Columbia, SC 29209. Would the owner entertain a cash as-is offer, fast close with a brief inspection window? What's the best email to send it to? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -12002,7 +12002,7 @@
       </c>
       <c r="F463" t="inlineStr">
         <is>
-          <t>Hi Jessica — my name's Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 8752 Woodcastle Dr, Dallas, TX 75217. is the seller open to a cash as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Thanks so much!</t>
+          <t>Hi Jessica — my name's Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 8752 Woodcastle Dr, Dallas, TX 75217. Is the seller open to a cash as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -12027,7 +12027,7 @@
       </c>
       <c r="F464" t="inlineStr">
         <is>
-          <t>Good day Jessica. Charles here with Paragon Government Solutions, and I came across 1521 Hamilton Ave, Hamilton, NJ 08629 and buy cash. would the owner entertain a cash as-is offer, a quick clean close and short due diligence? What's a good email for the written offer? Thanks much!</t>
+          <t>Good day Jessica. Charles here with Paragon Government Solutions, and I came across 1521 Hamilton Ave, Hamilton, NJ 08629 and buy cash. Would the owner entertain a cash as-is offer, a quick clean close and short due diligence? What's a good email for the written offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -12052,7 +12052,7 @@
       </c>
       <c r="F465" t="inlineStr">
         <is>
-          <t>Hello Jessica — my name's Charles Pleasant, Paragon Government Solutions. I'm interested in buying 5250 Alter Rd, Detroit, MI 48224 for cash. would the seller consider a cash, as-is offer with quick close and a short inspection. What's a good email for the written offer? Appreciate it!</t>
+          <t>Hello Jessica — my name's Charles Pleasant, Paragon Government Solutions. I'm interested in buying 5250 Alter Rd, Detroit, MI 48224 for cash. Would the seller consider a cash, as-is offer with quick close and a short inspection. What's a good email for the written offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -12127,7 +12127,7 @@
       </c>
       <c r="F468" t="inlineStr">
         <is>
-          <t>Hello Jim — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 5303 S Winchester Ave, Chicago, IL 60609. would the owner entertain a cash as-is offer with quick close and a short inspection. Where can I email the written terms? Thank you!</t>
+          <t>Hello Jim — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 5303 S Winchester Ave, Chicago, IL 60609. Would the owner entertain a cash as-is offer with quick close and a short inspection. Where can I email the written terms? Thank you!</t>
         </is>
       </c>
     </row>
@@ -12202,7 +12202,7 @@
       </c>
       <c r="F471" t="inlineStr">
         <is>
-          <t>Hello JoAnn. I'm Charles with Paragon Government Solutions, and I came across 16503 Wisconsin St, Detroit, MI 48221 and buy cash. would the seller consider a cash, as-is offer, fast close with a brief inspection window? What's a good email for the written offer? Thanks!</t>
+          <t>Hello JoAnn. I'm Charles with Paragon Government Solutions, and I came across 16503 Wisconsin St, Detroit, MI 48221 and buy cash. Would the seller consider a cash, as-is offer, fast close with a brief inspection window? What's a good email for the written offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -12327,7 +12327,7 @@
       </c>
       <c r="F476" t="inlineStr">
         <is>
-          <t>Hi there John. my name's Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 15346 Dexter Ave, Detroit, MI 48238. could the seller look at a cash, as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Thank you!</t>
+          <t>Hi there John. My name's Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 15346 Dexter Ave, Detroit, MI 48238. Could the seller look at a cash, as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Thank you!</t>
         </is>
       </c>
     </row>
@@ -12377,7 +12377,7 @@
       </c>
       <c r="F478" t="inlineStr">
         <is>
-          <t>Hi there John — I'm Charles with Paragon Government Solutions. I came across 1002 Prouty Ave, Toledo, OH 43609 and buy cash. would the seller consider a cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Thanks so much!</t>
+          <t>Hi there John — I'm Charles with Paragon Government Solutions. I came across 1002 Prouty Ave, Toledo, OH 43609 and buy cash. Would the seller consider a cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -12477,7 +12477,7 @@
       </c>
       <c r="F482" t="inlineStr">
         <is>
-          <t>Hello John. Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on Leadmine Rd, Gaffney, SC 29340. would the seller consider a cash, as-is offer, quick close and a short inspection? What email should I send the written offer to? Thanks much!</t>
+          <t>Hello John. Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on Leadmine Rd, Gaffney, SC 29340. Would the seller consider a cash, as-is offer, quick close and a short inspection? What email should I send the written offer to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -12502,7 +12502,7 @@
       </c>
       <c r="F483" t="inlineStr">
         <is>
-          <t>Hello JOHN. Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 3554 BROCKWAY Road, Jacksonville, FL 32250 for cash. could the seller look at a cash, as-is offer, close quickly, short inspection period? What's the best email to send it to? Much appreciated!</t>
+          <t>Hello JOHN. Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 3554 BROCKWAY Road, Jacksonville, FL 32250 for cash. Could the seller look at a cash, as-is offer, close quickly, short inspection period? What's the best email to send it to? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -12527,7 +12527,7 @@
       </c>
       <c r="F484" t="inlineStr">
         <is>
-          <t>Hi there Johnny. this is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 9016 Harris Ave, Cleveland, OH 44104. could the seller look at a cash, as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Thanks so much!</t>
+          <t>Hi there Johnny. This is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 9016 Harris Ave, Cleveland, OH 44104. Could the seller look at a cash, as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -12627,7 +12627,7 @@
       </c>
       <c r="F488" t="inlineStr">
         <is>
-          <t>Good day Jose — Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 9137 Meyers Rd, Detroit, MI 48228. is the seller open to a cash as-is offer with quick close and a short inspection. Where can I email the written terms? Much appreciated!</t>
+          <t>Good day Jose — Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 9137 Meyers Rd, Detroit, MI 48228. Is the seller open to a cash as-is offer with quick close and a short inspection. Where can I email the written terms? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -12652,7 +12652,7 @@
       </c>
       <c r="F489" t="inlineStr">
         <is>
-          <t>Jose, hi — I'm Charles with Paragon Government Solutions. I'd like to put in a cash offer on 5921 S Sawyer Ave, Chicago, IL 60629. would the seller consider a cash, as-is offer with fast close with a brief inspection window. Where should I send the offer in writing? Much appreciated!</t>
+          <t>Jose, hi — I'm Charles with Paragon Government Solutions. I'd like to put in a cash offer on 5921 S Sawyer Ave, Chicago, IL 60629. Would the seller consider a cash, as-is offer with fast close with a brief inspection window. Where should I send the offer in writing? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -12677,7 +12677,7 @@
       </c>
       <c r="F490" t="inlineStr">
         <is>
-          <t>Jose, hi. I'm Charles with Paragon Government Solutions, and I'm reaching out about 9122 S La Salle St, Chicago, IL 60620. any chance the seller would take a cash, as-is offer, fast close with a brief inspection window? What's a good email for the written offer? Much appreciated!</t>
+          <t>Jose, hi. I'm Charles with Paragon Government Solutions, and I'm reaching out about 9122 S La Salle St, Chicago, IL 60620. Any chance the seller would take a cash, as-is offer, fast close with a brief inspection window? What's a good email for the written offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -12702,7 +12702,7 @@
       </c>
       <c r="F491" t="inlineStr">
         <is>
-          <t>Hello Joseph — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 20505 Hamburg St, Detroit, MI 48205. any chance the seller would take a cash, as-is offer with quick close and a short inspection. Where can I email the written terms? Appreciate it!</t>
+          <t>Hello Joseph — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 20505 Hamburg St, Detroit, MI 48205. Any chance the seller would take a cash, as-is offer with quick close and a short inspection. Where can I email the written terms? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -12727,7 +12727,7 @@
       </c>
       <c r="F492" t="inlineStr">
         <is>
-          <t>Good day JOSEPH — I'm Charles with Paragon Government Solutions. I'm reaching out about 5250 SANTA MONICA Boulevard S, Jacksonville, FL 32207. would the seller consider a cash, as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Thanks much!</t>
+          <t>Good day JOSEPH — I'm Charles with Paragon Government Solutions. I'm reaching out about 5250 SANTA MONICA Boulevard S, Jacksonville, FL 32207. Would the seller consider a cash, as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -12752,7 +12752,7 @@
       </c>
       <c r="F493" t="inlineStr">
         <is>
-          <t>Joseph, hi — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 2856 E 79th St, Chicago, IL 60649. would the seller consider a cash, as-is offer with fast cash close, short feasibility window. What email should I send the written offer to? Thanks so much!</t>
+          <t>Joseph, hi — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 2856 E 79th St, Chicago, IL 60649. Would the seller consider a cash, as-is offer with fast cash close, short feasibility window. What email should I send the written offer to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -12777,7 +12777,7 @@
       </c>
       <c r="F494" t="inlineStr">
         <is>
-          <t>Hey JOSEPH — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 1334 W 32ND Street, Jacksonville, FL 32209. any chance the seller would take a cash, as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Appreciate it!</t>
+          <t>Hey JOSEPH — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 1334 W 32ND Street, Jacksonville, FL 32209. Any chance the seller would take a cash, as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -12827,7 +12827,7 @@
       </c>
       <c r="F496" t="inlineStr">
         <is>
-          <t>Hello Joshua. I'm Charles with Paragon Government Solutions, and I'm reaching out about 3403 Alabama Ave, Dallas, TX 75216. open to a discounted cash, as-is offer, close quickly, short inspection period? Where can I email the written terms? Thanks!</t>
+          <t>Hello Joshua. I'm Charles with Paragon Government Solutions, and I'm reaching out about 3403 Alabama Ave, Dallas, TX 75216. Open to a discounted cash, as-is offer, close quickly, short inspection period? Where can I email the written terms? Thanks!</t>
         </is>
       </c>
     </row>
@@ -12852,7 +12852,7 @@
       </c>
       <c r="F497" t="inlineStr">
         <is>
-          <t>Hi Joshua — my name's Charles Pleasant, Paragon Government Solutions. I'm interested in buying 20017 Hawthorne St, Detroit, MI 48203 for cash. any chance the seller would take a cash, as-is offer with quick close and a short inspection. Where can I email the written terms? Appreciate it!</t>
+          <t>Hi Joshua — my name's Charles Pleasant, Paragon Government Solutions. I'm interested in buying 20017 Hawthorne St, Detroit, MI 48203 for cash. Any chance the seller would take a cash, as-is offer with quick close and a short inspection. Where can I email the written terms? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -12902,7 +12902,7 @@
       </c>
       <c r="F499" t="inlineStr">
         <is>
-          <t>JOYOUS, hi — this is Charles Pleasant with Paragon Government Solutions. I'm reaching out about 5227 BUNCHE Drive, Jacksonville, FL 32209. any chance the seller would take a cash, as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Thanks!</t>
+          <t>JOYOUS, hi — this is Charles Pleasant with Paragon Government Solutions. I'm reaching out about 5227 BUNCHE Drive, Jacksonville, FL 32209. Any chance the seller would take a cash, as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -12977,7 +12977,7 @@
       </c>
       <c r="F502" t="inlineStr">
         <is>
-          <t>Judith, hi. my name's Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 12125 Angelus Ave, Cleveland, OH 44105 for cash. open to a discounted cash, as-is offer, fast cash close, short feasibility window? What's the best email to send it to? Thanks much!</t>
+          <t>Judith, hi. My name's Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 12125 Angelus Ave, Cleveland, OH 44105 for cash. Open to a discounted cash, as-is offer, fast cash close, short feasibility window? What's the best email to send it to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -13027,7 +13027,7 @@
       </c>
       <c r="F504" t="inlineStr">
         <is>
-          <t>Juliana, hi — Charles here with Paragon Government Solutions. I'm a cash buyer interested in 155 Locust Ave W, Hamilton, NJ 08610. is the seller open to a cash as-is offer with close quickly, short inspection period. What's the best email to send it to? Appreciate it!</t>
+          <t>Juliana, hi — Charles here with Paragon Government Solutions. I'm a cash buyer interested in 155 Locust Ave W, Hamilton, NJ 08610. Is the seller open to a cash as-is offer with close quickly, short inspection period. What's the best email to send it to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -13052,7 +13052,7 @@
       </c>
       <c r="F505" t="inlineStr">
         <is>
-          <t>Hey Julie — Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 178 Vermillion Dr, Columbia, SC 29209. could the seller look at a cash, as-is offer with quick close and a short inspection. Best email for the formal offer? Appreciate it!</t>
+          <t>Hey Julie — Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 178 Vermillion Dr, Columbia, SC 29209. Could the seller look at a cash, as-is offer with quick close and a short inspection. Best email for the formal offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -13102,7 +13102,7 @@
       </c>
       <c r="F507" t="inlineStr">
         <is>
-          <t>Hello Justin — my name's Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 1246 Junction St, Detroit, MI 48209. would the owner entertain a cash as-is offer with fast cash close, short feasibility window. Where should I send the offer in writing? Thank you!</t>
+          <t>Hello Justin — my name's Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 1246 Junction St, Detroit, MI 48209. Would the owner entertain a cash as-is offer with fast cash close, short feasibility window. Where should I send the offer in writing? Thank you!</t>
         </is>
       </c>
     </row>
@@ -13127,7 +13127,7 @@
       </c>
       <c r="F508" t="inlineStr">
         <is>
-          <t>Justin, hi. Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 4701 Morris St NE APT 2604, Albuquerque, NM 87111. open to a discounted cash, as-is offer, fast close with a brief inspection window? What's the best email to send it to? Thanks so much!</t>
+          <t>Justin, hi. Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 4701 Morris St NE APT 2604, Albuquerque, NM 87111. Open to a discounted cash, as-is offer, fast close with a brief inspection window? What's the best email to send it to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -13177,7 +13177,7 @@
       </c>
       <c r="F510" t="inlineStr">
         <is>
-          <t>Hi there KALICA. Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 2846 YELLOW PINE Drive, Jacksonville, FL 32277 for cash. any chance the seller would take a cash, as-is offer, fast cash close, short feasibility window? What's the best email to send it to? Thank you!</t>
+          <t>Hi there KALICA. Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 2846 YELLOW PINE Drive, Jacksonville, FL 32277 for cash. Any chance the seller would take a cash, as-is offer, fast cash close, short feasibility window? What's the best email to send it to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -13252,7 +13252,7 @@
       </c>
       <c r="F513" t="inlineStr">
         <is>
-          <t>Hi Karen. Charles Pleasant, Paragon Government Solutions, and I came across 226 Curvewood Rd, Columbia, SC 29229 and buy cash. would the owner entertain a cash as-is offer, a quick clean close and short due diligence? Where can I email the written terms? Thanks so much!</t>
+          <t>Hi Karen. Charles Pleasant, Paragon Government Solutions, and I came across 226 Curvewood Rd, Columbia, SC 29229 and buy cash. Would the owner entertain a cash as-is offer, a quick clean close and short due diligence? Where can I email the written terms? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -13277,7 +13277,7 @@
       </c>
       <c r="F514" t="inlineStr">
         <is>
-          <t>Hi Karen — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 1040 Kentucky St SE, Albuquerque, NM 87108. could the seller look at a cash, as-is offer with quick close and a short inspection. What's the best email to send it to? Thank you!</t>
+          <t>Hi Karen — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 1040 Kentucky St SE, Albuquerque, NM 87108. Could the seller look at a cash, as-is offer with quick close and a short inspection. What's the best email to send it to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -13302,7 +13302,7 @@
       </c>
       <c r="F515" t="inlineStr">
         <is>
-          <t>Hi KAREN. I'm Charles with Paragon Government Solutions, and I'm a cash buyer interested in 6929 ROLLO Road, Jacksonville, FL 32205. would the owner entertain a cash as-is offer, fast close with a brief inspection window? What's the best email to send it to? Thank you!</t>
+          <t>Hi KAREN. I'm Charles with Paragon Government Solutions, and I'm a cash buyer interested in 6929 ROLLO Road, Jacksonville, FL 32205. Would the owner entertain a cash as-is offer, fast close with a brief inspection window? What's the best email to send it to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -13327,7 +13327,7 @@
       </c>
       <c r="F516" t="inlineStr">
         <is>
-          <t>Hi Karina. Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 4030 W MARICOPA Street, Phoenix, AZ 85009 for cash. is the seller open to a cash as-is offer, fast cash close, short feasibility window? Where can I email the written terms? Thanks so much!</t>
+          <t>Hi Karina. Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 4030 W MARICOPA Street, Phoenix, AZ 85009 for cash. Is the seller open to a cash as-is offer, fast cash close, short feasibility window? Where can I email the written terms? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -13402,7 +13402,7 @@
       </c>
       <c r="F519" t="inlineStr">
         <is>
-          <t>Hey Karmen — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 10210 S Prairie Ave, Chicago, IL 60628. would the seller consider a cash, as-is offer with quick close and a short inspection. Where should I send the offer in writing? Much appreciated!</t>
+          <t>Hey Karmen — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 10210 S Prairie Ave, Chicago, IL 60628. Would the seller consider a cash, as-is offer with quick close and a short inspection. Where should I send the offer in writing? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -13427,7 +13427,7 @@
       </c>
       <c r="F520" t="inlineStr">
         <is>
-          <t>Good day Kashmir. my name's Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 7305 Tremper St, Houston, TX 77020. any chance the seller would take a cash, as-is offer, quick close and a short inspection? What email should I send the written offer to? Thanks!</t>
+          <t>Good day Kashmir. My name's Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 7305 Tremper St, Houston, TX 77020. Any chance the seller would take a cash, as-is offer, quick close and a short inspection? What email should I send the written offer to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -13477,7 +13477,7 @@
       </c>
       <c r="F522" t="inlineStr">
         <is>
-          <t>Katy, hi. this is Charles Pleasant with Paragon Government Solutions, and I'm a cash buyer interested in 2319 Kathleen Ave, Dallas, TX 75216. open to a discounted cash, as-is offer, fast cash close, short feasibility window? What's the best email to send it to? Thanks!</t>
+          <t>Katy, hi. This is Charles Pleasant with Paragon Government Solutions, and I'm a cash buyer interested in 2319 Kathleen Ave, Dallas, TX 75216. Open to a discounted cash, as-is offer, fast cash close, short feasibility window? What's the best email to send it to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -13502,7 +13502,7 @@
       </c>
       <c r="F523" t="inlineStr">
         <is>
-          <t>Hi Keith — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 112 Willow Branch Dr, West Monroe, LA 71291. would the owner entertain a cash as-is offer with close quickly, short inspection period. What's the best email to send it to? Thanks!</t>
+          <t>Hi Keith — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 112 Willow Branch Dr, West Monroe, LA 71291. Would the owner entertain a cash as-is offer with close quickly, short inspection period. What's the best email to send it to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -13527,7 +13527,7 @@
       </c>
       <c r="F524" t="inlineStr">
         <is>
-          <t>Hi KEITH. this is Charles Pleasant with Paragon Government Solutions, and I'd like to put in a cash offer on 4507 TRENTON Drive S, Jacksonville, FL 32209. any chance the seller would take a cash, as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Thank you!</t>
+          <t>Hi KEITH. This is Charles Pleasant with Paragon Government Solutions, and I'd like to put in a cash offer on 4507 TRENTON Drive S, Jacksonville, FL 32209. Any chance the seller would take a cash, as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Thank you!</t>
         </is>
       </c>
     </row>
@@ -13552,7 +13552,7 @@
       </c>
       <c r="F525" t="inlineStr">
         <is>
-          <t>Hi Kelley. my name's Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 1630 E ADAMS Street, Phoenix, AZ 85034. open to a discounted cash, as-is offer, fast cash close, short feasibility window? What's the best email to send it to? Thanks much!</t>
+          <t>Hi Kelley. My name's Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 1630 E ADAMS Street, Phoenix, AZ 85034. Open to a discounted cash, as-is offer, fast cash close, short feasibility window? What's the best email to send it to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -13627,7 +13627,7 @@
       </c>
       <c r="F528" t="inlineStr">
         <is>
-          <t>Hi there Kenisha. I'm Charles with Paragon Government Solutions, and I'm reaching out about 2324 Alpine Rd, Columbia, SC 29223. is the seller open to a cash as-is offer, fast cash close, short feasibility window? Best email for the formal offer? Much appreciated!</t>
+          <t>Hi there Kenisha. I'm Charles with Paragon Government Solutions, and I'm reaching out about 2324 Alpine Rd, Columbia, SC 29223. Is the seller open to a cash as-is offer, fast cash close, short feasibility window? Best email for the formal offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -13652,7 +13652,7 @@
       </c>
       <c r="F529" t="inlineStr">
         <is>
-          <t>Hello KENNETH — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 1113 Branson St, Fayetteville, NC 28305. could the seller look at a cash, as-is offer with close quickly, short inspection period. Where can I email the written terms? Thanks so much!</t>
+          <t>Hello KENNETH — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 1113 Branson St, Fayetteville, NC 28305. Could the seller look at a cash, as-is offer with close quickly, short inspection period. Where can I email the written terms? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -13752,7 +13752,7 @@
       </c>
       <c r="F533" t="inlineStr">
         <is>
-          <t>Hi there Kevin — Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 1223 Harvey St, Columbia, SC 29201. is the seller open to a cash as-is offer with a quick clean close and short due diligence. What email should I send the written offer to? Thanks so much!</t>
+          <t>Hi there Kevin — Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 1223 Harvey St, Columbia, SC 29201. Is the seller open to a cash as-is offer with a quick clean close and short due diligence. What email should I send the written offer to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -13802,7 +13802,7 @@
       </c>
       <c r="F535" t="inlineStr">
         <is>
-          <t>Good day Khaula. Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 3718 Barbara Ave, Bakersfield, CA 93309 for cash. any chance the seller would take a cash, as-is offer, a quick clean close and short due diligence? Best email for the formal offer? Much appreciated!</t>
+          <t>Good day Khaula. Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 3718 Barbara Ave, Bakersfield, CA 93309 for cash. Any chance the seller would take a cash, as-is offer, a quick clean close and short due diligence? Best email for the formal offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -13852,7 +13852,7 @@
       </c>
       <c r="F537" t="inlineStr">
         <is>
-          <t>Good day KIM. Charles here with Paragon Government Solutions, and I'm interested in buying 752 ACOSTA Street, Jacksonville, FL 32204 for cash. open to a discounted cash, as-is offer, quick close and a short inspection? Best email for the formal offer? Appreciate it!</t>
+          <t>Good day KIM. Charles here with Paragon Government Solutions, and I'm interested in buying 752 ACOSTA Street, Jacksonville, FL 32204 for cash. Open to a discounted cash, as-is offer, quick close and a short inspection? Best email for the formal offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -13877,7 +13877,7 @@
       </c>
       <c r="F538" t="inlineStr">
         <is>
-          <t>Hello Kim. I'm Charles with Paragon Government Solutions, and I'm reaching out about 3338 Taylor St, Detroit, MI 48206. any chance the seller would take a cash, as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Thank you!</t>
+          <t>Hello Kim. I'm Charles with Paragon Government Solutions, and I'm reaching out about 3338 Taylor St, Detroit, MI 48206. Any chance the seller would take a cash, as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Thank you!</t>
         </is>
       </c>
     </row>
@@ -14002,7 +14002,7 @@
       </c>
       <c r="F543" t="inlineStr">
         <is>
-          <t>Good day Kodee — my name's Charles Pleasant, Paragon Government Solutions. I'm reaching out about 311 Lockner Rd, Columbia, SC 29212. open to a discounted cash, as-is offer with fast close with a brief inspection window. Where can I email the written terms? Thank you!</t>
+          <t>Good day Kodee — my name's Charles Pleasant, Paragon Government Solutions. I'm reaching out about 311 Lockner Rd, Columbia, SC 29212. Open to a discounted cash, as-is offer with fast close with a brief inspection window. Where can I email the written terms? Thank you!</t>
         </is>
       </c>
     </row>
@@ -14027,7 +14027,7 @@
       </c>
       <c r="F544" t="inlineStr">
         <is>
-          <t>Hi KONT — Charles Pleasant, Paragon Government Solutions. I came across 4104 LEONARD Circle E, Jacksonville, FL 32209 and buy cash. could the seller look at a cash, as-is offer with close quickly, short inspection period. Where can I email the written terms? Thanks much!</t>
+          <t>Hi KONT — Charles Pleasant, Paragon Government Solutions. I came across 4104 LEONARD Circle E, Jacksonville, FL 32209 and buy cash. Could the seller look at a cash, as-is offer with close quickly, short inspection period. Where can I email the written terms? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -14127,7 +14127,7 @@
       </c>
       <c r="F548" t="inlineStr">
         <is>
-          <t>Hi Kristian — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 4114 Averill St, Houston, TX 77009. could the seller look at a cash, as-is offer with fast cash close, short feasibility window. Where should I send the offer in writing? Much appreciated!</t>
+          <t>Hi Kristian — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 4114 Averill St, Houston, TX 77009. Could the seller look at a cash, as-is offer with fast cash close, short feasibility window. Where should I send the offer in writing? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -14177,7 +14177,7 @@
       </c>
       <c r="F550" t="inlineStr">
         <is>
-          <t>Hi there Kya. my name's Charles Pleasant, Paragon Government Solutions, and I came across 5505 Hamlet Ave, Baltimore, MD 21214 and buy cash. any chance the seller would take a cash, as-is offer, a quick clean close and short due diligence? What's the best email to send it to? Thanks much!</t>
+          <t>Hi there Kya. My name's Charles Pleasant, Paragon Government Solutions, and I came across 5505 Hamlet Ave, Baltimore, MD 21214 and buy cash. Any chance the seller would take a cash, as-is offer, a quick clean close and short due diligence? What's the best email to send it to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -14227,7 +14227,7 @@
       </c>
       <c r="F552" t="inlineStr">
         <is>
-          <t>Hello Lache — my name's Charles Pleasant, Paragon Government Solutions. I'm reaching out about 4103 Sablemist Ct, Houston, TX 77014. would the seller consider a cash, as-is offer with a quick clean close and short due diligence. Where can I email the written terms? Appreciate it!</t>
+          <t>Hello Lache — my name's Charles Pleasant, Paragon Government Solutions. I'm reaching out about 4103 Sablemist Ct, Houston, TX 77014. Would the seller consider a cash, as-is offer with a quick clean close and short due diligence. Where can I email the written terms? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -14252,7 +14252,7 @@
       </c>
       <c r="F553" t="inlineStr">
         <is>
-          <t>LaCretia, hi — I'm Charles with Paragon Government Solutions. I'm a cash buyer interested in 17694 Avon Ave, Detroit, MI 48219. could the seller look at a cash, as-is offer with close quickly, short inspection period. Best email for the formal offer? Thanks!</t>
+          <t>LaCretia, hi — I'm Charles with Paragon Government Solutions. I'm a cash buyer interested in 17694 Avon Ave, Detroit, MI 48219. Could the seller look at a cash, as-is offer with close quickly, short inspection period. Best email for the formal offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -14302,7 +14302,7 @@
       </c>
       <c r="F555" t="inlineStr">
         <is>
-          <t>Hi there Lara. Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 5003 Gleneagles Ct, Houston, TX 77084. any chance the seller would take a cash, as-is offer, a quick clean close and short due diligence? What email should I send the written offer to? Thanks!</t>
+          <t>Hi there Lara. Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 5003 Gleneagles Ct, Houston, TX 77084. Any chance the seller would take a cash, as-is offer, a quick clean close and short due diligence? What email should I send the written offer to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -14327,7 +14327,7 @@
       </c>
       <c r="F556" t="inlineStr">
         <is>
-          <t>Lara, hi. Charles here with Paragon Government Solutions, and I'm interested in buying 113 Wescott Pl, Columbia, SC 29229 for cash. open to a discounted cash, as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Thank you!</t>
+          <t>Lara, hi. Charles here with Paragon Government Solutions, and I'm interested in buying 113 Wescott Pl, Columbia, SC 29229 for cash. Open to a discounted cash, as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Thank you!</t>
         </is>
       </c>
     </row>
@@ -14352,7 +14352,7 @@
       </c>
       <c r="F557" t="inlineStr">
         <is>
-          <t>Hello LASHAWN. this is Charles Pleasant with Paragon Government Solutions, and I came across 1730 AUDUBON Street, Jacksonville, FL 32208 and buy cash. would the owner entertain a cash as-is offer, a quick clean close and short due diligence? What's a good email for the written offer? Appreciate it!</t>
+          <t>Hello LASHAWN. This is Charles Pleasant with Paragon Government Solutions, and I came across 1730 AUDUBON Street, Jacksonville, FL 32208 and buy cash. Would the owner entertain a cash as-is offer, a quick clean close and short due diligence? What's a good email for the written offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -14377,7 +14377,7 @@
       </c>
       <c r="F558" t="inlineStr">
         <is>
-          <t>Hello LaToya. my name's Charles Pleasant, Paragon Government Solutions, and I came across 16525 Prevost St, Detroit, MI 48235 and buy cash. would the owner entertain a cash as-is offer, close quickly, short inspection period? Where should I send the offer in writing? Thank you!</t>
+          <t>Hello LaToya. My name's Charles Pleasant, Paragon Government Solutions, and I came across 16525 Prevost St, Detroit, MI 48235 and buy cash. Would the owner entertain a cash as-is offer, close quickly, short inspection period? Where should I send the offer in writing? Thank you!</t>
         </is>
       </c>
     </row>
@@ -14427,7 +14427,7 @@
       </c>
       <c r="F560" t="inlineStr">
         <is>
-          <t>Hey Laura — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 806 Homestead St, Baltimore, MD 21218. would the owner entertain a cash as-is offer with close quickly, short inspection period. What's the best email to send it to? Much appreciated!</t>
+          <t>Hey Laura — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 806 Homestead St, Baltimore, MD 21218. Would the owner entertain a cash as-is offer with close quickly, short inspection period. What's the best email to send it to? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -14477,7 +14477,7 @@
       </c>
       <c r="F562" t="inlineStr">
         <is>
-          <t>Hi Lauren. this is Charles Pleasant with Paragon Government Solutions, and I'm a cash investor looking at 2009 Bancroft St, Lake Charles, LA 70607. would the owner entertain a cash as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Appreciate it!</t>
+          <t>Hi Lauren. This is Charles Pleasant with Paragon Government Solutions, and I'm a cash investor looking at 2009 Bancroft St, Lake Charles, LA 70607. Would the owner entertain a cash as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -14502,7 +14502,7 @@
       </c>
       <c r="F563" t="inlineStr">
         <is>
-          <t>Good day Lauren. Charles here with Paragon Government Solutions, and I'm interested in buying 6526 Oak Garden Dr, Baton Rouge, LA 70817 for cash. could the seller look at a cash, as-is offer, quick close and a short inspection? Where should I send the offer in writing? Thanks!</t>
+          <t>Good day Lauren. Charles here with Paragon Government Solutions, and I'm interested in buying 6526 Oak Garden Dr, Baton Rouge, LA 70817 for cash. Could the seller look at a cash, as-is offer, quick close and a short inspection? Where should I send the offer in writing? Thanks!</t>
         </is>
       </c>
     </row>
@@ -14577,7 +14577,7 @@
       </c>
       <c r="F566" t="inlineStr">
         <is>
-          <t>Hi there Lee. my name's Charles Pleasant, Paragon Government Solutions, and I'm a cash investor looking at 9 Vicky Ct, Hamilton, NJ 08610. could the seller look at a cash, as-is offer, close quickly, short inspection period? Where can I email the written terms? Thanks much!</t>
+          <t>Hi there Lee. My name's Charles Pleasant, Paragon Government Solutions, and I'm a cash investor looking at 9 Vicky Ct, Hamilton, NJ 08610. Could the seller look at a cash, as-is offer, close quickly, short inspection period? Where can I email the written terms? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -14602,7 +14602,7 @@
       </c>
       <c r="F567" t="inlineStr">
         <is>
-          <t>Leilani, hi. this is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 10712 Grantwood Ave, Cleveland, OH 44108. could the seller look at a cash, as-is offer, fast cash close, short feasibility window? What's a good email for the written offer? Thanks!</t>
+          <t>Leilani, hi. This is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 10712 Grantwood Ave, Cleveland, OH 44108. Could the seller look at a cash, as-is offer, fast cash close, short feasibility window? What's a good email for the written offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -14677,7 +14677,7 @@
       </c>
       <c r="F570" t="inlineStr">
         <is>
-          <t>Hi there Lesa — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 146 Dunham Rd, Columbia, SC 29209. any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. What's the best email to send it to? Thank you!</t>
+          <t>Hi there Lesa — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 146 Dunham Rd, Columbia, SC 29209. Any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. What's the best email to send it to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -14727,7 +14727,7 @@
       </c>
       <c r="F572" t="inlineStr">
         <is>
-          <t>Hi there LeTanya. Charles here with Paragon Government Solutions, and I'm a cash investor looking at 2043 Parker Ranch Rd SE, Atlanta, GA 30316. could the seller look at a cash, as-is offer, quick close and a short inspection? What's a good email for the written offer? Thanks so much!</t>
+          <t>Hi there LeTanya. Charles here with Paragon Government Solutions, and I'm a cash investor looking at 2043 Parker Ranch Rd SE, Atlanta, GA 30316. Could the seller look at a cash, as-is offer, quick close and a short inspection? What's a good email for the written offer? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -14877,7 +14877,7 @@
       </c>
       <c r="F578" t="inlineStr">
         <is>
-          <t>Linda, hi — Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 10 Stacey Ave, Trenton, NJ 08618. open to a discounted cash, as-is offer with a quick clean close and short due diligence. Where should I send the offer in writing? Thank you!</t>
+          <t>Linda, hi — Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 10 Stacey Ave, Trenton, NJ 08618. Open to a discounted cash, as-is offer with a quick clean close and short due diligence. Where should I send the offer in writing? Thank you!</t>
         </is>
       </c>
     </row>
@@ -14902,7 +14902,7 @@
       </c>
       <c r="F579" t="inlineStr">
         <is>
-          <t>Lindsey, hi. Charles here with Paragon Government Solutions, and I'm a cash buyer interested in 5525 E THOMAS Road #R9, Phoenix, AZ 85018. could the seller look at a cash, as-is offer, fast cash close, short feasibility window? What's a good email for the written offer? Much appreciated!</t>
+          <t>Lindsey, hi. Charles here with Paragon Government Solutions, and I'm a cash buyer interested in 5525 E THOMAS Road #R9, Phoenix, AZ 85018. Could the seller look at a cash, as-is offer, fast cash close, short feasibility window? What's a good email for the written offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -15052,7 +15052,7 @@
       </c>
       <c r="F585" t="inlineStr">
         <is>
-          <t>Lori, hi. my name's Charles Pleasant, Paragon Government Solutions, and I came across 12346 Elmdale St, Detroit, MI 48213 and buy cash. would the seller consider a cash, as-is offer, fast close with a brief inspection window? Where should I send the offer in writing? Appreciate it!</t>
+          <t>Lori, hi. My name's Charles Pleasant, Paragon Government Solutions, and I came across 12346 Elmdale St, Detroit, MI 48213 and buy cash. Would the seller consider a cash, as-is offer, fast close with a brief inspection window? Where should I send the offer in writing? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -15127,7 +15127,7 @@
       </c>
       <c r="F588" t="inlineStr">
         <is>
-          <t>Good day Luan. this is Charles Pleasant with Paragon Government Solutions, and I'm a cash investor looking at 3220 Plymouth Pl, New Orleans, LA 70131. could the seller look at a cash, as-is offer, quick close and a short inspection? What's a good email for the written offer? Thanks!</t>
+          <t>Good day Luan. This is Charles Pleasant with Paragon Government Solutions, and I'm a cash investor looking at 3220 Plymouth Pl, New Orleans, LA 70131. Could the seller look at a cash, as-is offer, quick close and a short inspection? What's a good email for the written offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -15177,7 +15177,7 @@
       </c>
       <c r="F590" t="inlineStr">
         <is>
-          <t>Hi there LUCIE. Charles here with Paragon Government Solutions, and I'm interested in buying 162 E 54TH Street, Jacksonville, FL 32208 for cash. would the owner entertain a cash as-is offer, fast close with a brief inspection window? Best email for the formal offer? Much appreciated!</t>
+          <t>Hi there LUCIE. Charles here with Paragon Government Solutions, and I'm interested in buying 162 E 54TH Street, Jacksonville, FL 32208 for cash. Would the owner entertain a cash as-is offer, fast close with a brief inspection window? Best email for the formal offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -15202,7 +15202,7 @@
       </c>
       <c r="F591" t="inlineStr">
         <is>
-          <t>Hi Luis. my name's Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 342 Creekwood Run, Lakeland, FL 33809. would the seller consider a cash, as-is offer, a quick clean close and short due diligence? Where can I email the written terms? Thanks so much!</t>
+          <t>Hi Luis. My name's Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 342 Creekwood Run, Lakeland, FL 33809. Would the seller consider a cash, as-is offer, a quick clean close and short due diligence? Where can I email the written terms? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -15227,7 +15227,7 @@
       </c>
       <c r="F592" t="inlineStr">
         <is>
-          <t>Hello Lydia. this is Charles Pleasant with Paragon Government Solutions, and I'd like to put in a cash offer on 13515 S Baltimore Ave, Chicago, IL 60633. open to a discounted cash, as-is offer, fast close with a brief inspection window? Where can I email the written terms? Thanks so much!</t>
+          <t>Hello Lydia. This is Charles Pleasant with Paragon Government Solutions, and I'd like to put in a cash offer on 13515 S Baltimore Ave, Chicago, IL 60633. Open to a discounted cash, as-is offer, fast close with a brief inspection window? Where can I email the written terms? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -15277,7 +15277,7 @@
       </c>
       <c r="F594" t="inlineStr">
         <is>
-          <t>Hello Maico — this is Charles Pleasant with Paragon Government Solutions. I'm reaching out about 1638 W MOHAVE Street, Phoenix, AZ 85007. would the seller consider a cash, as-is offer with fast close with a brief inspection window. What's the best email to send it to? Appreciate it!</t>
+          <t>Hello Maico — this is Charles Pleasant with Paragon Government Solutions. I'm reaching out about 1638 W MOHAVE Street, Phoenix, AZ 85007. Would the seller consider a cash, as-is offer with fast close with a brief inspection window. What's the best email to send it to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -15302,7 +15302,7 @@
       </c>
       <c r="F595" t="inlineStr">
         <is>
-          <t>Hi there Makia. I'm Charles with Paragon Government Solutions, and I'm reaching out about 8357 Navy St, Detroit, MI 48209. would the seller consider a cash, as-is offer, quick close and a short inspection? Where can I email the written terms? Much appreciated!</t>
+          <t>Hi there Makia. I'm Charles with Paragon Government Solutions, and I'm reaching out about 8357 Navy St, Detroit, MI 48209. Would the seller consider a cash, as-is offer, quick close and a short inspection? Where can I email the written terms? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -15327,7 +15327,7 @@
       </c>
       <c r="F596" t="inlineStr">
         <is>
-          <t>Hi there Malaka. this is Charles Pleasant with Paragon Government Solutions, and I came across 10731 Roxbury St, Detroit, MI 48224 and buy cash. any chance the seller would take a cash, as-is offer, a quick clean close and short due diligence? What's the best email to send it to? Thank you!</t>
+          <t>Hi there Malaka. This is Charles Pleasant with Paragon Government Solutions, and I came across 10731 Roxbury St, Detroit, MI 48224 and buy cash. Any chance the seller would take a cash, as-is offer, a quick clean close and short due diligence? What's the best email to send it to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -15352,7 +15352,7 @@
       </c>
       <c r="F597" t="inlineStr">
         <is>
-          <t>Malwina, hi. Charles Pleasant, Paragon Government Solutions, and I'm a cash buyer interested in 8252 S Marshfield Ave, Chicago, IL 60620. open to a discounted cash, as-is offer, close quickly, short inspection period? What's the best email to send it to? Thank you!</t>
+          <t>Malwina, hi. Charles Pleasant, Paragon Government Solutions, and I'm a cash buyer interested in 8252 S Marshfield Ave, Chicago, IL 60620. Open to a discounted cash, as-is offer, close quickly, short inspection period? What's the best email to send it to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -15402,7 +15402,7 @@
       </c>
       <c r="F599" t="inlineStr">
         <is>
-          <t>Good day Marc — Charles Pleasant, Paragon Government Solutions. I came across 6003 Glenoak Ave, Baltimore, MD 21214 and buy cash. would the seller consider a cash, as-is offer with fast cash close, short feasibility window. Where should I send the offer in writing? Thanks so much!</t>
+          <t>Good day Marc — Charles Pleasant, Paragon Government Solutions. I came across 6003 Glenoak Ave, Baltimore, MD 21214 and buy cash. Would the seller consider a cash, as-is offer with fast cash close, short feasibility window. Where should I send the offer in writing? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -15427,7 +15427,7 @@
       </c>
       <c r="F600" t="inlineStr">
         <is>
-          <t>Hi there Marc — Charles here with Paragon Government Solutions. I'm a cash buyer interested in 3010 NE 6th Place Cpe, Coral, FL 33909. could the seller look at a cash, as-is offer with fast close with a brief inspection window. What's the best email to send it to? Thanks!</t>
+          <t>Hi there Marc — Charles here with Paragon Government Solutions. I'm a cash buyer interested in 3010 NE 6th Place Cpe, Coral, FL 33909. Could the seller look at a cash, as-is offer with fast close with a brief inspection window. What's the best email to send it to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -15477,7 +15477,7 @@
       </c>
       <c r="F602" t="inlineStr">
         <is>
-          <t>Hello Marc — I'm Charles with Paragon Government Solutions. I'm interested in buying 8313 S Wabash Ave, Chicago, IL 60619 for cash. could the seller look at a cash, as-is offer with a quick clean close and short due diligence. Where should I send the offer in writing? Thanks much!</t>
+          <t>Hello Marc — I'm Charles with Paragon Government Solutions. I'm interested in buying 8313 S Wabash Ave, Chicago, IL 60619 for cash. Could the seller look at a cash, as-is offer with a quick clean close and short due diligence. Where should I send the offer in writing? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -15502,7 +15502,7 @@
       </c>
       <c r="F603" t="inlineStr">
         <is>
-          <t>Hi Marcela. this is Charles Pleasant with Paragon Government Solutions, and I'm interested in buying 3712 W Cold Spring Ln, Baltimore, MD 21215 for cash. any chance the seller would take a cash, as-is offer, quick close and a short inspection? Best email for the formal offer? Thanks!</t>
+          <t>Hi Marcela. This is Charles Pleasant with Paragon Government Solutions, and I'm interested in buying 3712 W Cold Spring Ln, Baltimore, MD 21215 for cash. Any chance the seller would take a cash, as-is offer, quick close and a short inspection? Best email for the formal offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -15527,7 +15527,7 @@
       </c>
       <c r="F604" t="inlineStr">
         <is>
-          <t>Hi there Marcelo. this is Charles Pleasant with Paragon Government Solutions, and I'd like to put in a cash offer on 1918 Michigan Ave, Dallas, TX 75216. open to a discounted cash, as-is offer, fast close with a brief inspection window? Where can I email the written terms? Thanks so much!</t>
+          <t>Hi there Marcelo. This is Charles Pleasant with Paragon Government Solutions, and I'd like to put in a cash offer on 1918 Michigan Ave, Dallas, TX 75216. Open to a discounted cash, as-is offer, fast close with a brief inspection window? Where can I email the written terms? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -15602,7 +15602,7 @@
       </c>
       <c r="F607" t="inlineStr">
         <is>
-          <t>Hello Marcy. Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 1115 Belmont Green Rd, Columbia, SC 29209. is the seller open to a cash as-is offer, close quickly, short inspection period? What email should I send the written offer to? Thank you!</t>
+          <t>Hello Marcy. Charles Pleasant, Paragon Government Solutions, and I'm reaching out about 1115 Belmont Green Rd, Columbia, SC 29209. Is the seller open to a cash as-is offer, close quickly, short inspection period? What email should I send the written offer to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -15677,7 +15677,7 @@
       </c>
       <c r="F610" t="inlineStr">
         <is>
-          <t>Maria, hi. I'm Charles with Paragon Government Solutions, and I'm reaching out about 4541 S Laporte Ave, Chicago, IL 60638. would the owner entertain a cash as-is offer, quick close and a short inspection? What's the best email to send it to? Thanks so much!</t>
+          <t>Maria, hi. I'm Charles with Paragon Government Solutions, and I'm reaching out about 4541 S Laporte Ave, Chicago, IL 60638. Would the owner entertain a cash as-is offer, quick close and a short inspection? What's the best email to send it to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -15752,7 +15752,7 @@
       </c>
       <c r="F613" t="inlineStr">
         <is>
-          <t>Good day Maria. this is Charles Pleasant with Paragon Government Solutions, and I came across 19355 Alcoy St, Detroit, MI 48205 and buy cash. open to a discounted cash, as-is offer, fast close with a brief inspection window? Best email for the formal offer? Much appreciated!</t>
+          <t>Good day Maria. This is Charles Pleasant with Paragon Government Solutions, and I came across 19355 Alcoy St, Detroit, MI 48205 and buy cash. Open to a discounted cash, as-is offer, fast close with a brief inspection window? Best email for the formal offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -15877,7 +15877,7 @@
       </c>
       <c r="F618" t="inlineStr">
         <is>
-          <t>Good day Maricela — I'm Charles with Paragon Government Solutions. I'm reaching out about 124 Harriet Dr, San Antonio, TX 78216. any chance the seller would take a cash, as-is offer with quick close and a short inspection. Where can I email the written terms? Thanks much!</t>
+          <t>Good day Maricela — I'm Charles with Paragon Government Solutions. I'm reaching out about 124 Harriet Dr, San Antonio, TX 78216. Any chance the seller would take a cash, as-is offer with quick close and a short inspection. Where can I email the written terms? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -15902,7 +15902,7 @@
       </c>
       <c r="F619" t="inlineStr">
         <is>
-          <t>Hey Maricela — Charles here with Paragon Government Solutions. I'm reaching out about 7667 Ellsworth St, Detroit, MI 48238. open to a discounted cash, as-is offer with close quickly, short inspection period. What's the best email to send it to? Appreciate it!</t>
+          <t>Hey Maricela — Charles here with Paragon Government Solutions. I'm reaching out about 7667 Ellsworth St, Detroit, MI 48238. Open to a discounted cash, as-is offer with close quickly, short inspection period. What's the best email to send it to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -16002,7 +16002,7 @@
       </c>
       <c r="F623" t="inlineStr">
         <is>
-          <t>Mark, hi. Charles Pleasant, Paragon Government Solutions, and I came across 7039 Sheffield Dr, Lakeland, FL 33810 and buy cash. open to a discounted cash, as-is offer, fast close with a brief inspection window? Best email for the formal offer? Appreciate it!</t>
+          <t>Mark, hi. Charles Pleasant, Paragon Government Solutions, and I came across 7039 Sheffield Dr, Lakeland, FL 33810 and buy cash. Open to a discounted cash, as-is offer, fast close with a brief inspection window? Best email for the formal offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -16027,7 +16027,7 @@
       </c>
       <c r="F624" t="inlineStr">
         <is>
-          <t>Hey Mark — I'm Charles with Paragon Government Solutions. I came across 1010 N 18TH Street, Phoenix, AZ 85006 and buy cash. would the seller consider a cash, as-is offer with fast cash close, short feasibility window. Where should I send the offer in writing? Thanks much!</t>
+          <t>Hey Mark — I'm Charles with Paragon Government Solutions. I came across 1010 N 18TH Street, Phoenix, AZ 85006 and buy cash. Would the seller consider a cash, as-is offer with fast cash close, short feasibility window. Where should I send the offer in writing? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -16052,7 +16052,7 @@
       </c>
       <c r="F625" t="inlineStr">
         <is>
-          <t>Hey Marketta. I'm Charles with Paragon Government Solutions, and I'm a cash buyer interested in 16241 E State Fair St, Detroit, MI 48205. would the seller consider a cash, as-is offer, a quick clean close and short due diligence? What's the best email to send it to? Much appreciated!</t>
+          <t>Hey Marketta. I'm Charles with Paragon Government Solutions, and I'm a cash buyer interested in 16241 E State Fair St, Detroit, MI 48205. Would the seller consider a cash, as-is offer, a quick clean close and short due diligence? What's the best email to send it to? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -16127,7 +16127,7 @@
       </c>
       <c r="F628" t="inlineStr">
         <is>
-          <t>Hey Martha — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 4403 Allen St, Houston, TX 77007. open to a discounted cash, as-is offer with close quickly, short inspection period. What's the best email to send it to? Thanks much!</t>
+          <t>Hey Martha — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 4403 Allen St, Houston, TX 77007. Open to a discounted cash, as-is offer with close quickly, short inspection period. What's the best email to send it to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -16202,7 +16202,7 @@
       </c>
       <c r="F631" t="inlineStr">
         <is>
-          <t>Hi there Mary — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 511 Solar Dr, San Antonio, TX 78227. would the owner entertain a cash as-is offer with close quickly, short inspection period. What's a good email for the written offer? Thanks so much!</t>
+          <t>Hi there Mary — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 511 Solar Dr, San Antonio, TX 78227. Would the owner entertain a cash as-is offer with close quickly, short inspection period. What's a good email for the written offer? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -16227,7 +16227,7 @@
       </c>
       <c r="F632" t="inlineStr">
         <is>
-          <t>Hi there Matt — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 24 Merrymount Rd, Baltimore, MD 21210. is the seller open to a cash as-is offer with quick close and a short inspection. Where should I send the offer in writing? Thanks so much!</t>
+          <t>Hi there Matt — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 24 Merrymount Rd, Baltimore, MD 21210. Is the seller open to a cash as-is offer with quick close and a short inspection. Where should I send the offer in writing? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -16277,7 +16277,7 @@
       </c>
       <c r="F634" t="inlineStr">
         <is>
-          <t>Good day MATTHEW — Charles here with Paragon Government Solutions. I'm interested in buying 4840 COLONIAL Avenue, Jacksonville, FL 32210 for cash. would the owner entertain a cash as-is offer with fast close with a brief inspection window. What's the best email to send it to? Appreciate it!</t>
+          <t>Good day MATTHEW — Charles here with Paragon Government Solutions. I'm interested in buying 4840 COLONIAL Avenue, Jacksonville, FL 32210 for cash. Would the owner entertain a cash as-is offer with fast close with a brief inspection window. What's the best email to send it to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -16327,7 +16327,7 @@
       </c>
       <c r="F636" t="inlineStr">
         <is>
-          <t>Hello Mauricio. I'm Charles with Paragon Government Solutions, and I'm a cash buyer interested in 5242 W Monroe St, Chicago, IL 60644. would the owner entertain a cash as-is offer, close quickly, short inspection period? Best email for the formal offer? Appreciate it!</t>
+          <t>Hello Mauricio. I'm Charles with Paragon Government Solutions, and I'm a cash buyer interested in 5242 W Monroe St, Chicago, IL 60644. Would the owner entertain a cash as-is offer, close quickly, short inspection period? Best email for the formal offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -16352,7 +16352,7 @@
       </c>
       <c r="F637" t="inlineStr">
         <is>
-          <t>Hey Maya. my name's Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 5936 Hillcrest St, Detroit, MI 48236. is the seller open to a cash as-is offer, a quick clean close and short due diligence? Best email for the formal offer? Thanks!</t>
+          <t>Hey Maya. My name's Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 5936 Hillcrest St, Detroit, MI 48236. Is the seller open to a cash as-is offer, a quick clean close and short due diligence? Best email for the formal offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -16477,7 +16477,7 @@
       </c>
       <c r="F642" t="inlineStr">
         <is>
-          <t>Hi Michael — Charles here with Paragon Government Solutions. I'm a cash investor looking at 120 Curvewood Rd, Columbia, SC 29229. open to a discounted cash, as-is offer with fast cash close, short feasibility window. What email should I send the written offer to? Thanks!</t>
+          <t>Hi Michael — Charles here with Paragon Government Solutions. I'm a cash investor looking at 120 Curvewood Rd, Columbia, SC 29229. Open to a discounted cash, as-is offer with fast cash close, short feasibility window. What email should I send the written offer to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -16527,7 +16527,7 @@
       </c>
       <c r="F644" t="inlineStr">
         <is>
-          <t>Good day Michael — Charles here with Paragon Government Solutions. I'm a cash buyer interested in 7939 S Kingston Ave, Chicago, IL 60617. would the owner entertain a cash as-is offer with fast cash close, short feasibility window. Best email for the formal offer? Thanks much!</t>
+          <t>Good day Michael — Charles here with Paragon Government Solutions. I'm a cash buyer interested in 7939 S Kingston Ave, Chicago, IL 60617. Would the owner entertain a cash as-is offer with fast cash close, short feasibility window. Best email for the formal offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -16677,7 +16677,7 @@
       </c>
       <c r="F650" t="inlineStr">
         <is>
-          <t>Hello Michelle — my name's Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 5601 Howell St, Houston, TX 77032. could the seller look at a cash, as-is offer with fast cash close, short feasibility window. Best email for the formal offer? Much appreciated!</t>
+          <t>Hello Michelle — my name's Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 5601 Howell St, Houston, TX 77032. Could the seller look at a cash, as-is offer with fast cash close, short feasibility window. Best email for the formal offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -16702,7 +16702,7 @@
       </c>
       <c r="F651" t="inlineStr">
         <is>
-          <t>Good day Michelle — my name's Charles Pleasant, Paragon Government Solutions. I came across 16438 Vermillion Dr, Baton Rouge, LA 70819 and buy cash. would the owner entertain a cash as-is offer with quick close and a short inspection. Best email for the formal offer? Thanks!</t>
+          <t>Good day Michelle — my name's Charles Pleasant, Paragon Government Solutions. I came across 16438 Vermillion Dr, Baton Rouge, LA 70819 and buy cash. Would the owner entertain a cash as-is offer with quick close and a short inspection. Best email for the formal offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -16727,7 +16727,7 @@
       </c>
       <c r="F652" t="inlineStr">
         <is>
-          <t>Good day Michelle — Charles here with Paragon Government Solutions. I'm a cash buyer interested in 16438 Vermillion Dr, Baton Rouge, LA 70819. any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. Best email for the formal offer? Appreciate it!</t>
+          <t>Good day Michelle — Charles here with Paragon Government Solutions. I'm a cash buyer interested in 16438 Vermillion Dr, Baton Rouge, LA 70819. Any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. Best email for the formal offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -16752,7 +16752,7 @@
       </c>
       <c r="F653" t="inlineStr">
         <is>
-          <t>Hi Michelle — I'm Charles with Paragon Government Solutions. I'm reaching out about 13350 Tacoma St, Detroit, MI 48205. would the seller consider a cash, as-is offer with close quickly, short inspection period. Best email for the formal offer? Appreciate it!</t>
+          <t>Hi Michelle — I'm Charles with Paragon Government Solutions. I'm reaching out about 13350 Tacoma St, Detroit, MI 48205. Would the seller consider a cash, as-is offer with close quickly, short inspection period. Best email for the formal offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -16927,7 +16927,7 @@
       </c>
       <c r="F660" t="inlineStr">
         <is>
-          <t>Milton, hi — Charles Pleasant, Paragon Government Solutions. I'm interested in buying 1038 Canal Dr W, Lakeland, FL 33801 for cash. would the seller consider a cash, as-is offer with quick close and a short inspection. Where can I email the written terms? Thanks!</t>
+          <t>Milton, hi — Charles Pleasant, Paragon Government Solutions. I'm interested in buying 1038 Canal Dr W, Lakeland, FL 33801 for cash. Would the seller consider a cash, as-is offer with quick close and a short inspection. Where can I email the written terms? Thanks!</t>
         </is>
       </c>
     </row>
@@ -16952,7 +16952,7 @@
       </c>
       <c r="F661" t="inlineStr">
         <is>
-          <t>Hi Milton — Charles here with Paragon Government Solutions. I'm interested in buying 628 E 131st St, Cleveland, OH 44108 for cash. is the seller open to a cash as-is offer with fast cash close, short feasibility window. Where should I send the offer in writing? Much appreciated!</t>
+          <t>Hi Milton — Charles here with Paragon Government Solutions. I'm interested in buying 628 E 131st St, Cleveland, OH 44108 for cash. Is the seller open to a cash as-is offer with fast cash close, short feasibility window. Where should I send the offer in writing? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -16977,7 +16977,7 @@
       </c>
       <c r="F662" t="inlineStr">
         <is>
-          <t>Hi MINNA. Charles Pleasant, Paragon Government Solutions, and I'm a cash investor looking at 9852 OLIVIA Street, Jacksonville, FL 32219. could the seller look at a cash, as-is offer, quick close and a short inspection? What's a good email for the written offer? Much appreciated!</t>
+          <t>Hi MINNA. Charles Pleasant, Paragon Government Solutions, and I'm a cash investor looking at 9852 OLIVIA Street, Jacksonville, FL 32219. Could the seller look at a cash, as-is offer, quick close and a short inspection? What's a good email for the written offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -17052,7 +17052,7 @@
       </c>
       <c r="F665" t="inlineStr">
         <is>
-          <t>Good day Moe. my name's Charles Pleasant, Paragon Government Solutions, and I came across 11409 Manor St, Detroit, MI 48204 and buy cash. open to a discounted cash, as-is offer, close quickly, short inspection period? Where should I send the offer in writing? Thank you!</t>
+          <t>Good day Moe. My name's Charles Pleasant, Paragon Government Solutions, and I came across 11409 Manor St, Detroit, MI 48204 and buy cash. Open to a discounted cash, as-is offer, close quickly, short inspection period? Where should I send the offer in writing? Thank you!</t>
         </is>
       </c>
     </row>
@@ -17077,7 +17077,7 @@
       </c>
       <c r="F666" t="inlineStr">
         <is>
-          <t>Hey Mohammad — Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 3502 Goodhope St, Houston, TX 77021. any chance the seller would take a cash, as-is offer with close quickly, short inspection period. What's a good email for the written offer? Thank you!</t>
+          <t>Hey Mohammad — Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 3502 Goodhope St, Houston, TX 77021. Any chance the seller would take a cash, as-is offer with close quickly, short inspection period. What's a good email for the written offer? Thank you!</t>
         </is>
       </c>
     </row>
@@ -17152,7 +17152,7 @@
       </c>
       <c r="F669" t="inlineStr">
         <is>
-          <t>Hi Ms — Charles Pleasant, Paragon Government Solutions. I'm interested in buying 635 Marilyn Dr, Baton Rouge, LA 70815 for cash. any chance the seller would take a cash, as-is offer with a quick clean close and short due diligence. Where can I email the written terms? Thanks so much!</t>
+          <t>Hi Ms — Charles Pleasant, Paragon Government Solutions. I'm interested in buying 635 Marilyn Dr, Baton Rouge, LA 70815 for cash. Any chance the seller would take a cash, as-is offer with a quick clean close and short due diligence. Where can I email the written terms? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -17177,7 +17177,7 @@
       </c>
       <c r="F670" t="inlineStr">
         <is>
-          <t>Hello Mwood — Charles here with Paragon Government Solutions. I'm interested in buying 18982 Joann St, Detroit, MI 48205 for cash. open to a discounted cash, as-is offer with close quickly, short inspection period. What email should I send the written offer to? Thanks!</t>
+          <t>Hello Mwood — Charles here with Paragon Government Solutions. I'm interested in buying 18982 Joann St, Detroit, MI 48205 for cash. Open to a discounted cash, as-is offer with close quickly, short inspection period. What email should I send the written offer to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -17227,7 +17227,7 @@
       </c>
       <c r="F672" t="inlineStr">
         <is>
-          <t>Hello Nadia — Charles Pleasant, Paragon Government Solutions. I'm reaching out about 1333 W 71st St, Chicago, IL 60636. is the seller open to a cash as-is offer with close quickly, short inspection period. What's the best email to send it to? Thanks!</t>
+          <t>Hello Nadia — Charles Pleasant, Paragon Government Solutions. I'm reaching out about 1333 W 71st St, Chicago, IL 60636. Is the seller open to a cash as-is offer with close quickly, short inspection period. What's the best email to send it to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -17277,7 +17277,7 @@
       </c>
       <c r="F674" t="inlineStr">
         <is>
-          <t>Hey Nakashia — I'm Charles with Paragon Government Solutions. I came across 9937 Golden Gate Ave, Baton Rouge, LA 70818 and buy cash. could the seller look at a cash, as-is offer with close quickly, short inspection period. What's the best email to send it to? Thanks much!</t>
+          <t>Hey Nakashia — I'm Charles with Paragon Government Solutions. I came across 9937 Golden Gate Ave, Baton Rouge, LA 70818 and buy cash. Could the seller look at a cash, as-is offer with close quickly, short inspection period. What's the best email to send it to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -17327,7 +17327,7 @@
       </c>
       <c r="F676" t="inlineStr">
         <is>
-          <t>Nanci, hi. my name's Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 4500 Norfolk Ave, Baltimore, MD 21216. would the seller consider a cash, as-is offer, a quick clean close and short due diligence? Best email for the formal offer? Thanks so much!</t>
+          <t>Nanci, hi. My name's Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 4500 Norfolk Ave, Baltimore, MD 21216. Would the seller consider a cash, as-is offer, a quick clean close and short due diligence? Best email for the formal offer? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -17352,7 +17352,7 @@
       </c>
       <c r="F677" t="inlineStr">
         <is>
-          <t>Hello Nancy. I'm Charles with Paragon Government Solutions, and I came across 4217 NW 32nd Ter, Cape Coral, FL 33993 and buy cash. is the seller open to a cash as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Thanks so much!</t>
+          <t>Hello Nancy. I'm Charles with Paragon Government Solutions, and I came across 4217 NW 32nd Ter, Cape Coral, FL 33993 and buy cash. Is the seller open to a cash as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -17377,7 +17377,7 @@
       </c>
       <c r="F678" t="inlineStr">
         <is>
-          <t>Hey Nancy — Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 4903 Canal St, Houston, TX 77011. any chance the seller would take a cash, as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Thanks!</t>
+          <t>Hey Nancy — Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 4903 Canal St, Houston, TX 77011. Any chance the seller would take a cash, as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -17427,7 +17427,7 @@
       </c>
       <c r="F680" t="inlineStr">
         <is>
-          <t>Good day NARENDRA — Charles here with Paragon Government Solutions. I'm reaching out about 7007 LUCKY Drive E, Jacksonville, FL 32208. would the owner entertain a cash as-is offer with quick close and a short inspection. What's the best email to send it to? Thanks so much!</t>
+          <t>Good day NARENDRA — Charles here with Paragon Government Solutions. I'm reaching out about 7007 LUCKY Drive E, Jacksonville, FL 32208. Would the owner entertain a cash as-is offer with quick close and a short inspection. What's the best email to send it to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -17452,7 +17452,7 @@
       </c>
       <c r="F681" t="inlineStr">
         <is>
-          <t>Natalie, hi. this is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 4009 W ORANGE Drive #36, Phoenix, AZ 85019. could the seller look at a cash, as-is offer, a quick clean close and short due diligence? Where should I send the offer in writing? Much appreciated!</t>
+          <t>Natalie, hi. This is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 4009 W ORANGE Drive #36, Phoenix, AZ 85019. Could the seller look at a cash, as-is offer, a quick clean close and short due diligence? Where should I send the offer in writing? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -17477,7 +17477,7 @@
       </c>
       <c r="F682" t="inlineStr">
         <is>
-          <t>Good day Nataly. Charles here with Paragon Government Solutions, and I'm a cash buyer interested in 20260 Dean St, Detroit, MI 48234. open to a discounted cash, as-is offer, quick close and a short inspection? What email should I send the written offer to? Thanks so much!</t>
+          <t>Good day Nataly. Charles here with Paragon Government Solutions, and I'm a cash buyer interested in 20260 Dean St, Detroit, MI 48234. Open to a discounted cash, as-is offer, quick close and a short inspection? What email should I send the written offer to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -17527,7 +17527,7 @@
       </c>
       <c r="F684" t="inlineStr">
         <is>
-          <t>Nelly, hi. I'm Charles with Paragon Government Solutions, and I came across 315 Gober St, Houston, TX 77017 and buy cash. open to a discounted cash, as-is offer, quick close and a short inspection? Best email for the formal offer? Thanks much!</t>
+          <t>Nelly, hi. I'm Charles with Paragon Government Solutions, and I came across 315 Gober St, Houston, TX 77017 and buy cash. Open to a discounted cash, as-is offer, quick close and a short inspection? Best email for the formal offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -17652,7 +17652,7 @@
       </c>
       <c r="F689" t="inlineStr">
         <is>
-          <t>Good day NICOLE. Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 322 E 6TH Street, Jacksonville, FL 32206. could the seller look at a cash, as-is offer, a quick clean close and short due diligence? Best email for the formal offer? Much appreciated!</t>
+          <t>Good day NICOLE. Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 322 E 6TH Street, Jacksonville, FL 32206. Could the seller look at a cash, as-is offer, a quick clean close and short due diligence? Best email for the formal offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -17727,7 +17727,7 @@
       </c>
       <c r="F692" t="inlineStr">
         <is>
-          <t>Hey Nilsa. Charles here with Paragon Government Solutions, and I'm interested in buying 703 Monterey Ave, Cape Coral, FL 33904 for cash. any chance the seller would take a cash, as-is offer, fast cash close, short feasibility window? What's a good email for the written offer? Thanks much!</t>
+          <t>Hey Nilsa. Charles here with Paragon Government Solutions, and I'm interested in buying 703 Monterey Ave, Cape Coral, FL 33904 for cash. Any chance the seller would take a cash, as-is offer, fast cash close, short feasibility window? What's a good email for the written offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -17752,7 +17752,7 @@
       </c>
       <c r="F693" t="inlineStr">
         <is>
-          <t>Good day Nima. this is Charles Pleasant with Paragon Government Solutions, and I came across 409 Wilkes Rd, Columbia, SC 29203 and buy cash. is the seller open to a cash as-is offer, fast cash close, short feasibility window? What email should I send the written offer to? Thanks so much!</t>
+          <t>Good day Nima. This is Charles Pleasant with Paragon Government Solutions, and I came across 409 Wilkes Rd, Columbia, SC 29203 and buy cash. Is the seller open to a cash as-is offer, fast cash close, short feasibility window? What email should I send the written offer to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -17777,7 +17777,7 @@
       </c>
       <c r="F694" t="inlineStr">
         <is>
-          <t>Hello NM — I'm Charles with Paragon Government Solutions. I came across 3809 Santa Anita Rd SW, Albuquerque, NM 87105 and buy cash. is the seller open to a cash as-is offer with fast cash close, short feasibility window. What's the best email to send it to? Thanks much!</t>
+          <t>Hello NM — I'm Charles with Paragon Government Solutions. I came across 3809 Santa Anita Rd SW, Albuquerque, NM 87105 and buy cash. Is the seller open to a cash as-is offer with fast cash close, short feasibility window. What's the best email to send it to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -17852,7 +17852,7 @@
       </c>
       <c r="F697" t="inlineStr">
         <is>
-          <t>Hey Norma — Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 11326 S Union Ave, Chicago, IL 60628. any chance the seller would take a cash, as-is offer with close quickly, short inspection period. What's the best email to send it to? Thanks so much!</t>
+          <t>Hey Norma — Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 11326 S Union Ave, Chicago, IL 60628. Any chance the seller would take a cash, as-is offer with close quickly, short inspection period. What's the best email to send it to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -17902,7 +17902,7 @@
       </c>
       <c r="F699" t="inlineStr">
         <is>
-          <t>Hi there Orlando. I'm Charles with Paragon Government Solutions, and I came across 13420 Chico Rd NE, Albuquerque, NM 87123 and buy cash. open to a discounted cash, as-is offer, fast close with a brief inspection window? What's a good email for the written offer? Thanks so much!</t>
+          <t>Hi there Orlando. I'm Charles with Paragon Government Solutions, and I came across 13420 Chico Rd NE, Albuquerque, NM 87123 and buy cash. Open to a discounted cash, as-is offer, fast close with a brief inspection window? What's a good email for the written offer? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -17977,7 +17977,7 @@
       </c>
       <c r="F702" t="inlineStr">
         <is>
-          <t>Good day Pablo. I'm Charles with Paragon Government Solutions, and I'm a cash investor looking at 213 Hogan St, Houston, TX 77009. any chance the seller would take a cash, as-is offer, quick close and a short inspection? What's the best email to send it to? Much appreciated!</t>
+          <t>Good day Pablo. I'm Charles with Paragon Government Solutions, and I'm a cash investor looking at 213 Hogan St, Houston, TX 77009. Any chance the seller would take a cash, as-is offer, quick close and a short inspection? What's the best email to send it to? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -18027,7 +18027,7 @@
       </c>
       <c r="F704" t="inlineStr">
         <is>
-          <t>Hi Pamela. my name's Charles Pleasant, Paragon Government Solutions, and I came across 520 W CLARENDON Avenue #C3, Phoenix, AZ 85013 and buy cash. open to a discounted cash, as-is offer, fast close with a brief inspection window? What's a good email for the written offer? Appreciate it!</t>
+          <t>Hi Pamela. My name's Charles Pleasant, Paragon Government Solutions, and I came across 520 W CLARENDON Avenue #C3, Phoenix, AZ 85013 and buy cash. Open to a discounted cash, as-is offer, fast close with a brief inspection window? What's a good email for the written offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -18052,7 +18052,7 @@
       </c>
       <c r="F705" t="inlineStr">
         <is>
-          <t>Pamela, hi. this is Charles Pleasant with Paragon Government Solutions, and I came across 11401 S Morgan St, Chicago, IL 60643 and buy cash. any chance the seller would take a cash, as-is offer, fast cash close, short feasibility window? What email should I send the written offer to? Thank you!</t>
+          <t>Pamela, hi. This is Charles Pleasant with Paragon Government Solutions, and I came across 11401 S Morgan St, Chicago, IL 60643 and buy cash. Any chance the seller would take a cash, as-is offer, fast cash close, short feasibility window? What email should I send the written offer to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -18102,7 +18102,7 @@
       </c>
       <c r="F707" t="inlineStr">
         <is>
-          <t>Patricia, hi — this is Charles Pleasant with Paragon Government Solutions. I'm a cash investor looking at 109 Oakley Dr, Columbia, SC 29223. would the owner entertain a cash as-is offer with close quickly, short inspection period. Best email for the formal offer? Appreciate it!</t>
+          <t>Patricia, hi — this is Charles Pleasant with Paragon Government Solutions. I'm a cash investor looking at 109 Oakley Dr, Columbia, SC 29223. Would the owner entertain a cash as-is offer with close quickly, short inspection period. Best email for the formal offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -18127,7 +18127,7 @@
       </c>
       <c r="F708" t="inlineStr">
         <is>
-          <t>PATRICIA, hi — Charles Pleasant, Paragon Government Solutions. I'm reaching out about 1934 N Pearl St, Fayetteville, NC 28303. would the owner entertain a cash as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Much appreciated!</t>
+          <t>PATRICIA, hi — Charles Pleasant, Paragon Government Solutions. I'm reaching out about 1934 N Pearl St, Fayetteville, NC 28303. Would the owner entertain a cash as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -18177,7 +18177,7 @@
       </c>
       <c r="F710" t="inlineStr">
         <is>
-          <t>Good day Patti. this is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 218 Florien St, Pittsburgh, PA 15204. any chance the seller would take a cash, as-is offer, close quickly, short inspection period? Best email for the formal offer? Thanks much!</t>
+          <t>Good day Patti. This is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 218 Florien St, Pittsburgh, PA 15204. Any chance the seller would take a cash, as-is offer, close quickly, short inspection period? Best email for the formal offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -18202,7 +18202,7 @@
       </c>
       <c r="F711" t="inlineStr">
         <is>
-          <t>Hello Paul. Charles here with Paragon Government Solutions, and I came across 4629 Larkspur St, Houston, TX 77051 and buy cash. is the seller open to a cash as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Thanks much!</t>
+          <t>Hello Paul. Charles here with Paragon Government Solutions, and I came across 4629 Larkspur St, Houston, TX 77051 and buy cash. Is the seller open to a cash as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -18227,7 +18227,7 @@
       </c>
       <c r="F712" t="inlineStr">
         <is>
-          <t>Good day PEPPER. Charles here with Paragon Government Solutions, and I'm a cash investor looking at 2185 MOREHOUSE Road, Jacksonville, FL 32209. could the seller look at a cash, as-is offer, close quickly, short inspection period? What's the best email to send it to? Appreciate it!</t>
+          <t>Good day PEPPER. Charles here with Paragon Government Solutions, and I'm a cash investor looking at 2185 MOREHOUSE Road, Jacksonville, FL 32209. Could the seller look at a cash, as-is offer, close quickly, short inspection period? What's the best email to send it to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -18302,7 +18302,7 @@
       </c>
       <c r="F715" t="inlineStr">
         <is>
-          <t>Hi Phyllis. Charles Pleasant, Paragon Government Solutions, and I came across 847 Glenmore Ave, Baton Rouge, LA 70806 and buy cash. would the owner entertain a cash as-is offer, a quick clean close and short due diligence? Where should I send the offer in writing? Appreciate it!</t>
+          <t>Hi Phyllis. Charles Pleasant, Paragon Government Solutions, and I came across 847 Glenmore Ave, Baton Rouge, LA 70806 and buy cash. Would the owner entertain a cash as-is offer, a quick clean close and short due diligence? Where should I send the offer in writing? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -18327,7 +18327,7 @@
       </c>
       <c r="F716" t="inlineStr">
         <is>
-          <t>Good day Ponce — I'm Charles with Paragon Government Solutions. I came across 12 Sea Hawk Ct, Columbia, SC 29203 and buy cash. is the seller open to a cash as-is offer with quick close and a short inspection. What's a good email for the written offer? Thanks much!</t>
+          <t>Good day Ponce — I'm Charles with Paragon Government Solutions. I came across 12 Sea Hawk Ct, Columbia, SC 29203 and buy cash. Is the seller open to a cash as-is offer with quick close and a short inspection. What's a good email for the written offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -18352,7 +18352,7 @@
       </c>
       <c r="F717" t="inlineStr">
         <is>
-          <t>QUINNEICE, hi — I'm Charles with Paragon Government Solutions. I'm interested in buying 1921 Ashridge Dr, Fayetteville, NC 28304 for cash. would the owner entertain a cash as-is offer with fast close with a brief inspection window. Where can I email the written terms? Thank you!</t>
+          <t>QUINNEICE, hi — I'm Charles with Paragon Government Solutions. I'm interested in buying 1921 Ashridge Dr, Fayetteville, NC 28304 for cash. Would the owner entertain a cash as-is offer with fast close with a brief inspection window. Where can I email the written terms? Thank you!</t>
         </is>
       </c>
     </row>
@@ -18377,7 +18377,7 @@
       </c>
       <c r="F718" t="inlineStr">
         <is>
-          <t>Rachel, hi — Charles here with Paragon Government Solutions. I'd like to put in a cash offer on 330 Klamath Dr, Pittsburgh, PA 15205. could the seller look at a cash, as-is offer with fast cash close, short feasibility window. Where can I email the written terms? Much appreciated!</t>
+          <t>Rachel, hi — Charles here with Paragon Government Solutions. I'd like to put in a cash offer on 330 Klamath Dr, Pittsburgh, PA 15205. Could the seller look at a cash, as-is offer with fast cash close, short feasibility window. Where can I email the written terms? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -18452,7 +18452,7 @@
       </c>
       <c r="F721" t="inlineStr">
         <is>
-          <t>Good day Ray. Charles Pleasant, Paragon Government Solutions, and I'm a cash investor looking at 6627 Eastwood St, Houston, TX 77021. would the owner entertain a cash as-is offer, fast cash close, short feasibility window? What's the best email to send it to? Thanks much!</t>
+          <t>Good day Ray. Charles Pleasant, Paragon Government Solutions, and I'm a cash investor looking at 6627 Eastwood St, Houston, TX 77021. Would the owner entertain a cash as-is offer, fast cash close, short feasibility window? What's the best email to send it to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -18477,7 +18477,7 @@
       </c>
       <c r="F722" t="inlineStr">
         <is>
-          <t>Hey Re/Max. Charles here with Paragon Government Solutions, and I'm reaching out about 1720 Morninghill Dr, Columbia, SC 29210. could the seller look at a cash, as-is offer, fast cash close, short feasibility window? What email should I send the written offer to? Thanks much!</t>
+          <t>Hey Re/Max. Charles here with Paragon Government Solutions, and I'm reaching out about 1720 Morninghill Dr, Columbia, SC 29210. Could the seller look at a cash, as-is offer, fast cash close, short feasibility window? What email should I send the written offer to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -18502,7 +18502,7 @@
       </c>
       <c r="F723" t="inlineStr">
         <is>
-          <t>Hi Rebecca. Charles here with Paragon Government Solutions, and I'm a cash buyer interested in 6408 Macroom Meadows Ln, Houston, TX 77048. any chance the seller would take a cash, as-is offer, a quick clean close and short due diligence? What email should I send the written offer to? Thanks!</t>
+          <t>Hi Rebecca. Charles here with Paragon Government Solutions, and I'm a cash buyer interested in 6408 Macroom Meadows Ln, Houston, TX 77048. Any chance the seller would take a cash, as-is offer, a quick clean close and short due diligence? What email should I send the written offer to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -18552,7 +18552,7 @@
       </c>
       <c r="F725" t="inlineStr">
         <is>
-          <t>Hello Reid — Charles Pleasant, Paragon Government Solutions. I'm reaching out about 6224 Highland Hills Dr, Dallas, TX 75241. any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. What email should I send the written offer to? Thank you!</t>
+          <t>Hello Reid — Charles Pleasant, Paragon Government Solutions. I'm reaching out about 6224 Highland Hills Dr, Dallas, TX 75241. Any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. What email should I send the written offer to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -18577,7 +18577,7 @@
       </c>
       <c r="F726" t="inlineStr">
         <is>
-          <t>Hello Rene. Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 7331 S Peoria St, Chicago, IL 60621 for cash. could the seller look at a cash, as-is offer, close quickly, short inspection period? What's the best email to send it to? Thanks so much!</t>
+          <t>Hello Rene. Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 7331 S Peoria St, Chicago, IL 60621 for cash. Could the seller look at a cash, as-is offer, close quickly, short inspection period? What's the best email to send it to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -18602,7 +18602,7 @@
       </c>
       <c r="F727" t="inlineStr">
         <is>
-          <t>Hello Reva — Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 8451 Greenview Ave, Detroit, MI 48228. any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. What email should I send the written offer to? Thanks much!</t>
+          <t>Hello Reva — Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 8451 Greenview Ave, Detroit, MI 48228. Any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. What email should I send the written offer to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -18627,7 +18627,7 @@
       </c>
       <c r="F728" t="inlineStr">
         <is>
-          <t>Hi Rhonda. my name's Charles Pleasant, Paragon Government Solutions, and I came across 37985 Falcon Wood Dr, Denham Springs, LA 70706 and buy cash. any chance the seller would take a cash, as-is offer, close quickly, short inspection period? Where should I send the offer in writing? Thanks so much!</t>
+          <t>Hi Rhonda. My name's Charles Pleasant, Paragon Government Solutions, and I came across 37985 Falcon Wood Dr, Denham Springs, LA 70706 and buy cash. Any chance the seller would take a cash, as-is offer, close quickly, short inspection period? Where should I send the offer in writing? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -18652,7 +18652,7 @@
       </c>
       <c r="F729" t="inlineStr">
         <is>
-          <t>Hey Rhonda — this is Charles Pleasant with Paragon Government Solutions. I'm interested in buying 2802 W Mosher St, Baltimore, MD 21216 for cash. could the seller look at a cash, as-is offer with fast close with a brief inspection window. Where should I send the offer in writing? Thank you!</t>
+          <t>Hey Rhonda — this is Charles Pleasant with Paragon Government Solutions. I'm interested in buying 2802 W Mosher St, Baltimore, MD 21216 for cash. Could the seller look at a cash, as-is offer with fast close with a brief inspection window. Where should I send the offer in writing? Thank you!</t>
         </is>
       </c>
     </row>
@@ -18727,7 +18727,7 @@
       </c>
       <c r="F732" t="inlineStr">
         <is>
-          <t>Hello Robbie — Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 33870 Perkins Crossing Rd, Walker, LA 70785. could the seller look at a cash, as-is offer with fast cash close, short feasibility window. What email should I send the written offer to? Appreciate it!</t>
+          <t>Hello Robbie — Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 33870 Perkins Crossing Rd, Walker, LA 70785. Could the seller look at a cash, as-is offer with fast cash close, short feasibility window. What email should I send the written offer to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -18777,7 +18777,7 @@
       </c>
       <c r="F734" t="inlineStr">
         <is>
-          <t>Hi ROBERT — Charles here with Paragon Government Solutions. I'm a cash buyer interested in 784 Yardville Hamilton Sq, Trenton, NJ 08691. any chance the seller would take a cash, as-is offer with a quick clean close and short due diligence. Where can I email the written terms? Appreciate it!</t>
+          <t>Hi ROBERT — Charles here with Paragon Government Solutions. I'm a cash buyer interested in 784 Yardville Hamilton Sq, Trenton, NJ 08691. Any chance the seller would take a cash, as-is offer with a quick clean close and short due diligence. Where can I email the written terms? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -18827,7 +18827,7 @@
       </c>
       <c r="F736" t="inlineStr">
         <is>
-          <t>Hello Robert. I'm Charles with Paragon Government Solutions, and I'm interested in buying 6235 Leaf Arbor Dr, Houston, TX 77092 for cash. is the seller open to a cash as-is offer, fast cash close, short feasibility window? Best email for the formal offer? Thanks!</t>
+          <t>Hello Robert. I'm Charles with Paragon Government Solutions, and I'm interested in buying 6235 Leaf Arbor Dr, Houston, TX 77092 for cash. Is the seller open to a cash as-is offer, fast cash close, short feasibility window? Best email for the formal offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -18927,7 +18927,7 @@
       </c>
       <c r="F740" t="inlineStr">
         <is>
-          <t>Robyn, hi. Charles here with Paragon Government Solutions, and I'm a cash buyer interested in 15212 Crystal Dr, Pride, LA 70770. could the seller look at a cash, as-is offer, fast close with a brief inspection window? What's the best email to send it to? Thanks!</t>
+          <t>Robyn, hi. Charles here with Paragon Government Solutions, and I'm a cash buyer interested in 15212 Crystal Dr, Pride, LA 70770. Could the seller look at a cash, as-is offer, fast close with a brief inspection window? What's the best email to send it to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -18952,7 +18952,7 @@
       </c>
       <c r="F741" t="inlineStr">
         <is>
-          <t>Hello Rodney. Charles here with Paragon Government Solutions, and I'd like to put in a cash offer on 14035 Kentfield St, Detroit, MI 48223. any chance the seller would take a cash, as-is offer, close quickly, short inspection period? What's the best email to send it to? Thank you!</t>
+          <t>Hello Rodney. Charles here with Paragon Government Solutions, and I'd like to put in a cash offer on 14035 Kentfield St, Detroit, MI 48223. Any chance the seller would take a cash, as-is offer, close quickly, short inspection period? What's the best email to send it to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -19002,7 +19002,7 @@
       </c>
       <c r="F743" t="inlineStr">
         <is>
-          <t>Hi Ross — this is Charles Pleasant with Paragon Government Solutions. I'm reaching out about 2507 Parktrail Rd, Baltimore, MD 21234. would the seller consider a cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Much appreciated!</t>
+          <t>Hi Ross — this is Charles Pleasant with Paragon Government Solutions. I'm reaching out about 2507 Parktrail Rd, Baltimore, MD 21234. Would the seller consider a cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -19052,7 +19052,7 @@
       </c>
       <c r="F745" t="inlineStr">
         <is>
-          <t>Hello Roxanne. this is Charles Pleasant with Paragon Government Solutions, and I came across 1316 E Applegate Dr, Austin, TX 78753 and buy cash. is the seller open to a cash as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Thank you!</t>
+          <t>Hello Roxanne. This is Charles Pleasant with Paragon Government Solutions, and I came across 1316 E Applegate Dr, Austin, TX 78753 and buy cash. Is the seller open to a cash as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Thank you!</t>
         </is>
       </c>
     </row>
@@ -19127,7 +19127,7 @@
       </c>
       <c r="F748" t="inlineStr">
         <is>
-          <t>Hi RYAN — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 3318 NOLAN Street, Jacksonville, FL 32254. could the seller look at a cash, as-is offer with quick close and a short inspection. What email should I send the written offer to? Appreciate it!</t>
+          <t>Hi RYAN — I'm Charles with Paragon Government Solutions. I'm a cash investor looking at 3318 NOLAN Street, Jacksonville, FL 32254. Could the seller look at a cash, as-is offer with quick close and a short inspection. What email should I send the written offer to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -19227,7 +19227,7 @@
       </c>
       <c r="F752" t="inlineStr">
         <is>
-          <t>Hi there Samantha. my name's Charles Pleasant, Paragon Government Solutions, and I came across 6159 Lyndhurst Dr, Houston, TX 77033 and buy cash. is the seller open to a cash as-is offer, a quick clean close and short due diligence? Where should I send the offer in writing? Appreciate it!</t>
+          <t>Hi there Samantha. My name's Charles Pleasant, Paragon Government Solutions, and I came across 6159 Lyndhurst Dr, Houston, TX 77033 and buy cash. Is the seller open to a cash as-is offer, a quick clean close and short due diligence? Where should I send the offer in writing? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -19252,7 +19252,7 @@
       </c>
       <c r="F753" t="inlineStr">
         <is>
-          <t>Good day Sara. I'm Charles with Paragon Government Solutions, and I'd like to put in a cash offer on 6537 S 15th Dr, Phoenix, AZ 85041. could the seller look at a cash, as-is offer, close quickly, short inspection period? What's the best email to send it to? Much appreciated!</t>
+          <t>Good day Sara. I'm Charles with Paragon Government Solutions, and I'd like to put in a cash offer on 6537 S 15th Dr, Phoenix, AZ 85041. Could the seller look at a cash, as-is offer, close quickly, short inspection period? What's the best email to send it to? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -19277,7 +19277,7 @@
       </c>
       <c r="F754" t="inlineStr">
         <is>
-          <t>Hello Sarah. this is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 5953 S Throop St, Chicago, IL 60636. could the seller look at a cash, as-is offer, a quick clean close and short due diligence? Where should I send the offer in writing? Thank you!</t>
+          <t>Hello Sarah. This is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 5953 S Throop St, Chicago, IL 60636. Could the seller look at a cash, as-is offer, a quick clean close and short due diligence? Where should I send the offer in writing? Thank you!</t>
         </is>
       </c>
     </row>
@@ -19302,7 +19302,7 @@
       </c>
       <c r="F755" t="inlineStr">
         <is>
-          <t>Good day Schlanda — this is Charles Pleasant with Paragon Government Solutions. I'm interested in buying 1319 Reynes St, New Orleans, LA 70117 for cash. could the seller look at a cash, as-is offer with a quick clean close and short due diligence. What's the best email to send it to? Thanks much!</t>
+          <t>Good day Schlanda — this is Charles Pleasant with Paragon Government Solutions. I'm interested in buying 1319 Reynes St, New Orleans, LA 70117 for cash. Could the seller look at a cash, as-is offer with a quick clean close and short due diligence. What's the best email to send it to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -19352,7 +19352,7 @@
       </c>
       <c r="F757" t="inlineStr">
         <is>
-          <t>Hi there Scott. Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 7607 Dobel St, Detroit, MI 48234 for cash. open to a discounted cash, as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Thanks much!</t>
+          <t>Hi there Scott. Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 7607 Dobel St, Detroit, MI 48234 for cash. Open to a discounted cash, as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -19377,7 +19377,7 @@
       </c>
       <c r="F758" t="inlineStr">
         <is>
-          <t>Good day Scott. my name's Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 6104 Franklin Villas Way, Indianapolis, IN 46237 for cash. open to a discounted cash, as-is offer, quick close and a short inspection? Where should I send the offer in writing? Much appreciated!</t>
+          <t>Good day Scott. My name's Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 6104 Franklin Villas Way, Indianapolis, IN 46237 for cash. Open to a discounted cash, as-is offer, quick close and a short inspection? Where should I send the offer in writing? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -19402,7 +19402,7 @@
       </c>
       <c r="F759" t="inlineStr">
         <is>
-          <t>SCOTT, hi — I'm Charles with Paragon Government Solutions. I came across 6711 CAVALIER Road, Jacksonville, FL 32208 and buy cash. is the seller open to a cash as-is offer with quick close and a short inspection. What's a good email for the written offer? Much appreciated!</t>
+          <t>SCOTT, hi — I'm Charles with Paragon Government Solutions. I came across 6711 CAVALIER Road, Jacksonville, FL 32208 and buy cash. Is the seller open to a cash as-is offer with quick close and a short inspection. What's a good email for the written offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -19452,7 +19452,7 @@
       </c>
       <c r="F761" t="inlineStr">
         <is>
-          <t>Hey Sean. Charles here with Paragon Government Solutions, and I'm reaching out about 8605 Fireside Dr, Austin, TX 78757. is the seller open to a cash as-is offer, quick close and a short inspection? Best email for the formal offer? Thanks so much!</t>
+          <t>Hey Sean. Charles here with Paragon Government Solutions, and I'm reaching out about 8605 Fireside Dr, Austin, TX 78757. Is the seller open to a cash as-is offer, quick close and a short inspection? Best email for the formal offer? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -19477,7 +19477,7 @@
       </c>
       <c r="F762" t="inlineStr">
         <is>
-          <t>Hi Sean — Charles here with Paragon Government Solutions. I'm a cash buyer interested in 8506 McDade St, Houston, TX 77080. would the owner entertain a cash as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Thanks!</t>
+          <t>Hi Sean — Charles here with Paragon Government Solutions. I'm a cash buyer interested in 8506 McDade St, Houston, TX 77080. Would the owner entertain a cash as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -19527,7 +19527,7 @@
       </c>
       <c r="F764" t="inlineStr">
         <is>
-          <t>Hi there Sergio. I'm Charles with Paragon Government Solutions, and I'm a cash investor looking at 16203 Barbarossa Dr, Houston, TX 77083. is the seller open to a cash as-is offer, a quick clean close and short due diligence? Best email for the formal offer? Much appreciated!</t>
+          <t>Hi there Sergio. I'm Charles with Paragon Government Solutions, and I'm a cash investor looking at 16203 Barbarossa Dr, Houston, TX 77083. Is the seller open to a cash as-is offer, a quick clean close and short due diligence? Best email for the formal offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -19552,7 +19552,7 @@
       </c>
       <c r="F765" t="inlineStr">
         <is>
-          <t>Sergio, hi — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 10841 S Vernon Ave, Chicago, IL 60628. would the seller consider a cash, as-is offer with a quick clean close and short due diligence. Where can I email the written terms? Thanks so much!</t>
+          <t>Sergio, hi — my name's Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 10841 S Vernon Ave, Chicago, IL 60628. Would the seller consider a cash, as-is offer with a quick clean close and short due diligence. Where can I email the written terms? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -19577,7 +19577,7 @@
       </c>
       <c r="F766" t="inlineStr">
         <is>
-          <t>SETH, hi — Charles here with Paragon Government Solutions. I'm interested in buying 2837 LIPPIA Road, Jacksonville, FL 32209 for cash. could the seller look at a cash, as-is offer with a quick clean close and short due diligence. What email should I send the written offer to? Much appreciated!</t>
+          <t>SETH, hi — Charles here with Paragon Government Solutions. I'm interested in buying 2837 LIPPIA Road, Jacksonville, FL 32209 for cash. Could the seller look at a cash, as-is offer with a quick clean close and short due diligence. What email should I send the written offer to? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -19602,7 +19602,7 @@
       </c>
       <c r="F767" t="inlineStr">
         <is>
-          <t>Hey Shakena. my name's Charles Pleasant, Paragon Government Solutions, and I'm a cash buyer interested in 130 Brandon Hall Rd, Columbia, SC 29229. would the seller consider a cash, as-is offer, a quick clean close and short due diligence? What's a good email for the written offer? Thanks so much!</t>
+          <t>Hey Shakena. My name's Charles Pleasant, Paragon Government Solutions, and I'm a cash buyer interested in 130 Brandon Hall Rd, Columbia, SC 29229. Would the seller consider a cash, as-is offer, a quick clean close and short due diligence? What's a good email for the written offer? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -19627,7 +19627,7 @@
       </c>
       <c r="F768" t="inlineStr">
         <is>
-          <t>Hi Shane — my name's Charles Pleasant, Paragon Government Solutions. I'm reaching out about 889 E 128th St, Cleveland, OH 44108. could the seller look at a cash, as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Thank you!</t>
+          <t>Hi Shane — my name's Charles Pleasant, Paragon Government Solutions. I'm reaching out about 889 E 128th St, Cleveland, OH 44108. Could the seller look at a cash, as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -19652,7 +19652,7 @@
       </c>
       <c r="F769" t="inlineStr">
         <is>
-          <t>Hi Shannon — Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 8710 Files St, Dallas, TX 75217. would the seller consider a cash, as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Appreciate it!</t>
+          <t>Hi Shannon — Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 8710 Files St, Dallas, TX 75217. Would the seller consider a cash, as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -19702,7 +19702,7 @@
       </c>
       <c r="F771" t="inlineStr">
         <is>
-          <t>Hi Sharon — I'm Charles with Paragon Government Solutions. I'm reaching out about 516 Lakeside Ave, Columbia, SC 29203. open to a discounted cash, as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Thanks so much!</t>
+          <t>Hi Sharon — I'm Charles with Paragon Government Solutions. I'm reaching out about 516 Lakeside Ave, Columbia, SC 29203. Open to a discounted cash, as-is offer with fast cash close, short feasibility window. What's a good email for the written offer? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -19727,7 +19727,7 @@
       </c>
       <c r="F772" t="inlineStr">
         <is>
-          <t>Good day Sharon — Charles here with Paragon Government Solutions. I'm reaching out about 515 W Main St, Gonzales, LA 70737. would the owner entertain a cash as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Thanks!</t>
+          <t>Good day Sharon — Charles here with Paragon Government Solutions. I'm reaching out about 515 W Main St, Gonzales, LA 70737. Would the owner entertain a cash as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Thanks!</t>
         </is>
       </c>
     </row>
@@ -19752,7 +19752,7 @@
       </c>
       <c r="F773" t="inlineStr">
         <is>
-          <t>Shauntell, hi — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 337 W 110th Pl, Chicago, IL 60628. is the seller open to a cash as-is offer with fast cash close, short feasibility window. What email should I send the written offer to? Thanks much!</t>
+          <t>Shauntell, hi — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 337 W 110th Pl, Chicago, IL 60628. Is the seller open to a cash as-is offer with fast cash close, short feasibility window. What email should I send the written offer to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -19777,7 +19777,7 @@
       </c>
       <c r="F774" t="inlineStr">
         <is>
-          <t>SHAWANA, hi. this is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 8342 BARRACUDA Road, Jacksonville, FL 32244. would the owner entertain a cash as-is offer, close quickly, short inspection period? What email should I send the written offer to? Thanks much!</t>
+          <t>SHAWANA, hi. This is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 8342 BARRACUDA Road, Jacksonville, FL 32244. Would the owner entertain a cash as-is offer, close quickly, short inspection period? What email should I send the written offer to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -19802,7 +19802,7 @@
       </c>
       <c r="F775" t="inlineStr">
         <is>
-          <t>Hi Shawn — Charles Pleasant, Paragon Government Solutions. I'm interested in buying 5404 Dixie Ln, Alexandria, LA 71301 for cash. would the owner entertain a cash as-is offer with quick close and a short inspection. Where should I send the offer in writing? Thank you!</t>
+          <t>Hi Shawn — Charles Pleasant, Paragon Government Solutions. I'm interested in buying 5404 Dixie Ln, Alexandria, LA 71301 for cash. Would the owner entertain a cash as-is offer with quick close and a short inspection. Where should I send the offer in writing? Thank you!</t>
         </is>
       </c>
     </row>
@@ -19827,7 +19827,7 @@
       </c>
       <c r="F776" t="inlineStr">
         <is>
-          <t>Hi there SHAWN — I'm Charles with Paragon Government Solutions. I'm a cash buyer interested in 3862 ORLANDO Circle W, Jacksonville, FL 32207. could the seller look at a cash, as-is offer with fast close with a brief inspection window. Where can I email the written terms? Thank you!</t>
+          <t>Hi there SHAWN — I'm Charles with Paragon Government Solutions. I'm a cash buyer interested in 3862 ORLANDO Circle W, Jacksonville, FL 32207. Could the seller look at a cash, as-is offer with fast close with a brief inspection window. Where can I email the written terms? Thank you!</t>
         </is>
       </c>
     </row>
@@ -19877,7 +19877,7 @@
       </c>
       <c r="F778" t="inlineStr">
         <is>
-          <t>Hi there Shelby. my name's Charles Pleasant, Paragon Government Solutions, and I came across 4235 Elmwood St, Houston, TX 77051 and buy cash. open to a discounted cash, as-is offer, a quick clean close and short due diligence? Where should I send the offer in writing? Appreciate it!</t>
+          <t>Hi there Shelby. My name's Charles Pleasant, Paragon Government Solutions, and I came across 4235 Elmwood St, Houston, TX 77051 and buy cash. Open to a discounted cash, as-is offer, a quick clean close and short due diligence? Where should I send the offer in writing? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -19902,7 +19902,7 @@
       </c>
       <c r="F779" t="inlineStr">
         <is>
-          <t>Hi Shelly — Charles Pleasant, Paragon Government Solutions. I'm reaching out about 4500 Blossom Valley Ln, Bakersfield, CA 93313. could the seller look at a cash, as-is offer with close quickly, short inspection period. What email should I send the written offer to? Thanks!</t>
+          <t>Hi Shelly — Charles Pleasant, Paragon Government Solutions. I'm reaching out about 4500 Blossom Valley Ln, Bakersfield, CA 93313. Could the seller look at a cash, as-is offer with close quickly, short inspection period. What email should I send the written offer to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -19927,7 +19927,7 @@
       </c>
       <c r="F780" t="inlineStr">
         <is>
-          <t>Good day Shemika. this is Charles Pleasant with Paragon Government Solutions, and I'd like to put in a cash offer on 2764 Dalton St, Baton Rouge, LA 70805. could the seller look at a cash, as-is offer, quick close and a short inspection? What's the best email to send it to? Appreciate it!</t>
+          <t>Good day Shemika. This is Charles Pleasant with Paragon Government Solutions, and I'd like to put in a cash offer on 2764 Dalton St, Baton Rouge, LA 70805. Could the seller look at a cash, as-is offer, quick close and a short inspection? What's the best email to send it to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -19952,7 +19952,7 @@
       </c>
       <c r="F781" t="inlineStr">
         <is>
-          <t>Good day Shemika — my name's Charles Pleasant, Paragon Government Solutions. I came across 2764 Dalton St, Baton Rouge, LA 70805 and buy cash. would the seller consider a cash, as-is offer with fast cash close, short feasibility window. Where can I email the written terms? Thanks!</t>
+          <t>Good day Shemika — my name's Charles Pleasant, Paragon Government Solutions. I came across 2764 Dalton St, Baton Rouge, LA 70805 and buy cash. Would the seller consider a cash, as-is offer with fast cash close, short feasibility window. Where can I email the written terms? Thanks!</t>
         </is>
       </c>
     </row>
@@ -20002,7 +20002,7 @@
       </c>
       <c r="F783" t="inlineStr">
         <is>
-          <t>Sherri, hi — Charles here with Paragon Government Solutions. I'm interested in buying 2108 Blake Ave, Dallas, TX 75228 for cash. is the seller open to a cash as-is offer with a quick clean close and short due diligence. Best email for the formal offer? Appreciate it!</t>
+          <t>Sherri, hi — Charles here with Paragon Government Solutions. I'm interested in buying 2108 Blake Ave, Dallas, TX 75228 for cash. Is the seller open to a cash as-is offer with a quick clean close and short due diligence. Best email for the formal offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -20052,7 +20052,7 @@
       </c>
       <c r="F785" t="inlineStr">
         <is>
-          <t>Hello SHINESHA — Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 235 Whitney Dr, Fayetteville, NC 28314. any chance the seller would take a cash, as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Much appreciated!</t>
+          <t>Hello SHINESHA — Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 235 Whitney Dr, Fayetteville, NC 28314. Any chance the seller would take a cash, as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -20102,7 +20102,7 @@
       </c>
       <c r="F787" t="inlineStr">
         <is>
-          <t>Hi Shoaib. Charles Pleasant, Paragon Government Solutions, and I'm a cash buyer interested in 5093 Garland St, Detroit, MI 48213. could the seller look at a cash, as-is offer, quick close and a short inspection? Where should I send the offer in writing? Thanks much!</t>
+          <t>Hi Shoaib. Charles Pleasant, Paragon Government Solutions, and I'm a cash buyer interested in 5093 Garland St, Detroit, MI 48213. Could the seller look at a cash, as-is offer, quick close and a short inspection? Where should I send the offer in writing? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -20177,7 +20177,7 @@
       </c>
       <c r="F790" t="inlineStr">
         <is>
-          <t>Hi there Shonda — Charles here with Paragon Government Solutions. I came across 218 Sanhican Dr, Trenton, NJ 08618 and buy cash. would the owner entertain a cash as-is offer with quick close and a short inspection. What email should I send the written offer to? Thanks!</t>
+          <t>Hi there Shonda — Charles here with Paragon Government Solutions. I came across 218 Sanhican Dr, Trenton, NJ 08618 and buy cash. Would the owner entertain a cash as-is offer with quick close and a short inspection. What email should I send the written offer to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -20202,7 +20202,7 @@
       </c>
       <c r="F791" t="inlineStr">
         <is>
-          <t>Sidra, hi — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 7106 Tierwester St, Houston, TX 77021. could the seller look at a cash, as-is offer with a quick clean close and short due diligence. What's the best email to send it to? Thanks so much!</t>
+          <t>Sidra, hi — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 7106 Tierwester St, Houston, TX 77021. Could the seller look at a cash, as-is offer with a quick clean close and short due diligence. What's the best email to send it to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -20227,7 +20227,7 @@
       </c>
       <c r="F792" t="inlineStr">
         <is>
-          <t>Hey Sonia — Charles here with Paragon Government Solutions. I'm reaching out about 514 L St, Bakersfield, CA 93304. would the seller consider a cash, as-is offer with a quick clean close and short due diligence. Where should I send the offer in writing? Appreciate it!</t>
+          <t>Hey Sonia — Charles here with Paragon Government Solutions. I'm reaching out about 514 L St, Bakersfield, CA 93304. Would the seller consider a cash, as-is offer with a quick clean close and short due diligence. Where should I send the offer in writing? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -20327,7 +20327,7 @@
       </c>
       <c r="F796" t="inlineStr">
         <is>
-          <t>Hello Stacy — this is Charles Pleasant with Paragon Government Solutions. I'm interested in buying 11833 Beachberry Dr, Houston, TX 77034 for cash. open to a discounted cash, as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Thanks so much!</t>
+          <t>Hello Stacy — this is Charles Pleasant with Paragon Government Solutions. I'm interested in buying 11833 Beachberry Dr, Houston, TX 77034 for cash. Open to a discounted cash, as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -20377,7 +20377,7 @@
       </c>
       <c r="F798" t="inlineStr">
         <is>
-          <t>Hello Stephanie — Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 5135 S May St, Chicago, IL 60609. would the owner entertain a cash as-is offer with fast cash close, short feasibility window. Best email for the formal offer? Thanks so much!</t>
+          <t>Hello Stephanie — Charles Pleasant, Paragon Government Solutions. I'm a cash investor looking at 5135 S May St, Chicago, IL 60609. Would the owner entertain a cash as-is offer with fast cash close, short feasibility window. Best email for the formal offer? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -20402,7 +20402,7 @@
       </c>
       <c r="F799" t="inlineStr">
         <is>
-          <t>Hi Stephanie. I'm Charles with Paragon Government Solutions, and I'm a cash buyer interested in 1404 SE 34th Ter, Cape Coral, FL 33904. could the seller look at a cash, as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Thanks much!</t>
+          <t>Hi Stephanie. I'm Charles with Paragon Government Solutions, and I'm a cash buyer interested in 1404 SE 34th Ter, Cape Coral, FL 33904. Could the seller look at a cash, as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -20452,7 +20452,7 @@
       </c>
       <c r="F801" t="inlineStr">
         <is>
-          <t>Hey STEPHANIE. I'm Charles with Paragon Government Solutions, and I'd like to put in a cash offer on 115 Brookwood Ave, Fayetteville, NC 28301. would the seller consider a cash, as-is offer, fast close with a brief inspection window? Best email for the formal offer? Thanks much!</t>
+          <t>Hey STEPHANIE. I'm Charles with Paragon Government Solutions, and I'd like to put in a cash offer on 115 Brookwood Ave, Fayetteville, NC 28301. Would the seller consider a cash, as-is offer, fast close with a brief inspection window? Best email for the formal offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -20477,7 +20477,7 @@
       </c>
       <c r="F802" t="inlineStr">
         <is>
-          <t>Good day Stephanie — this is Charles Pleasant with Paragon Government Solutions. I'm reaching out about 6106 Sandy Creek Ln, Zachary, LA 70791. could the seller look at a cash, as-is offer with quick close and a short inspection. Where should I send the offer in writing? Thanks!</t>
+          <t>Good day Stephanie — this is Charles Pleasant with Paragon Government Solutions. I'm reaching out about 6106 Sandy Creek Ln, Zachary, LA 70791. Could the seller look at a cash, as-is offer with quick close and a short inspection. Where should I send the offer in writing? Thanks!</t>
         </is>
       </c>
     </row>
@@ -20502,7 +20502,7 @@
       </c>
       <c r="F803" t="inlineStr">
         <is>
-          <t>Stephanie, hi. Charles here with Paragon Government Solutions, and I'm interested in buying 16127 Long Rd, Houston, TX 77044 for cash. is the seller open to a cash as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Appreciate it!</t>
+          <t>Stephanie, hi. Charles here with Paragon Government Solutions, and I'm interested in buying 16127 Long Rd, Houston, TX 77044 for cash. Is the seller open to a cash as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -20527,7 +20527,7 @@
       </c>
       <c r="F804" t="inlineStr">
         <is>
-          <t>Hey STEPHEN. this is Charles Pleasant with Paragon Government Solutions, and I'm a cash investor looking at 4222 Woodlea Ave, Baltimore, MD 21206. open to a discounted cash, as-is offer, quick close and a short inspection? Where should I send the offer in writing? Appreciate it!</t>
+          <t>Hey STEPHEN. This is Charles Pleasant with Paragon Government Solutions, and I'm a cash investor looking at 4222 Woodlea Ave, Baltimore, MD 21206. Open to a discounted cash, as-is offer, quick close and a short inspection? Where should I send the offer in writing? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -20552,7 +20552,7 @@
       </c>
       <c r="F805" t="inlineStr">
         <is>
-          <t>Hi Steve — Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 6831 S Emerald Ave, Chicago, IL 60621. would the seller consider a cash, as-is offer with close quickly, short inspection period. What's a good email for the written offer? Thanks much!</t>
+          <t>Hi Steve — Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 6831 S Emerald Ave, Chicago, IL 60621. Would the seller consider a cash, as-is offer with close quickly, short inspection period. What's a good email for the written offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -20577,7 +20577,7 @@
       </c>
       <c r="F806" t="inlineStr">
         <is>
-          <t>Hello Steve — this is Charles Pleasant with Paragon Government Solutions. I'm a cash investor looking at 2666 Olympia Ave, North Charleston, SC 29405. any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. Where should I send the offer in writing? Appreciate it!</t>
+          <t>Hello Steve — this is Charles Pleasant with Paragon Government Solutions. I'm a cash investor looking at 2666 Olympia Ave, North Charleston, SC 29405. Any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. Where should I send the offer in writing? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -20677,7 +20677,7 @@
       </c>
       <c r="F810" t="inlineStr">
         <is>
-          <t>Hi Steven. this is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 3061 Horse Ranch Rd, San Antonio, TX 78264. is the seller open to a cash as-is offer, quick close and a short inspection? Best email for the formal offer? Much appreciated!</t>
+          <t>Hi Steven. This is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 3061 Horse Ranch Rd, San Antonio, TX 78264. Is the seller open to a cash as-is offer, quick close and a short inspection? Best email for the formal offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -20702,7 +20702,7 @@
       </c>
       <c r="F811" t="inlineStr">
         <is>
-          <t>Good day Summer — Charles here with Paragon Government Solutions. I came across 1201 Willow Dr, Lake Charles, LA 70611 and buy cash. is the seller open to a cash as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Much appreciated!</t>
+          <t>Good day Summer — Charles here with Paragon Government Solutions. I came across 1201 Willow Dr, Lake Charles, LA 70611 and buy cash. Is the seller open to a cash as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -20727,7 +20727,7 @@
       </c>
       <c r="F812" t="inlineStr">
         <is>
-          <t>Hello Susan. my name's Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 3419 SE 5th Ave, Cape Coral, FL 33904. any chance the seller would take a cash, as-is offer, a quick clean close and short due diligence? Where should I send the offer in writing? Much appreciated!</t>
+          <t>Hello Susan. My name's Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 3419 SE 5th Ave, Cape Coral, FL 33904. Any chance the seller would take a cash, as-is offer, a quick clean close and short due diligence? Where should I send the offer in writing? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -20777,7 +20777,7 @@
       </c>
       <c r="F814" t="inlineStr">
         <is>
-          <t>Hello Suzy. Charles Pleasant, Paragon Government Solutions, and I'm a cash buyer interested in 13050 N 19TH Street #50, Phoenix, AZ 85022. open to a discounted cash, as-is offer, close quickly, short inspection period? What email should I send the written offer to? Appreciate it!</t>
+          <t>Hello Suzy. Charles Pleasant, Paragon Government Solutions, and I'm a cash buyer interested in 13050 N 19TH Street #50, Phoenix, AZ 85022. Open to a discounted cash, as-is offer, close quickly, short inspection period? What email should I send the written offer to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -20832,7 +20832,7 @@
       </c>
       <c r="F816" t="inlineStr">
         <is>
-          <t>Hello T'Keyah. Charles here with Paragon Government Solutions, and I'm a cash buyer interested in your listing. would the owner entertain a cash as-is offer, close quickly, short inspection period? Best email for the formal offer? Thanks!</t>
+          <t>Hello T'Keyah. Charles here with Paragon Government Solutions, and I'm a cash buyer interested in your listing. Would the owner entertain a cash as-is offer, close quickly, short inspection period? Best email for the formal offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -20882,7 +20882,7 @@
       </c>
       <c r="F818" t="inlineStr">
         <is>
-          <t>Hi there Tal. Charles Pleasant, Paragon Government Solutions, and I'm a cash buyer interested in 2166 W 93rd St, Cleveland, OH 44102. could the seller look at a cash, as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Thanks much!</t>
+          <t>Hi there Tal. Charles Pleasant, Paragon Government Solutions, and I'm a cash buyer interested in 2166 W 93rd St, Cleveland, OH 44102. Could the seller look at a cash, as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -20957,7 +20957,7 @@
       </c>
       <c r="F821" t="inlineStr">
         <is>
-          <t>Good day Tamara — Charles here with Paragon Government Solutions. I came across 3846 W 84th Pl, Chicago, IL 60652 and buy cash. is the seller open to a cash as-is offer with close quickly, short inspection period. Where can I email the written terms? Thank you!</t>
+          <t>Good day Tamara — Charles here with Paragon Government Solutions. I came across 3846 W 84th Pl, Chicago, IL 60652 and buy cash. Is the seller open to a cash as-is offer with close quickly, short inspection period. Where can I email the written terms? Thank you!</t>
         </is>
       </c>
     </row>
@@ -20982,7 +20982,7 @@
       </c>
       <c r="F822" t="inlineStr">
         <is>
-          <t>Hi Tamesha. this is Charles Pleasant with Paragon Government Solutions, and I'm a cash investor looking at 12323 Misty Laurel Dr, Houston, TX 77014. open to a discounted cash, as-is offer, fast close with a brief inspection window? What's a good email for the written offer? Thanks much!</t>
+          <t>Hi Tamesha. This is Charles Pleasant with Paragon Government Solutions, and I'm a cash investor looking at 12323 Misty Laurel Dr, Houston, TX 77014. Open to a discounted cash, as-is offer, fast close with a brief inspection window? What's a good email for the written offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -21007,7 +21007,7 @@
       </c>
       <c r="F823" t="inlineStr">
         <is>
-          <t>Tami, hi. I'm Charles with Paragon Government Solutions, and I'm interested in buying 6243 S 31st West Ave, Tulsa, OK 74132 for cash. would the owner entertain a cash as-is offer, a quick clean close and short due diligence? Where should I send the offer in writing? Much appreciated!</t>
+          <t>Tami, hi. I'm Charles with Paragon Government Solutions, and I'm interested in buying 6243 S 31st West Ave, Tulsa, OK 74132 for cash. Would the owner entertain a cash as-is offer, a quick clean close and short due diligence? Where should I send the offer in writing? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -21182,7 +21182,7 @@
       </c>
       <c r="F830" t="inlineStr">
         <is>
-          <t>Hey Tara — Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 1430 Dahlia Rd, Columbia, SC 29205. would the seller consider a cash, as-is offer with quick close and a short inspection. What email should I send the written offer to? Thanks much!</t>
+          <t>Hey Tara — Charles Pleasant, Paragon Government Solutions. I'm a cash buyer interested in 1430 Dahlia Rd, Columbia, SC 29205. Would the seller consider a cash, as-is offer with quick close and a short inspection. What email should I send the written offer to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -21232,7 +21232,7 @@
       </c>
       <c r="F832" t="inlineStr">
         <is>
-          <t>Hey Tashia. this is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 2433 W Tonto St, Phoenix, AZ 85009. would the owner entertain a cash as-is offer, fast cash close, short feasibility window? What's the best email to send it to? Appreciate it!</t>
+          <t>Hey Tashia. This is Charles Pleasant with Paragon Government Solutions, and I'm reaching out about 2433 W Tonto St, Phoenix, AZ 85009. Would the owner entertain a cash as-is offer, fast cash close, short feasibility window? What's the best email to send it to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -21282,7 +21282,7 @@
       </c>
       <c r="F834" t="inlineStr">
         <is>
-          <t>Good day Taz. my name's Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 10615 Kirkdale Dr, Houston, TX 77089. would the owner entertain a cash as-is offer, close quickly, short inspection period? Best email for the formal offer? Thanks!</t>
+          <t>Good day Taz. My name's Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 10615 Kirkdale Dr, Houston, TX 77089. Would the owner entertain a cash as-is offer, close quickly, short inspection period? Best email for the formal offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -21357,7 +21357,7 @@
       </c>
       <c r="F837" t="inlineStr">
         <is>
-          <t>Tera, hi. I'm Charles with Paragon Government Solutions, and I'd like to put in a cash offer on 2222 Detroit Ave APT 504, Cleveland, OH 44113. is the seller open to a cash as-is offer, fast cash close, short feasibility window? What email should I send the written offer to? Thanks much!</t>
+          <t>Tera, hi. I'm Charles with Paragon Government Solutions, and I'd like to put in a cash offer on 2222 Detroit Ave APT 504, Cleveland, OH 44113. Is the seller open to a cash as-is offer, fast cash close, short feasibility window? What email should I send the written offer to? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -21407,7 +21407,7 @@
       </c>
       <c r="F839" t="inlineStr">
         <is>
-          <t>Teresa, hi. I'm Charles with Paragon Government Solutions, and I came across 189 Regina Ave, Hamilton, NJ 08619 and buy cash. would the seller consider a cash, as-is offer, quick close and a short inspection? What email should I send the written offer to? Thanks so much!</t>
+          <t>Teresa, hi. I'm Charles with Paragon Government Solutions, and I came across 189 Regina Ave, Hamilton, NJ 08619 and buy cash. Would the seller consider a cash, as-is offer, quick close and a short inspection? What email should I send the written offer to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -21432,7 +21432,7 @@
       </c>
       <c r="F840" t="inlineStr">
         <is>
-          <t>Hi there Teresa. this is Charles Pleasant with Paragon Government Solutions, and I'd like to put in a cash offer on 2602 Falls Dr, Dallas, TX 75211. could the seller look at a cash, as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Much appreciated!</t>
+          <t>Hi there Teresa. This is Charles Pleasant with Paragon Government Solutions, and I'd like to put in a cash offer on 2602 Falls Dr, Dallas, TX 75211. Could the seller look at a cash, as-is offer, fast cash close, short feasibility window? Where should I send the offer in writing? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -21457,7 +21457,7 @@
       </c>
       <c r="F841" t="inlineStr">
         <is>
-          <t>Terry, hi — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 609 Lufkin Circle, Fayetteville, NC 28311. could the seller look at a cash, as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Thank you!</t>
+          <t>Terry, hi — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 609 Lufkin Circle, Fayetteville, NC 28311. Could the seller look at a cash, as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Thank you!</t>
         </is>
       </c>
     </row>
@@ -21532,7 +21532,7 @@
       </c>
       <c r="F844" t="inlineStr">
         <is>
-          <t>Thao, hi — this is Charles Pleasant with Paragon Government Solutions. I'm reaching out about 1263 James St, Baltimore, MD 21223. would the seller consider a cash, as-is offer with fast close with a brief inspection window. What's the best email to send it to? Thanks!</t>
+          <t>Thao, hi — this is Charles Pleasant with Paragon Government Solutions. I'm reaching out about 1263 James St, Baltimore, MD 21223. Would the seller consider a cash, as-is offer with fast close with a brief inspection window. What's the best email to send it to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -21682,7 +21682,7 @@
       </c>
       <c r="F850" t="inlineStr">
         <is>
-          <t>Hi Tiffany. I'm Charles with Paragon Government Solutions, and I'm interested in buying 11744 Wade St, Detroit, MI 48213 for cash. any chance the seller would take a cash, as-is offer, fast close with a brief inspection window? What's the best email to send it to? Appreciate it!</t>
+          <t>Hi Tiffany. I'm Charles with Paragon Government Solutions, and I'm interested in buying 11744 Wade St, Detroit, MI 48213 for cash. Any chance the seller would take a cash, as-is offer, fast close with a brief inspection window? What's the best email to send it to? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -21732,7 +21732,7 @@
       </c>
       <c r="F852" t="inlineStr">
         <is>
-          <t>Timothy, hi — Charles here with Paragon Government Solutions. I'd like to put in a cash offer on 230 Sterling Rd, Bakersfield, CA 93307. any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. What's the best email to send it to? Thanks so much!</t>
+          <t>Timothy, hi — Charles here with Paragon Government Solutions. I'd like to put in a cash offer on 230 Sterling Rd, Bakersfield, CA 93307. Any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. What's the best email to send it to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -21782,7 +21782,7 @@
       </c>
       <c r="F854" t="inlineStr">
         <is>
-          <t>Hi TJ — this is Charles Pleasant with Paragon Government Solutions. I'm a cash investor looking at 1809 Manteo St, Fayetteville, NC 28303. any chance the seller would take a cash, as-is offer with fast close with a brief inspection window. Best email for the formal offer? Thanks much!</t>
+          <t>Hi TJ — this is Charles Pleasant with Paragon Government Solutions. I'm a cash investor looking at 1809 Manteo St, Fayetteville, NC 28303. Any chance the seller would take a cash, as-is offer with fast close with a brief inspection window. Best email for the formal offer? Thanks much!</t>
         </is>
       </c>
     </row>
@@ -21807,7 +21807,7 @@
       </c>
       <c r="F855" t="inlineStr">
         <is>
-          <t>Hi TLeice. Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 2684 Iroquois St, Baton Rouge, LA 70805. could the seller look at a cash, as-is offer, fast close with a brief inspection window? Best email for the formal offer? Thanks!</t>
+          <t>Hi TLeice. Charles Pleasant, Paragon Government Solutions, and I'd like to put in a cash offer on 2684 Iroquois St, Baton Rouge, LA 70805. Could the seller look at a cash, as-is offer, fast close with a brief inspection window? Best email for the formal offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -21882,7 +21882,7 @@
       </c>
       <c r="F858" t="inlineStr">
         <is>
-          <t>Hi there TONY — this is Charles Pleasant with Paragon Government Solutions. I'm reaching out about 3252 THOMAS Street, Jacksonville, FL 32254. could the seller look at a cash, as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Much appreciated!</t>
+          <t>Hi there TONY — this is Charles Pleasant with Paragon Government Solutions. I'm reaching out about 3252 THOMAS Street, Jacksonville, FL 32254. Could the seller look at a cash, as-is offer with fast close with a brief inspection window. What email should I send the written offer to? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -21932,7 +21932,7 @@
       </c>
       <c r="F860" t="inlineStr">
         <is>
-          <t>Good day Tonya — this is Charles Pleasant with Paragon Government Solutions. I'm interested in buying 12746 Woodland Dr, Jacksonville, FL 32218 for cash. could the seller look at a cash, as-is offer with fast close with a brief inspection window. Best email for the formal offer? Appreciate it!</t>
+          <t>Good day Tonya — this is Charles Pleasant with Paragon Government Solutions. I'm interested in buying 12746 Woodland Dr, Jacksonville, FL 32218 for cash. Could the seller look at a cash, as-is offer with fast close with a brief inspection window. Best email for the formal offer? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -21957,7 +21957,7 @@
       </c>
       <c r="F861" t="inlineStr">
         <is>
-          <t>Good day TORANIQUE. this is Charles Pleasant with Paragon Government Solutions, and I'm a cash investor looking at 1354 Worstead Dr, Fayetteville, NC 28314. is the seller open to a cash as-is offer, fast close with a brief inspection window? What's a good email for the written offer? Much appreciated!</t>
+          <t>Good day TORANIQUE. This is Charles Pleasant with Paragon Government Solutions, and I'm a cash investor looking at 1354 Worstead Dr, Fayetteville, NC 28314. Is the seller open to a cash as-is offer, fast close with a brief inspection window? What's a good email for the written offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -22007,7 +22007,7 @@
       </c>
       <c r="F863" t="inlineStr">
         <is>
-          <t>Good day TRACEY. Charles Pleasant, Paragon Government Solutions, and I came across 1181 Torrey Dr, Fayetteville, NC 28301 and buy cash. could the seller look at a cash, as-is offer, close quickly, short inspection period? What's a good email for the written offer? Thanks!</t>
+          <t>Good day TRACEY. Charles Pleasant, Paragon Government Solutions, and I came across 1181 Torrey Dr, Fayetteville, NC 28301 and buy cash. Could the seller look at a cash, as-is offer, close quickly, short inspection period? What's a good email for the written offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -22082,7 +22082,7 @@
       </c>
       <c r="F866" t="inlineStr">
         <is>
-          <t>Good day Trinh. Charles Pleasant, Paragon Government Solutions, and I came across 255 Sorrel Tree Dr, Columbia, SC 29223 and buy cash. could the seller look at a cash, as-is offer, fast close with a brief inspection window? Where can I email the written terms? Appreciate it!</t>
+          <t>Good day Trinh. Charles Pleasant, Paragon Government Solutions, and I came across 255 Sorrel Tree Dr, Columbia, SC 29223 and buy cash. Could the seller look at a cash, as-is offer, fast close with a brief inspection window? Where can I email the written terms? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -22132,7 +22132,7 @@
       </c>
       <c r="F868" t="inlineStr">
         <is>
-          <t>Hey Tucker — this is Charles Pleasant with Paragon Government Solutions. I'm a cash investor looking at 4538 Larkspur St, Houston, TX 77051. would the owner entertain a cash as-is offer with fast close with a brief inspection window. Best email for the formal offer? Thanks!</t>
+          <t>Hey Tucker — this is Charles Pleasant with Paragon Government Solutions. I'm a cash investor looking at 4538 Larkspur St, Houston, TX 77051. Would the owner entertain a cash as-is offer with fast close with a brief inspection window. Best email for the formal offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -22182,7 +22182,7 @@
       </c>
       <c r="F870" t="inlineStr">
         <is>
-          <t>Hello Tyler — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 338 Bowling Ave, Columbia, SC 29203. any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. Where can I email the written terms? Appreciate it!</t>
+          <t>Hello Tyler — this is Charles Pleasant with Paragon Government Solutions. I'm a cash buyer interested in 338 Bowling Ave, Columbia, SC 29203. Any chance the seller would take a cash, as-is offer with fast cash close, short feasibility window. Where can I email the written terms? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -22207,7 +22207,7 @@
       </c>
       <c r="F871" t="inlineStr">
         <is>
-          <t>Hello Tyreeta. Charles here with Paragon Government Solutions, and I'm a cash investor looking at 3628 W 83rd St, Chicago, IL 60652. open to a discounted cash, as-is offer, fast cash close, short feasibility window? Where can I email the written terms? Thank you!</t>
+          <t>Hello Tyreeta. Charles here with Paragon Government Solutions, and I'm a cash investor looking at 3628 W 83rd St, Chicago, IL 60652. Open to a discounted cash, as-is offer, fast cash close, short feasibility window? Where can I email the written terms? Thank you!</t>
         </is>
       </c>
     </row>
@@ -22282,7 +22282,7 @@
       </c>
       <c r="F874" t="inlineStr">
         <is>
-          <t>Hello Vanessa. Charles here with Paragon Government Solutions, and I'd like to put in a cash offer on 15560 Tiger Bend Rd, Baton Rouge, LA 70817. any chance the seller would take a cash, as-is offer, close quickly, short inspection period? Where can I email the written terms? Thank you!</t>
+          <t>Hello Vanessa. Charles here with Paragon Government Solutions, and I'd like to put in a cash offer on 15560 Tiger Bend Rd, Baton Rouge, LA 70817. Any chance the seller would take a cash, as-is offer, close quickly, short inspection period? Where can I email the written terms? Thank you!</t>
         </is>
       </c>
     </row>
@@ -22307,7 +22307,7 @@
       </c>
       <c r="F875" t="inlineStr">
         <is>
-          <t>Vanessa, hi. my name's Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 2248 Cooper St, Dallas, TX 75215 for cash. would the seller consider a cash, as-is offer, a quick clean close and short due diligence? What email should I send the written offer to? Thanks!</t>
+          <t>Vanessa, hi. My name's Charles Pleasant, Paragon Government Solutions, and I'm interested in buying 2248 Cooper St, Dallas, TX 75215 for cash. Would the seller consider a cash, as-is offer, a quick clean close and short due diligence? What email should I send the written offer to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -22407,7 +22407,7 @@
       </c>
       <c r="F879" t="inlineStr">
         <is>
-          <t>Hey VANETTA — Charles Pleasant, Paragon Government Solutions. I came across 4022 TYNDALE Drive, Jacksonville, FL 32210 and buy cash. is the seller open to a cash as-is offer with fast close with a brief inspection window. What's a good email for the written offer? Thanks so much!</t>
+          <t>Hey VANETTA — Charles Pleasant, Paragon Government Solutions. I came across 4022 TYNDALE Drive, Jacksonville, FL 32210 and buy cash. Is the seller open to a cash as-is offer with fast close with a brief inspection window. What's a good email for the written offer? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -22457,7 +22457,7 @@
       </c>
       <c r="F881" t="inlineStr">
         <is>
-          <t>Hi there Veronica. Charles here with Paragon Government Solutions, and I'd like to put in a cash offer on 213 T St, Bakersfield, CA 93304. would the seller consider a cash, as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Thanks!</t>
+          <t>Hi there Veronica. Charles here with Paragon Government Solutions, and I'd like to put in a cash offer on 213 T St, Bakersfield, CA 93304. Would the seller consider a cash, as-is offer, fast close with a brief inspection window? What email should I send the written offer to? Thanks!</t>
         </is>
       </c>
     </row>
@@ -22507,7 +22507,7 @@
       </c>
       <c r="F883" t="inlineStr">
         <is>
-          <t>Victoria, hi — my name's Charles Pleasant, Paragon Government Solutions. I came across 2127 Coelum Ct, Dallas TX 75253 and buy cash. open to a discounted cash, as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Much appreciated!</t>
+          <t>Victoria, hi — my name's Charles Pleasant, Paragon Government Solutions. I came across 2127 Coelum Ct, Dallas TX 75253 and buy cash. Open to a discounted cash, as-is offer with a quick clean close and short due diligence. What's a good email for the written offer? Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -22607,7 +22607,7 @@
       </c>
       <c r="F887" t="inlineStr">
         <is>
-          <t>Hey Viveka — I'm Charles with Paragon Government Solutions. I'm reaching out about 8028 S Ada St, Chicago, IL 60620. would the owner entertain a cash as-is offer with fast cash close, short feasibility window. What's the best email to send it to? Thanks so much!</t>
+          <t>Hey Viveka — I'm Charles with Paragon Government Solutions. I'm reaching out about 8028 S Ada St, Chicago, IL 60620. Would the owner entertain a cash as-is offer with fast cash close, short feasibility window. What's the best email to send it to? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -22632,7 +22632,7 @@
       </c>
       <c r="F888" t="inlineStr">
         <is>
-          <t>Good day Wally. Charles Pleasant, Paragon Government Solutions, and I'm a cash investor looking at 5604 Creekmore Dr, Oklahoma City, OK 73179. would the owner entertain a cash as-is offer, quick close and a short inspection? What's a good email for the written offer? Thanks!</t>
+          <t>Good day Wally. Charles Pleasant, Paragon Government Solutions, and I'm a cash investor looking at 5604 Creekmore Dr, Oklahoma City, OK 73179. Would the owner entertain a cash as-is offer, quick close and a short inspection? What's a good email for the written offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -22657,7 +22657,7 @@
       </c>
       <c r="F889" t="inlineStr">
         <is>
-          <t>Hi there Wayne — Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 2011 Lake Carolina Dr, Columbia, SC 29229. could the seller look at a cash, as-is offer with a quick clean close and short due diligence. Where should I send the offer in writing? Appreciate it!</t>
+          <t>Hi there Wayne — Charles Pleasant, Paragon Government Solutions. I'd like to put in a cash offer on 2011 Lake Carolina Dr, Columbia, SC 29229. Could the seller look at a cash, as-is offer with a quick clean close and short due diligence. Where should I send the offer in writing? Appreciate it!</t>
         </is>
       </c>
     </row>
@@ -22682,7 +22682,7 @@
       </c>
       <c r="F890" t="inlineStr">
         <is>
-          <t>Hi there WELCOME. Charles here with Paragon Government Solutions, and I'm interested in buying 603 Faison Ave, Fayetteville, NC 28304 for cash. would the owner entertain a cash as-is offer, a quick clean close and short due diligence? What's a good email for the written offer? Thanks!</t>
+          <t>Hi there WELCOME. Charles here with Paragon Government Solutions, and I'm interested in buying 603 Faison Ave, Fayetteville, NC 28304 for cash. Would the owner entertain a cash as-is offer, a quick clean close and short due diligence? What's a good email for the written offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -22732,7 +22732,7 @@
       </c>
       <c r="F892" t="inlineStr">
         <is>
-          <t>Hello Wes — Charles here with Paragon Government Solutions. I'm a cash buyer interested in 1013 N Ruth Ave, Lakeland, FL 33805. would the seller consider a cash, as-is offer with fast close with a brief inspection window. Where should I send the offer in writing? Thanks so much!</t>
+          <t>Hello Wes — Charles here with Paragon Government Solutions. I'm a cash buyer interested in 1013 N Ruth Ave, Lakeland, FL 33805. Would the seller consider a cash, as-is offer with fast close with a brief inspection window. Where should I send the offer in writing? Thanks so much!</t>
         </is>
       </c>
     </row>
@@ -22832,7 +22832,7 @@
       </c>
       <c r="F896" t="inlineStr">
         <is>
-          <t>Hi William. my name's Charles Pleasant, Paragon Government Solutions, and I'm a cash investor looking at 14711 Lappin St, Detroit, MI 48205. could the seller look at a cash, as-is offer, close quickly, short inspection period? What's a good email for the written offer? Thanks!</t>
+          <t>Hi William. My name's Charles Pleasant, Paragon Government Solutions, and I'm a cash investor looking at 14711 Lappin St, Detroit, MI 48205. Could the seller look at a cash, as-is offer, close quickly, short inspection period? What's a good email for the written offer? Thanks!</t>
         </is>
       </c>
     </row>
@@ -22857,7 +22857,7 @@
       </c>
       <c r="F897" t="inlineStr">
         <is>
-          <t>Hey William. I'm Charles with Paragon Government Solutions, and I'd like to put in a cash offer on 2640 Cypress Ave, Dallas, TX 75227. open to a discounted cash, as-is offer, a quick clean close and short due diligence? What's a good email for the written offer? Thank you!</t>
+          <t>Hey William. I'm Charles with Paragon Government Solutions, and I'd like to put in a cash offer on 2640 Cypress Ave, Dallas, TX 75227. Open to a discounted cash, as-is offer, a quick clean close and short due diligence? What's a good email for the written offer? Thank you!</t>
         </is>
       </c>
     </row>
@@ -23007,7 +23007,7 @@
       </c>
       <c r="F903" t="inlineStr">
         <is>
-          <t>Hi there Zachary — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 2937 Seyburn St, Detroit, MI 48214. open to a discounted cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Appreciate it!</t>
+          <t>Hi there Zachary — this is Charles Pleasant with Paragon Government Solutions. I'd like to put in a cash offer on 2937 Seyburn St, Detroit, MI 48214. Open to a discounted cash, as-is offer with close quickly, short inspection period. Where should I send the offer in writing? Appreciate it!</t>
         </is>
       </c>
     </row>

</xml_diff>